<commit_message>
Updated BRA_grids model - 2025-09-19 23:02
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF08F1FE-3E08-4FEF-B1F6-C83F6CCCB1FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E370F03-41AA-44C4-887F-3FDC18BBAF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9587,7 +9587,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045A06FE-6910-4BF5-BA4F-7D6646D61BB9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{210118A5-B969-4A27-96E1-F7022EE1971F}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15509,7 +15509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D33341D-1611-4E4C-8DF3-4C5B012C5322}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF9BB1A-0EFE-4FC3-9952-6E9651B40A25}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-20 09:01
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E370F03-41AA-44C4-887F-3FDC18BBAF9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13F66FA9-8507-4B72-9216-24229193B799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9587,7 +9587,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{210118A5-B969-4A27-96E1-F7022EE1971F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A098E839-C770-44EE-901F-7E7020586EDE}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15509,7 +15509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF9BB1A-0EFE-4FC3-9952-6E9651B40A25}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4831C7EF-419F-4435-9289-CE36FA72BE0B}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-21 15:06
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA2D5E73-070E-4888-8ADE-901607AB3C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAE758B4-947E-41B4-B181-FC966B634DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52D86749-46AF-4DEF-8389-85C9A2E6DA4C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69C434C0-C79A-4C81-A61F-ECCFD83BF284}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{824FE8E2-77B1-4B16-9624-9B98F58B82C8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428515DF-F61B-452E-BB23-A760B3D0F52C}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 02:33
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAE758B4-947E-41B4-B181-FC966B634DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1000DCAD-328F-4029-8183-DAF5D97200A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69C434C0-C79A-4C81-A61F-ECCFD83BF284}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2885D707-9737-44B0-ADA4-9B3309D6D3F3}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13158,10 +13158,10 @@
         <v>726</v>
       </c>
       <c r="C332">
-        <v>-31.97045859914089</v>
+        <v>-29.91778906765273</v>
       </c>
       <c r="D332">
-        <v>-52.97655154895552</v>
+        <v>-55.756257153342048</v>
       </c>
     </row>
     <row r="333" spans="2:4">
@@ -13169,10 +13169,10 @@
         <v>727</v>
       </c>
       <c r="C333">
-        <v>-29.996400987558729</v>
+        <v>-31.925049565997167</v>
       </c>
       <c r="D333">
-        <v>-54.208011523226133</v>
+        <v>-52.988639879938802</v>
       </c>
     </row>
     <row r="334" spans="2:4">
@@ -13180,10 +13180,10 @@
         <v>728</v>
       </c>
       <c r="C334">
-        <v>-30.08663379997256</v>
+        <v>-27.026337837617159</v>
       </c>
       <c r="D334">
-        <v>-56.101122318328237</v>
+        <v>-52.999922322189846</v>
       </c>
     </row>
     <row r="335" spans="2:4">
@@ -13191,10 +13191,10 @@
         <v>729</v>
       </c>
       <c r="C335">
-        <v>-28.255409001374037</v>
+        <v>-29.154729365098586</v>
       </c>
       <c r="D335">
-        <v>-54.339846654291598</v>
+        <v>-51.473031804213456</v>
       </c>
     </row>
     <row r="336" spans="2:4">
@@ -13202,10 +13202,10 @@
         <v>730</v>
       </c>
       <c r="C336">
-        <v>-30.298601757555229</v>
+        <v>-28.474474218178731</v>
       </c>
       <c r="D336">
-        <v>-51.691159021067229</v>
+        <v>-50.264942603177197</v>
       </c>
     </row>
     <row r="337" spans="2:4">
@@ -13213,10 +13213,10 @@
         <v>731</v>
       </c>
       <c r="C337">
-        <v>-28.838896618314362</v>
+        <v>-30.38909064864206</v>
       </c>
       <c r="D337">
-        <v>-50.912133246589491</v>
+        <v>-51.498693829725681</v>
       </c>
     </row>
     <row r="338" spans="2:4">
@@ -13224,10 +13224,10 @@
         <v>732</v>
       </c>
       <c r="C338">
-        <v>-24.07925466867616</v>
+        <v>-28.657105430504327</v>
       </c>
       <c r="D338">
-        <v>-53.496349781236376</v>
+        <v>-53.981494798031832</v>
       </c>
     </row>
     <row r="339" spans="2:4">
@@ -13235,10 +13235,10 @@
         <v>733</v>
       </c>
       <c r="C339">
-        <v>-25.638156147970559</v>
+        <v>-18.339825503898322</v>
       </c>
       <c r="D339">
-        <v>-53.201270522362563</v>
+        <v>-56.661942712831042</v>
       </c>
     </row>
     <row r="340" spans="2:4">
@@ -13246,10 +13246,10 @@
         <v>734</v>
       </c>
       <c r="C340">
-        <v>-27.026337837617159</v>
+        <v>-15.393254216021999</v>
       </c>
       <c r="D340">
-        <v>-52.999922322189846</v>
+        <v>-59.870929653083621</v>
       </c>
     </row>
     <row r="341" spans="2:4">
@@ -13257,10 +13257,10 @@
         <v>735</v>
       </c>
       <c r="C341">
-        <v>-24.294116923063548</v>
+        <v>-15.80297747383729</v>
       </c>
       <c r="D341">
-        <v>-50.133107472111739</v>
+        <v>-57.273493715548582</v>
       </c>
     </row>
     <row r="342" spans="2:4">
@@ -13268,10 +13268,10 @@
         <v>736</v>
       </c>
       <c r="C342">
-        <v>-25.807259122346117</v>
+        <v>-20.583933777481352</v>
       </c>
       <c r="D342">
-        <v>-49.206932384677074</v>
+        <v>-52.781795105336087</v>
       </c>
     </row>
     <row r="343" spans="2:4">
@@ -13279,10 +13279,10 @@
         <v>737</v>
       </c>
       <c r="C343">
-        <v>-27.011349164888419</v>
+        <v>-22.44729831898637</v>
       </c>
       <c r="D343">
-        <v>-51.036777370505931</v>
+        <v>-51.009511468399197</v>
       </c>
     </row>
     <row r="344" spans="2:4">
@@ -13290,10 +13290,10 @@
         <v>738</v>
       </c>
       <c r="C344">
-        <v>-26.775277569410729</v>
+        <v>-19.830741226253327</v>
       </c>
       <c r="D344">
-        <v>-49.987040139397152</v>
+        <v>-49.754339767969107</v>
       </c>
     </row>
     <row r="345" spans="2:4">
@@ -13301,10 +13301,10 @@
         <v>739</v>
       </c>
       <c r="C345">
-        <v>-22.970272660934874</v>
+        <v>-18.476312794026995</v>
       </c>
       <c r="D345">
-        <v>-47.138938843249413</v>
+        <v>-52.914440034503912</v>
       </c>
     </row>
     <row r="346" spans="2:4">
@@ -13312,10 +13312,10 @@
         <v>740</v>
       </c>
       <c r="C346">
-        <v>-24.317475893549901</v>
+        <v>-24.294116923063548</v>
       </c>
       <c r="D346">
-        <v>-47.675635256259191</v>
+        <v>-50.133107472111739</v>
       </c>
     </row>
     <row r="347" spans="2:4">
@@ -13323,10 +13323,10 @@
         <v>741</v>
       </c>
       <c r="C347">
-        <v>-26.606655001212371</v>
+        <v>-25.807259122346117</v>
       </c>
       <c r="D347">
-        <v>-48.419250768260682</v>
+        <v>-49.206932384677074</v>
       </c>
     </row>
     <row r="348" spans="2:4">
@@ -13334,10 +13334,10 @@
         <v>742</v>
       </c>
       <c r="C348">
-        <v>-20.382411431224103</v>
+        <v>-27.011349164888419</v>
       </c>
       <c r="D348">
-        <v>-53.700225492088805</v>
+        <v>-51.036777370505931</v>
       </c>
     </row>
     <row r="349" spans="2:4">
@@ -13345,10 +13345,10 @@
         <v>743</v>
       </c>
       <c r="C349">
-        <v>-22.11005318258967</v>
+        <v>-26.775277569410729</v>
       </c>
       <c r="D349">
-        <v>-53.946792740805101</v>
+        <v>-49.987040139397152</v>
       </c>
     </row>
     <row r="350" spans="2:4">
@@ -13356,10 +13356,10 @@
         <v>744</v>
       </c>
       <c r="C350">
-        <v>-20.611185909715431</v>
+        <v>-20.883707232056199</v>
       </c>
       <c r="D350">
-        <v>-50.438947220610409</v>
+        <v>-56.760138094544068</v>
       </c>
     </row>
     <row r="351" spans="2:4">
@@ -13367,10 +13367,10 @@
         <v>745</v>
       </c>
       <c r="C351">
-        <v>-22.484770000808226</v>
+        <v>-22.955414324490736</v>
       </c>
       <c r="D351">
-        <v>-50.891359225936746</v>
+        <v>-54.352311066683242</v>
       </c>
     </row>
     <row r="352" spans="2:4">
@@ -13378,10 +13378,10 @@
         <v>746</v>
       </c>
       <c r="C352">
-        <v>-21.196227651708281</v>
+        <v>-24.223456037342338</v>
       </c>
       <c r="D352">
-        <v>-57.021203110316613</v>
+        <v>-52.127413454774775</v>
       </c>
     </row>
     <row r="353" spans="2:4">
@@ -13389,10 +13389,10 @@
         <v>747</v>
       </c>
       <c r="C353">
-        <v>-19.536997697488896</v>
+        <v>-25.236262066013079</v>
       </c>
       <c r="D353">
-        <v>-56.477839613136076</v>
+        <v>-53.353080673286442</v>
       </c>
     </row>
     <row r="354" spans="2:4">
@@ -13400,10 +13400,10 @@
         <v>748</v>
       </c>
       <c r="C354">
-        <v>-17.688394727610671</v>
+        <v>-11.677936963385005</v>
       </c>
       <c r="D354">
-        <v>-56.80351566607748</v>
+        <v>-64.778792032293467</v>
       </c>
     </row>
     <row r="355" spans="2:4">
@@ -13411,10 +13411,10 @@
         <v>749</v>
       </c>
       <c r="C355">
-        <v>-11.205793772429621</v>
+        <v>-9.4786898920949962</v>
       </c>
       <c r="D355">
-        <v>-52.372806573735268</v>
+        <v>-65.224961339494342</v>
       </c>
     </row>
     <row r="356" spans="2:4">
@@ -13422,10 +13422,10 @@
         <v>750</v>
       </c>
       <c r="C356">
-        <v>-10.51524420742685</v>
+        <v>-5.5625584900581444</v>
       </c>
       <c r="D356">
-        <v>-54.437224876101297</v>
+        <v>-67.341786830325262</v>
       </c>
     </row>
     <row r="357" spans="2:4">
@@ -13433,10 +13433,10 @@
         <v>751</v>
       </c>
       <c r="C357">
-        <v>-7.9253183547526111</v>
+        <v>-6.665203457755184</v>
       </c>
       <c r="D357">
-        <v>-49.633822771196449</v>
+        <v>-64.897339432757434</v>
       </c>
     </row>
     <row r="358" spans="2:4">
@@ -13444,10 +13444,10 @@
         <v>752</v>
       </c>
       <c r="C358">
-        <v>-8.6951910903652845</v>
+        <v>-5.732956032658584</v>
       </c>
       <c r="D358">
-        <v>-51.168562564021748</v>
+        <v>-72.068833227143116</v>
       </c>
     </row>
     <row r="359" spans="2:4">
@@ -13455,10 +13455,10 @@
         <v>753</v>
       </c>
       <c r="C359">
-        <v>-13.566509727206537</v>
+        <v>-4.8880682172647409</v>
       </c>
       <c r="D359">
-        <v>-49.683397138663217</v>
+        <v>-69.904781628357057</v>
       </c>
     </row>
     <row r="360" spans="2:4">
@@ -13466,10 +13466,10 @@
         <v>754</v>
       </c>
       <c r="C360">
-        <v>-11.05250052861294</v>
+        <v>-8.6973323293265334</v>
       </c>
       <c r="D360">
-        <v>-49.807333057330133</v>
+        <v>-71.665379878676774</v>
       </c>
     </row>
     <row r="361" spans="2:4">
@@ -13477,10 +13477,10 @@
         <v>755</v>
       </c>
       <c r="C361">
-        <v>-16.489300909311286</v>
+        <v>-9.9371096878896488</v>
       </c>
       <c r="D361">
-        <v>-55.256700065792337</v>
+        <v>-68.498640105424712</v>
       </c>
     </row>
     <row r="362" spans="2:4">
@@ -13488,10 +13488,10 @@
         <v>756</v>
       </c>
       <c r="C362">
-        <v>-18.306171103592614</v>
+        <v>-8.2830025903248714</v>
       </c>
       <c r="D362">
-        <v>-52.988131661819374</v>
+        <v>-67.369052732431996</v>
       </c>
     </row>
     <row r="363" spans="2:4">
@@ -13499,10 +13499,10 @@
         <v>757</v>
       </c>
       <c r="C363">
-        <v>-16.264470818380147</v>
+        <v>-7.2412898356772812</v>
       </c>
       <c r="D363">
-        <v>-49.34209668571895</v>
+        <v>-69.868427092214745</v>
       </c>
     </row>
     <row r="364" spans="2:4">
@@ -13510,10 +13510,10 @@
         <v>758</v>
       </c>
       <c r="C364">
-        <v>-18.44082609859354</v>
+        <v>-8.9613692439963994</v>
       </c>
       <c r="D364">
-        <v>-49.989766729607837</v>
+        <v>-60.961565737352473</v>
       </c>
     </row>
     <row r="365" spans="2:4">
@@ -13521,10 +13521,10 @@
         <v>759</v>
       </c>
       <c r="C365">
-        <v>-15.90184163945896</v>
+        <v>-7.4960972720659012</v>
       </c>
       <c r="D365">
-        <v>-52.588295154901282</v>
+        <v>-63.142837905890175</v>
       </c>
     </row>
     <row r="366" spans="2:4">
@@ -13532,10 +13532,10 @@
         <v>760</v>
       </c>
       <c r="C366">
-        <v>-13.566509727206531</v>
+        <v>-9.6994321631910196</v>
       </c>
       <c r="D366">
-        <v>-54.076925455405352</v>
+        <v>-63.070128833605601</v>
       </c>
     </row>
     <row r="367" spans="2:4">
@@ -13543,10 +13543,10 @@
         <v>761</v>
       </c>
       <c r="C367">
-        <v>-14.262757750735211</v>
+        <v>-12.217529181619728</v>
       </c>
       <c r="D367">
-        <v>-51.550431784387378</v>
+        <v>-62.541107652500472</v>
       </c>
     </row>
     <row r="368" spans="2:4">
@@ -13554,10 +13554,10 @@
         <v>762</v>
       </c>
       <c r="C368">
-        <v>-19.38211474595856</v>
+        <v>-11.361724319365733</v>
       </c>
       <c r="D368">
-        <v>-41.330116220513162</v>
+        <v>-58.340520954190247</v>
       </c>
     </row>
     <row r="369" spans="2:4">
@@ -13565,10 +13565,10 @@
         <v>763</v>
       </c>
       <c r="C369">
-        <v>-17.838281454898095</v>
+        <v>-11.318208817895188</v>
       </c>
       <c r="D369">
-        <v>-41.057457199445935</v>
+        <v>-60.620741961018453</v>
       </c>
     </row>
     <row r="370" spans="2:4">
@@ -13576,10 +13576,10 @@
         <v>764</v>
       </c>
       <c r="C370">
-        <v>-17.463564636679532</v>
+        <v>-13.140515870705434</v>
       </c>
       <c r="D370">
-        <v>-43.075133955343311</v>
+        <v>-59.813527753911572</v>
       </c>
     </row>
     <row r="371" spans="2:4">
@@ -13587,10 +13587,10 @@
         <v>765</v>
       </c>
       <c r="C371">
-        <v>-15.023408716440285</v>
+        <v>-9.4615474218187234</v>
       </c>
       <c r="D371">
-        <v>-41.635494324108421</v>
+        <v>-56.898066778221747</v>
       </c>
     </row>
     <row r="372" spans="2:4">
@@ -13598,10 +13598,10 @@
         <v>766</v>
       </c>
       <c r="C372">
-        <v>-16.039640727449015</v>
+        <v>-7.3252264029582399</v>
       </c>
       <c r="D372">
-        <v>-39.733113382833757</v>
+        <v>-56.817148617130833</v>
       </c>
     </row>
     <row r="373" spans="2:4">
@@ -13609,10 +13609,10 @@
         <v>767</v>
       </c>
       <c r="C373">
-        <v>-16.180159534280975</v>
+        <v>-5.9035507946370318</v>
       </c>
       <c r="D373">
-        <v>-45.113260137820717</v>
+        <v>-53.440721072915188</v>
       </c>
     </row>
     <row r="374" spans="2:4">
@@ -13620,10 +13620,10 @@
         <v>768</v>
       </c>
       <c r="C374">
-        <v>-19.079734565691755</v>
+        <v>-4.1645241064499992</v>
       </c>
       <c r="D374">
-        <v>-44.957666674711717</v>
+        <v>-55.40923658107468</v>
       </c>
     </row>
     <row r="375" spans="2:4">
@@ -13631,10 +13631,10 @@
         <v>769</v>
       </c>
       <c r="C375">
-        <v>-16.880671808339553</v>
+        <v>-5.7536640673496082</v>
       </c>
       <c r="D375">
-        <v>-47.247826825897839</v>
+        <v>-56.712629325721743</v>
       </c>
     </row>
     <row r="376" spans="2:4">
@@ -13642,10 +13642,10 @@
         <v>770</v>
       </c>
       <c r="C376">
-        <v>-22.309902152306229</v>
+        <v>-4.0178435123665857</v>
       </c>
       <c r="D376">
-        <v>-43.178138474413146</v>
+        <v>-62.982450246438873</v>
       </c>
     </row>
     <row r="377" spans="2:4">
@@ -13653,10 +13653,10 @@
         <v>771</v>
       </c>
       <c r="C377">
-        <v>-21.093430162727142</v>
+        <v>-7.0291424678243146</v>
       </c>
       <c r="D377">
-        <v>-42.065110103389983</v>
+        <v>-60.416247695218047</v>
       </c>
     </row>
     <row r="378" spans="2:4">
@@ -13664,10 +13664,10 @@
         <v>772</v>
       </c>
       <c r="C378">
-        <v>-21.060846091577702</v>
+        <v>-5.6412490218840405</v>
       </c>
       <c r="D378">
-        <v>-44.844388047601669</v>
+        <v>-61.688656460198366</v>
       </c>
     </row>
     <row r="379" spans="2:4">
@@ -13675,10 +13675,10 @@
         <v>773</v>
       </c>
       <c r="C379">
-        <v>-22.110053182589667</v>
+        <v>-1.7935886020853082</v>
       </c>
       <c r="D379">
-        <v>-45.69266055758856</v>
+        <v>-56.797318870144117</v>
       </c>
     </row>
     <row r="380" spans="2:4">
@@ -13686,10 +13686,10 @@
         <v>774</v>
       </c>
       <c r="C380">
-        <v>-20.664716883746653</v>
+        <v>-3.3742122716617691</v>
       </c>
       <c r="D380">
-        <v>-47.912884014850157</v>
+        <v>-57.663689958729989</v>
       </c>
     </row>
     <row r="381" spans="2:4">
@@ -13697,10 +13697,10 @@
         <v>775</v>
       </c>
       <c r="C381">
-        <v>-19.392541648726372</v>
+        <v>-2.6247786352246538</v>
       </c>
       <c r="D381">
-        <v>-47.06781040297102</v>
+        <v>-60.182539962874714</v>
       </c>
     </row>
     <row r="382" spans="2:4">
@@ -13708,10 +13708,10 @@
         <v>776</v>
       </c>
       <c r="C382">
-        <v>-8.7156301895408426</v>
+        <v>-4.4076418124329484</v>
       </c>
       <c r="D382">
-        <v>-71.752253055951869</v>
+        <v>-60.100537249771811</v>
       </c>
     </row>
     <row r="383" spans="2:4">
@@ -13719,10 +13719,10 @@
         <v>777</v>
       </c>
       <c r="C383">
-        <v>-4.7531701627060601</v>
+        <v>-1.844333951762555</v>
       </c>
       <c r="D383">
-        <v>-70.013845236783936</v>
+        <v>-49.867164190479677</v>
       </c>
     </row>
     <row r="384" spans="2:4">
@@ -13730,10 +13730,10 @@
         <v>778</v>
       </c>
       <c r="C384">
-        <v>-5.8693854376818102</v>
+        <v>-4.2893101856270874</v>
       </c>
       <c r="D384">
-        <v>-72.124546835163073</v>
+        <v>-49.91170014673385</v>
       </c>
     </row>
     <row r="385" spans="2:4">
@@ -13741,10 +13741,10 @@
         <v>779</v>
       </c>
       <c r="C385">
-        <v>-6.9253747335484057</v>
+        <v>-6.139363964722846</v>
       </c>
       <c r="D385">
-        <v>-70.231972453637695</v>
+        <v>-50.544110725543099</v>
       </c>
     </row>
     <row r="386" spans="2:4">
@@ -13752,10 +13752,10 @@
         <v>780</v>
       </c>
       <c r="C386">
-        <v>-8.075922243414615</v>
+        <v>1.7083103899935743</v>
       </c>
       <c r="D386">
-        <v>-64.807492981879449</v>
+        <v>-50.91449393075456</v>
       </c>
     </row>
     <row r="387" spans="2:4">
@@ -13763,10 +13763,10 @@
         <v>781</v>
       </c>
       <c r="C387">
-        <v>-5.6439255705856022</v>
+        <v>1.1759205209921435</v>
       </c>
       <c r="D387">
-        <v>-66.051200797273779</v>
+        <v>-55.15782371749323</v>
       </c>
     </row>
     <row r="388" spans="2:4">
@@ -13774,10 +13774,10 @@
         <v>782</v>
       </c>
       <c r="C388">
-        <v>-9.7806610992693646</v>
+        <v>-1.9586154028361076</v>
       </c>
       <c r="D388">
-        <v>-68.648791040989394</v>
+        <v>-52.175886169631163</v>
       </c>
     </row>
     <row r="389" spans="2:4">
@@ -13785,10 +13785,10 @@
         <v>783</v>
       </c>
       <c r="C389">
-        <v>-11.121482488330445</v>
+        <v>-2.5498352715809425</v>
       </c>
       <c r="D389">
-        <v>-64.778792032293467</v>
+        <v>-54.230296154755656</v>
       </c>
     </row>
     <row r="390" spans="2:4">
@@ -13796,10 +13796,10 @@
         <v>784</v>
       </c>
       <c r="C390">
-        <v>-8.5827760448997186</v>
+        <v>0.78173789403495986</v>
       </c>
       <c r="D390">
-        <v>-67.028228956097962</v>
+        <v>-68.596018327234432</v>
       </c>
     </row>
     <row r="391" spans="2:4">
@@ -13807,10 +13807,10 @@
         <v>785</v>
       </c>
       <c r="C391">
-        <v>-9.6994321631910196</v>
+        <v>-2.4655239874817667</v>
       </c>
       <c r="D391">
-        <v>-63.070128833605601</v>
+        <v>-68.800512593034838</v>
       </c>
     </row>
     <row r="392" spans="2:4">
@@ -13818,10 +13818,10 @@
         <v>786</v>
       </c>
       <c r="C392">
-        <v>-7.4960972720659012</v>
+        <v>0.68425911335153089</v>
       </c>
       <c r="D392">
-        <v>-63.142837905890175</v>
+        <v>-64.778792032293467</v>
       </c>
     </row>
     <row r="393" spans="2:4">
@@ -13829,10 +13829,10 @@
         <v>787</v>
       </c>
       <c r="C393">
-        <v>-8.8744034816872048</v>
+        <v>-2.5948012897671693</v>
       </c>
       <c r="D393">
-        <v>-61.388336379022896</v>
+        <v>-66.033023529202637</v>
       </c>
     </row>
     <row r="394" spans="2:4">
@@ -13840,10 +13840,10 @@
         <v>788</v>
       </c>
       <c r="C394">
-        <v>-6.1631760186884605</v>
+        <v>3.4177977134197421</v>
       </c>
       <c r="D394">
-        <v>-60.163064318512767</v>
+        <v>-60.883663159904685</v>
       </c>
     </row>
     <row r="395" spans="2:4">
@@ -13851,10 +13851,10 @@
         <v>789</v>
       </c>
       <c r="C395">
-        <v>-3.7148639245877302</v>
+        <v>1.0871220817168219</v>
       </c>
       <c r="D395">
-        <v>-63.241986640823711</v>
+        <v>-60.640790418449861</v>
       </c>
     </row>
     <row r="396" spans="2:4">
@@ -13862,10 +13862,10 @@
         <v>790</v>
       </c>
       <c r="C396">
-        <v>-5.3227397263982672</v>
+        <v>-0.2265909986258858</v>
       </c>
       <c r="D396">
-        <v>-62.256696087421737</v>
+        <v>-62.688406204111487</v>
       </c>
     </row>
     <row r="397" spans="2:4">
@@ -13873,10 +13873,10 @@
         <v>791</v>
       </c>
       <c r="C397">
-        <v>-13.819443579504057</v>
+        <v>-1.1687361415754016</v>
       </c>
       <c r="D397">
-        <v>-56.53085664501026</v>
+        <v>-61.078419603524146</v>
       </c>
     </row>
     <row r="398" spans="2:4">
@@ -13884,10 +13884,10 @@
         <v>792</v>
       </c>
       <c r="C398">
-        <v>-11.842812363401167</v>
+        <v>-11.767868999757455</v>
       </c>
       <c r="D398">
-        <v>-56.053703358142648</v>
+        <v>-41.875434262647573</v>
       </c>
     </row>
     <row r="399" spans="2:4">
@@ -13895,10 +13895,10 @@
         <v>793</v>
       </c>
       <c r="C399">
-        <v>-9.2010587949603355</v>
+        <v>-9.4895907449886234</v>
       </c>
       <c r="D399">
-        <v>-56.894402006433211</v>
+        <v>-42.202625087928233</v>
       </c>
     </row>
     <row r="400" spans="2:4">
@@ -13906,10 +13906,10 @@
         <v>794</v>
       </c>
       <c r="C400">
-        <v>-9.7443981813772478</v>
+        <v>-12.901794675757964</v>
       </c>
       <c r="D400">
-        <v>-59.325611610949181</v>
+        <v>-43.463969428865255</v>
       </c>
     </row>
     <row r="401" spans="2:4">
@@ -13917,10 +13917,10 @@
         <v>795</v>
       </c>
       <c r="C401">
-        <v>-11.382445986732655</v>
+        <v>-15.347855832276291</v>
       </c>
       <c r="D401">
-        <v>-58.001267794337032</v>
+        <v>-44.119627743739251</v>
       </c>
     </row>
     <row r="402" spans="2:4">
@@ -13928,10 +13928,10 @@
         <v>796</v>
       </c>
       <c r="C402">
-        <v>-15.497403449320981</v>
+        <v>-9.5876984210313037</v>
       </c>
       <c r="D402">
-        <v>-59.710541993632312</v>
+        <v>-47.559961732170073</v>
       </c>
     </row>
     <row r="403" spans="2:4">
@@ -13939,10 +13939,10 @@
         <v>797</v>
       </c>
       <c r="C403">
-        <v>-14.780592218234659</v>
+        <v>-12.912458553588689</v>
       </c>
       <c r="D403">
-        <v>-57.925961969470833</v>
+        <v>-46.11404268105607</v>
       </c>
     </row>
     <row r="404" spans="2:4">
@@ -13950,10 +13950,10 @@
         <v>798</v>
       </c>
       <c r="C404">
-        <v>-11.82182822158093</v>
+        <v>-13.116849545344261</v>
       </c>
       <c r="D404">
-        <v>-60.45987313858879</v>
+        <v>-47.951835303574043</v>
       </c>
     </row>
     <row r="405" spans="2:4">
@@ -13961,10 +13961,10 @@
         <v>799</v>
       </c>
       <c r="C405">
-        <v>-12.402683374151248</v>
+        <v>-7.3611992175072203</v>
       </c>
       <c r="D405">
-        <v>-62.22862824701776</v>
+        <v>-44.356631354359209</v>
       </c>
     </row>
     <row r="406" spans="2:4">
@@ -13972,10 +13972,10 @@
         <v>800</v>
       </c>
       <c r="C406">
-        <v>3.103035586116154</v>
+        <v>-10.408431240638969</v>
       </c>
       <c r="D406">
-        <v>-51.262694845104477</v>
+        <v>-44.982478921320464</v>
       </c>
     </row>
     <row r="407" spans="2:4">
@@ -13983,10 +13983,10 @@
         <v>801</v>
       </c>
       <c r="C407">
-        <v>0.4504835280862664</v>
+        <v>-4.303509980843792</v>
       </c>
       <c r="D407">
-        <v>-51.352685753535525</v>
+        <v>-39.460454361766537</v>
       </c>
     </row>
     <row r="408" spans="2:4">
@@ -13994,10 +13994,10 @@
         <v>802</v>
       </c>
       <c r="C408">
-        <v>-2.7318405832870987</v>
+        <v>-4.191776238684076</v>
       </c>
       <c r="D408">
-        <v>-53.976301292868648</v>
+        <v>-42.602524985493474</v>
       </c>
     </row>
     <row r="409" spans="2:4">
@@ -14005,10 +14005,10 @@
         <v>803</v>
       </c>
       <c r="C409">
-        <v>-2.4299258897510043</v>
+        <v>-6.4930091740654543</v>
       </c>
       <c r="D409">
-        <v>-51.981995310205598</v>
+        <v>-40.721876865824747</v>
       </c>
     </row>
     <row r="410" spans="2:4">
@@ -14016,10 +14016,10 @@
         <v>804</v>
       </c>
       <c r="C410">
-        <v>-1.6016388011322449</v>
+        <v>-1.9811473945198379</v>
       </c>
       <c r="D410">
-        <v>-49.699562693271943</v>
+        <v>-46.141746004052202</v>
       </c>
     </row>
     <row r="411" spans="2:4">
@@ -14027,10 +14027,10 @@
         <v>805</v>
       </c>
       <c r="C411">
-        <v>-4.9139577428871144</v>
+        <v>-6.5030977037867244</v>
       </c>
       <c r="D411">
-        <v>-49.972580948886019</v>
+        <v>-47.533108949792243</v>
       </c>
     </row>
     <row r="412" spans="2:4">
@@ -14038,10 +14038,10 @@
         <v>806</v>
       </c>
       <c r="C412">
-        <v>-1.4706508351114969</v>
+        <v>-4.1063512857195654</v>
       </c>
       <c r="D412">
-        <v>-59.870929653083614</v>
+        <v>-47.265693371437855</v>
       </c>
     </row>
     <row r="413" spans="2:4">
@@ -14049,10 +14049,10 @@
         <v>807</v>
       </c>
       <c r="C413">
-        <v>-3.2243255443743459</v>
+        <v>-5.2400436009983089</v>
       </c>
       <c r="D413">
-        <v>-60.623987901745423</v>
+        <v>-44.451591909972265</v>
       </c>
     </row>
     <row r="414" spans="2:4">
@@ -14060,10 +14060,10 @@
         <v>808</v>
       </c>
       <c r="C414">
-        <v>1.1598612287827772</v>
+        <v>-6.8526180462974819</v>
       </c>
       <c r="D414">
-        <v>-56.008260187964773</v>
+        <v>-36.41285180609411</v>
       </c>
     </row>
     <row r="415" spans="2:4">
@@ -14071,10 +14071,10 @@
         <v>809</v>
       </c>
       <c r="C415">
-        <v>-4.0198781738229759</v>
+        <v>-8.6347528938784208</v>
       </c>
       <c r="D415">
-        <v>-57.605762401140623</v>
+        <v>-39.518253048260057</v>
       </c>
     </row>
     <row r="416" spans="2:4">
@@ -14082,10 +14082,10 @@
         <v>810</v>
       </c>
       <c r="C416">
-        <v>-1.9913863360423181</v>
+        <v>-11.717906757328317</v>
       </c>
       <c r="D416">
-        <v>-57.021203110316613</v>
+        <v>-38.724707796982003</v>
       </c>
     </row>
     <row r="417" spans="2:4">
@@ -14093,10 +14093,10 @@
         <v>811</v>
       </c>
       <c r="C417">
-        <v>-6.8109008044662529</v>
+        <v>-9.9551763916251836</v>
       </c>
       <c r="D417">
-        <v>-56.62498892609301</v>
+        <v>-37.325436848588453</v>
       </c>
     </row>
     <row r="418" spans="2:4">
@@ -14104,10 +14104,10 @@
         <v>812</v>
       </c>
       <c r="C418">
-        <v>-4.2735326353863066</v>
+        <v>-17.538508000323247</v>
       </c>
       <c r="D418">
-        <v>-54.932771827088544</v>
+        <v>-41.60277524158036</v>
       </c>
     </row>
     <row r="419" spans="2:4">
@@ -14115,10 +14115,10 @@
         <v>813</v>
       </c>
       <c r="C419">
-        <v>-6.1833796443712101</v>
+        <v>-18.921553711202652</v>
       </c>
       <c r="D419">
-        <v>-52.711431486996162</v>
+        <v>-42.519901039715528</v>
       </c>
     </row>
     <row r="420" spans="2:4">
@@ -14126,10 +14126,10 @@
         <v>814</v>
       </c>
       <c r="C420">
-        <v>-7.3577402930313562</v>
+        <v>-19.648755345027759</v>
       </c>
       <c r="D420">
-        <v>-41.896408033498901</v>
+        <v>-40.641293430448606</v>
       </c>
     </row>
     <row r="421" spans="2:4">
@@ -14137,10 +14137,10 @@
         <v>815</v>
       </c>
       <c r="C421">
-        <v>-7.4711161508513291</v>
+        <v>-12.506596441388329</v>
       </c>
       <c r="D421">
-        <v>-44.682812331413686</v>
+        <v>-40.258955780606243</v>
       </c>
     </row>
     <row r="422" spans="2:4">
@@ -14148,10 +14148,10 @@
         <v>816</v>
       </c>
       <c r="C422">
-        <v>-5.729575129035557</v>
+        <v>-15.023408716440285</v>
       </c>
       <c r="D422">
-        <v>-44.056706431185262</v>
+        <v>-41.635494324108421</v>
       </c>
     </row>
     <row r="423" spans="2:4">
@@ -14159,10 +14159,10 @@
         <v>817</v>
       </c>
       <c r="C423">
-        <v>-6.3505344277977391</v>
+        <v>-16.039640727449015</v>
       </c>
       <c r="D423">
-        <v>-47.432484787255532</v>
+        <v>-39.733113382833757</v>
       </c>
     </row>
     <row r="424" spans="2:4">
@@ -14170,10 +14170,10 @@
         <v>818</v>
       </c>
       <c r="C424">
-        <v>-4.1063512857195654</v>
+        <v>-11.205793772429621</v>
       </c>
       <c r="D424">
-        <v>-47.265693371437855</v>
+        <v>-52.372806573735268</v>
       </c>
     </row>
     <row r="425" spans="2:4">
@@ -14181,10 +14181,10 @@
         <v>819</v>
       </c>
       <c r="C425">
-        <v>-4.0750339965462077</v>
+        <v>-10.51524420742685</v>
       </c>
       <c r="D425">
-        <v>-43.157668577936633</v>
+        <v>-54.437224876101297</v>
       </c>
     </row>
     <row r="426" spans="2:4">
@@ -14192,10 +14192,10 @@
         <v>820</v>
       </c>
       <c r="C426">
-        <v>-1.9811473945198379</v>
+        <v>-12.032374989088204</v>
       </c>
       <c r="D426">
-        <v>-46.141746004052202</v>
+        <v>-50.039166128718826</v>
       </c>
     </row>
     <row r="427" spans="2:4">
@@ -14203,10 +14203,10 @@
         <v>821</v>
       </c>
       <c r="C427">
-        <v>-10.32350599135138</v>
+        <v>-8.6006972840319094</v>
       </c>
       <c r="D427">
-        <v>-42.123306099981406</v>
+        <v>-50.434556576148779</v>
       </c>
     </row>
     <row r="428" spans="2:4">
@@ -14214,10 +14214,10 @@
         <v>822</v>
       </c>
       <c r="C428">
-        <v>-13.744007167415322</v>
+        <v>-16.902698173281436</v>
       </c>
       <c r="D428">
-        <v>-43.511388389050843</v>
+        <v>-50.477386604703518</v>
       </c>
     </row>
     <row r="429" spans="2:4">
@@ -14225,10 +14225,10 @@
         <v>823</v>
       </c>
       <c r="C429">
-        <v>-14.590735697003923</v>
+        <v>-14.562185844187271</v>
       </c>
       <c r="D429">
-        <v>-47.813341832555771</v>
+        <v>-50.808263143325782</v>
       </c>
     </row>
     <row r="430" spans="2:4">
@@ -14236,10 +14236,10 @@
         <v>824</v>
       </c>
       <c r="C430">
-        <v>-12.399534493325881</v>
+        <v>-15.907048622540906</v>
       </c>
       <c r="D430">
-        <v>-46.96506932256888</v>
+        <v>-54.263941578829673</v>
       </c>
     </row>
     <row r="431" spans="2:4">
@@ -14247,10 +14247,10 @@
         <v>825</v>
       </c>
       <c r="C431">
-        <v>-8.9735521553276421</v>
+        <v>-13.566509727206531</v>
       </c>
       <c r="D431">
-        <v>-47.562322416335135</v>
+        <v>-54.076925455405352</v>
       </c>
     </row>
     <row r="432" spans="2:4">
@@ -14258,10 +14258,10 @@
         <v>826</v>
       </c>
       <c r="C432">
-        <v>-10.308971520826541</v>
+        <v>-12.986303040932638</v>
       </c>
       <c r="D432">
-        <v>-45.062515264455449</v>
+        <v>-56.282385117747381</v>
       </c>
     </row>
     <row r="433" spans="2:4">
@@ -14269,10 +14269,10 @@
         <v>827</v>
       </c>
       <c r="C433">
-        <v>-12.410240688132127</v>
+        <v>-24.317475893549901</v>
       </c>
       <c r="D433">
-        <v>-40.453712224225683</v>
+        <v>-47.675635256259191</v>
       </c>
     </row>
     <row r="434" spans="2:4">
@@ -14280,10 +14280,10 @@
         <v>828</v>
       </c>
       <c r="C434">
-        <v>-9.1341450774213087</v>
+        <v>-26.606655001212371</v>
       </c>
       <c r="D434">
-        <v>-39.798032197373566</v>
+        <v>-48.419250768260682</v>
       </c>
     </row>
     <row r="435" spans="2:4">
@@ -14291,10 +14291,10 @@
         <v>829</v>
       </c>
       <c r="C435">
-        <v>-10.275814759941746</v>
+        <v>-23.369101691804023</v>
       </c>
       <c r="D435">
-        <v>-37.711187395439225</v>
+        <v>-45.747192361801993</v>
       </c>
     </row>
     <row r="436" spans="2:4">
@@ -14302,10 +14302,10 @@
         <v>830</v>
       </c>
       <c r="C436">
-        <v>-11.789281389369949</v>
+        <v>-22.709600091739361</v>
       </c>
       <c r="D436">
-        <v>-38.837233742184345</v>
+        <v>-47.764869117699376</v>
       </c>
     </row>
     <row r="437" spans="2:4">
@@ -14313,10 +14313,10 @@
         <v>831</v>
       </c>
       <c r="C437">
-        <v>-7.2391485967160323</v>
+        <v>-20.761072637002851</v>
       </c>
       <c r="D437">
-        <v>-36.468995387771983</v>
+        <v>-47.873932726126263</v>
       </c>
     </row>
     <row r="438" spans="2:4">
@@ -14324,10 +14324,10 @@
         <v>832</v>
       </c>
       <c r="C438">
-        <v>-6.5558987099902479</v>
+        <v>-21.990143800759729</v>
       </c>
       <c r="D438">
-        <v>-39.793310829043406</v>
+        <v>-45.801724166015447</v>
       </c>
     </row>
     <row r="439" spans="2:4">
@@ -14335,10 +14335,10 @@
         <v>833</v>
       </c>
       <c r="C439">
-        <v>-4.2778151133088054</v>
+        <v>-22.309902152306229</v>
       </c>
       <c r="D439">
-        <v>-39.47603487725609</v>
+        <v>-43.178138474413146</v>
       </c>
     </row>
     <row r="440" spans="2:4">
@@ -14346,10 +14346,10 @@
         <v>834</v>
       </c>
       <c r="C440">
-        <v>0.78173789403495986</v>
+        <v>-21.093430162727142</v>
       </c>
       <c r="D440">
-        <v>-68.596018327234432</v>
+        <v>-42.065110103389983</v>
       </c>
     </row>
     <row r="441" spans="2:4">
@@ -14357,10 +14357,10 @@
         <v>835</v>
       </c>
       <c r="C441">
-        <v>-2.4655239874817667</v>
+        <v>-18.422839691319048</v>
       </c>
       <c r="D441">
-        <v>-68.800512593034838</v>
+        <v>-47.98299633455315</v>
       </c>
     </row>
     <row r="442" spans="2:4">
@@ -14368,10 +14368,10 @@
         <v>836</v>
       </c>
       <c r="C442">
-        <v>0.68425911335153089</v>
+        <v>-20.311412455140584</v>
       </c>
       <c r="D442">
-        <v>-64.778792032293467</v>
+        <v>-45.536855402693007</v>
       </c>
     </row>
     <row r="443" spans="2:4">
@@ -14379,10 +14379,10 @@
         <v>837</v>
       </c>
       <c r="C443">
-        <v>-2.5948012897671693</v>
+        <v>-16.558479398828556</v>
       </c>
       <c r="D443">
-        <v>-66.033023529202637</v>
+        <v>-47.370562225694478</v>
       </c>
     </row>
     <row r="444" spans="2:4">
@@ -14390,10 +14390,10 @@
         <v>838</v>
       </c>
       <c r="C444">
-        <v>3.2839139299479689</v>
+        <v>-15.76984461833165</v>
       </c>
       <c r="D444">
-        <v>-60.889813363387418</v>
+        <v>-46.074383187082653</v>
       </c>
     </row>
     <row r="445" spans="2:4">
@@ -14401,10 +14401,10 @@
         <v>839</v>
       </c>
       <c r="C445">
-        <v>0.62990458587367415</v>
+        <v>-18.724376519156099</v>
       </c>
       <c r="D445">
-        <v>-60.260442540322501</v>
+        <v>-45.083187451673609</v>
       </c>
     </row>
     <row r="446" spans="2:4">
@@ -14412,10 +14412,10 @@
         <v>840</v>
       </c>
       <c r="C446">
-        <v>-0.39411145853535851</v>
+        <v>-17.645569948385692</v>
       </c>
       <c r="D446">
-        <v>-62.453170970249573</v>
+        <v>-43.861949987565843</v>
       </c>
     </row>
     <row r="447" spans="2:4">
@@ -14423,10 +14423,10 @@
         <v>841</v>
       </c>
       <c r="C447">
-        <v>-14.17968270247326</v>
+        <v>-23.035824145247283</v>
       </c>
       <c r="D447">
-        <v>-58.284549894147112</v>
+        <v>-49.958972298993167</v>
       </c>
     </row>
     <row r="448" spans="2:4">
@@ -14434,10 +14434,10 @@
         <v>842</v>
       </c>
       <c r="C448">
-        <v>-18.437828364047789</v>
+        <v>-23.548965764548932</v>
       </c>
       <c r="D448">
-        <v>-56.09914652832051</v>
+        <v>-46.892360250284291</v>
       </c>
     </row>
     <row r="449" spans="2:4">
@@ -14445,10 +14445,10 @@
         <v>843</v>
       </c>
       <c r="C449">
-        <v>-17.035316844429754</v>
+        <v>-23.493622972935107</v>
       </c>
       <c r="D449">
-        <v>-58.273926815404231</v>
+        <v>-48.335355684855394</v>
       </c>
     </row>
     <row r="450" spans="2:4">
@@ -14456,10 +14456,10 @@
         <v>844</v>
       </c>
       <c r="C450">
-        <v>-19.476329260253511</v>
+        <v>-19.412092091416039</v>
       </c>
       <c r="D450">
-        <v>-55.196775006217123</v>
+        <v>-44.874683494386922</v>
       </c>
     </row>
     <row r="451" spans="2:4">
@@ -14467,10 +14467,10 @@
         <v>845</v>
       </c>
       <c r="C451">
-        <v>-19.974167318743884</v>
+        <v>-20.940936709747763</v>
       </c>
       <c r="D451">
-        <v>-54.008760700138552</v>
+        <v>-44.492960864892822</v>
       </c>
     </row>
     <row r="452" spans="2:4">
@@ -14478,10 +14478,10 @@
         <v>846</v>
       </c>
       <c r="C452">
-        <v>-19.611941061132608</v>
+        <v>-20.96092160671942</v>
       </c>
       <c r="D452">
-        <v>-52.418249743913137</v>
+        <v>-47.995114513267239</v>
       </c>
     </row>
     <row r="453" spans="2:4">
@@ -14489,10 +14489,10 @@
         <v>847</v>
       </c>
       <c r="C453">
-        <v>-17.838281454898095</v>
+        <v>-21.922694773480387</v>
       </c>
       <c r="D453">
-        <v>-52.859697682783867</v>
+        <v>-48.237478087549214</v>
       </c>
     </row>
     <row r="454" spans="2:4">
@@ -14500,10 +14500,10 @@
         <v>848</v>
       </c>
       <c r="C454">
-        <v>-22.074080368040683</v>
+        <v>-27.345382442843249</v>
       </c>
       <c r="D454">
-        <v>-54.832190943761525</v>
+        <v>-51.53535386617169</v>
       </c>
     </row>
     <row r="455" spans="2:4">
@@ -14511,10 +14511,10 @@
         <v>849</v>
       </c>
       <c r="C455">
-        <v>-21.092401192059267</v>
+        <v>-28.899921928709954</v>
       </c>
       <c r="D455">
-        <v>-57.574853686201827</v>
+        <v>-51.25490458735969</v>
       </c>
     </row>
     <row r="456" spans="2:4">
@@ -14522,10 +14522,10 @@
         <v>850</v>
       </c>
       <c r="C456">
-        <v>-19.681888200533407</v>
+        <v>-28.180465637730322</v>
       </c>
       <c r="D456">
-        <v>-56.889857689415422</v>
+        <v>-50.259699160464372</v>
       </c>
     </row>
     <row r="457" spans="2:4">
@@ -14533,10 +14533,10 @@
         <v>851</v>
       </c>
       <c r="C457">
-        <v>-28.904918152952877</v>
+        <v>-25.932164728418968</v>
       </c>
       <c r="D457">
-        <v>-55.266021741726256</v>
+        <v>-49.946141286237072</v>
       </c>
     </row>
     <row r="458" spans="2:4">
@@ -14544,10 +14544,10 @@
         <v>852</v>
       </c>
       <c r="C458">
-        <v>-28.092488645626837</v>
+        <v>-25.068343852736184</v>
       </c>
       <c r="D458">
-        <v>-53.374532107656123</v>
+        <v>-51.088439079760768</v>
       </c>
     </row>
     <row r="459" spans="2:4">
@@ -14555,10 +14555,10 @@
         <v>853</v>
       </c>
       <c r="C459">
-        <v>-30.336189450775912</v>
+        <v>-28.904918152952877</v>
       </c>
       <c r="D459">
-        <v>-52.396864722652957</v>
+        <v>-55.266021741726256</v>
       </c>
     </row>
     <row r="460" spans="2:4">
@@ -14566,10 +14566,10 @@
         <v>854</v>
       </c>
       <c r="C460">
-        <v>-30.611440995923225</v>
+        <v>-28.135499619544092</v>
       </c>
       <c r="D460">
-        <v>-55.184602728490901</v>
+        <v>-53.572506266431006</v>
       </c>
     </row>
     <row r="461" spans="2:4">
@@ -14588,10 +14588,10 @@
         <v>856</v>
       </c>
       <c r="C462">
-        <v>-28.630125819592596</v>
+        <v>-30.336189450775912</v>
       </c>
       <c r="D462">
-        <v>-50.146091235019703</v>
+        <v>-52.396864722652957</v>
       </c>
     </row>
     <row r="463" spans="2:4">
@@ -14599,10 +14599,10 @@
         <v>857</v>
       </c>
       <c r="C463">
-        <v>-28.899921928709954</v>
+        <v>-30.611440995923225</v>
       </c>
       <c r="D463">
-        <v>-51.25490458735969</v>
+        <v>-55.184602728490901</v>
       </c>
     </row>
     <row r="464" spans="2:4">
@@ -14610,10 +14610,10 @@
         <v>858</v>
       </c>
       <c r="C464">
-        <v>-21.833339224520579</v>
+        <v>-14.17968270247326</v>
       </c>
       <c r="D464">
-        <v>-50.810260645311615</v>
+        <v>-58.284549894147112</v>
       </c>
     </row>
     <row r="465" spans="2:4">
@@ -14621,10 +14621,10 @@
         <v>859</v>
       </c>
       <c r="C465">
-        <v>-21.435562909796261</v>
+        <v>-21.092401192059267</v>
       </c>
       <c r="D465">
-        <v>-52.463692914091013</v>
+        <v>-57.574853686201827</v>
       </c>
     </row>
     <row r="466" spans="2:4">
@@ -14632,10 +14632,10 @@
         <v>860</v>
       </c>
       <c r="C466">
-        <v>-23.90869391003875</v>
+        <v>-17.135687420738297</v>
       </c>
       <c r="D466">
-        <v>-51.09130917471937</v>
+        <v>-58.064563638513327</v>
       </c>
     </row>
     <row r="467" spans="2:4">
@@ -14643,10 +14643,10 @@
         <v>861</v>
       </c>
       <c r="C467">
-        <v>-23.530032704259995</v>
+        <v>-18.635406322744849</v>
       </c>
       <c r="D467">
-        <v>-52.523486559061887</v>
+        <v>-55.954554623209113</v>
       </c>
     </row>
     <row r="468" spans="2:4">
@@ -14654,10 +14654,10 @@
         <v>862</v>
       </c>
       <c r="C468">
-        <v>-25.077810382880653</v>
+        <v>-19.681888200533407</v>
       </c>
       <c r="D468">
-        <v>-54.046932963087968</v>
+        <v>-56.889857689415422</v>
       </c>
     </row>
     <row r="469" spans="2:4">
@@ -14665,10 +14665,10 @@
         <v>863</v>
       </c>
       <c r="C469">
-        <v>-27.337352796738564</v>
+        <v>-21.840257073472305</v>
       </c>
       <c r="D469">
-        <v>-51.14584097893281</v>
+        <v>-51.000422834363619</v>
       </c>
     </row>
     <row r="470" spans="2:4">
@@ -14676,10 +14676,10 @@
         <v>864</v>
       </c>
       <c r="C470">
-        <v>-25.91717605569022</v>
+        <v>-23.4162089489515</v>
       </c>
       <c r="D470">
-        <v>-52.381895207770853</v>
+        <v>-52.548087372992768</v>
       </c>
     </row>
     <row r="471" spans="2:4">
@@ -14687,10 +14687,10 @@
         <v>865</v>
       </c>
       <c r="C471">
-        <v>-25.557447910200409</v>
+        <v>-25.83580897516277</v>
       </c>
       <c r="D471">
-        <v>-50.18504252374359</v>
+        <v>-53.482918302366073</v>
       </c>
     </row>
     <row r="472" spans="2:4">
@@ -14698,10 +14698,10 @@
         <v>866</v>
       </c>
       <c r="C472">
-        <v>-19.412092091416039</v>
+        <v>-21.685374121941965</v>
       </c>
       <c r="D472">
-        <v>-44.874683494386922</v>
+        <v>-55.175135401370511</v>
       </c>
     </row>
     <row r="473" spans="2:4">
@@ -14709,10 +14709,10 @@
         <v>867</v>
       </c>
       <c r="C473">
-        <v>-20.940936709747763</v>
+        <v>-23.144271600872891</v>
       </c>
       <c r="D473">
-        <v>-44.492960864892822</v>
+        <v>-54.363217427525932</v>
       </c>
     </row>
     <row r="474" spans="2:4">
@@ -14720,10 +14720,10 @@
         <v>868</v>
       </c>
       <c r="C474">
-        <v>-22.217115130652115</v>
+        <v>-15.927225681983444</v>
       </c>
       <c r="D474">
-        <v>-48.704893552235859</v>
+        <v>-49.918875384130345</v>
       </c>
     </row>
     <row r="475" spans="2:4">
@@ -14731,10 +14731,10 @@
         <v>869</v>
       </c>
       <c r="C475">
-        <v>-23.548965764548932</v>
+        <v>-17.50968362969105</v>
       </c>
       <c r="D475">
-        <v>-46.892360250284291</v>
+        <v>-50.768313103608975</v>
       </c>
     </row>
     <row r="476" spans="2:4">
@@ -14742,10 +14742,10 @@
         <v>870</v>
       </c>
       <c r="C476">
-        <v>-23.518988419091443</v>
+        <v>-20.311412455140584</v>
       </c>
       <c r="D476">
-        <v>-48.564668912829866</v>
+        <v>-52.42894225454323</v>
       </c>
     </row>
     <row r="477" spans="2:4">
@@ -14753,10 +14753,10 @@
         <v>871</v>
       </c>
       <c r="C477">
-        <v>-12.195046172526611</v>
+        <v>-19.243469523217691</v>
       </c>
       <c r="D477">
-        <v>-42.202625087928219</v>
+        <v>-49.57805160779634</v>
       </c>
     </row>
     <row r="478" spans="2:4">
@@ -14764,10 +14764,10 @@
         <v>872</v>
       </c>
       <c r="C478">
-        <v>-7.3121453794858811</v>
+        <v>-20.2552049324078</v>
       </c>
       <c r="D478">
-        <v>-38.950546582108387</v>
+        <v>-50.430111048631375</v>
       </c>
     </row>
     <row r="479" spans="2:4">
@@ -14775,10 +14775,10 @@
         <v>873</v>
       </c>
       <c r="C479">
-        <v>-9.5524700549726198</v>
+        <v>-18.095230130247963</v>
       </c>
       <c r="D479">
-        <v>-39.601059013745463</v>
+        <v>-53.482918302366059</v>
       </c>
     </row>
     <row r="480" spans="2:4">
@@ -14786,10 +14786,10 @@
         <v>874</v>
       </c>
       <c r="C480">
-        <v>-15.814810636517883</v>
+        <v>-19.909084924000659</v>
       </c>
       <c r="D480">
-        <v>-41.506025266362961</v>
+        <v>-54.360347332567322</v>
       </c>
     </row>
     <row r="481" spans="2:4">
@@ -14797,10 +14797,10 @@
         <v>875</v>
       </c>
       <c r="C481">
-        <v>-12.237079624309391</v>
+        <v>-11.719691123129357</v>
       </c>
       <c r="D481">
-        <v>-40.049804295501879</v>
+        <v>-41.739104752113967</v>
       </c>
     </row>
     <row r="482" spans="2:4">
@@ -14808,10 +14808,10 @@
         <v>876</v>
       </c>
       <c r="C482">
-        <v>-13.22926459080983</v>
+        <v>-7.3121453794858811</v>
       </c>
       <c r="D482">
-        <v>-39.148844051975445</v>
+        <v>-38.950546582108387</v>
       </c>
     </row>
     <row r="483" spans="2:4">
@@ -14819,10 +14819,10 @@
         <v>877</v>
       </c>
       <c r="C483">
-        <v>-10.618737423887216</v>
+        <v>-8.9973820727996046</v>
       </c>
       <c r="D483">
-        <v>-37.967321627350856</v>
+        <v>-39.13125314739046</v>
       </c>
     </row>
     <row r="484" spans="2:4">
@@ -14830,10 +14830,10 @@
         <v>878</v>
       </c>
       <c r="C484">
-        <v>0.56780865599745611</v>
+        <v>-17.368182173860266</v>
       </c>
       <c r="D484">
-        <v>-50.346041183802321</v>
+        <v>-41.776285527714045</v>
       </c>
     </row>
     <row r="485" spans="2:4">
@@ -14841,10 +14841,10 @@
         <v>879</v>
       </c>
       <c r="C485">
-        <v>-1.8224438009213897</v>
+        <v>-14.960456290979568</v>
       </c>
       <c r="D485">
-        <v>-46.302133663503504</v>
+        <v>-41.357382122619882</v>
       </c>
     </row>
     <row r="486" spans="2:4">
@@ -14852,10 +14852,10 @@
         <v>880</v>
       </c>
       <c r="C486">
-        <v>-2.692908965809846</v>
+        <v>-12.981951490785582</v>
       </c>
       <c r="D486">
-        <v>-43.461814021584082</v>
+        <v>-39.039780443548558</v>
       </c>
     </row>
     <row r="487" spans="2:4">
@@ -14863,10 +14863,10 @@
         <v>881</v>
       </c>
       <c r="C487">
-        <v>-10.306473408705084</v>
+        <v>-11.641402073608694</v>
       </c>
       <c r="D487">
-        <v>-36.524500974203519</v>
+        <v>-39.489667828309457</v>
       </c>
     </row>
     <row r="488" spans="2:4">
@@ -14874,10 +14874,10 @@
         <v>882</v>
       </c>
       <c r="C488">
-        <v>-6.4242328850686317</v>
+        <v>0.56780865599745611</v>
       </c>
       <c r="D488">
-        <v>-36.358844766636523</v>
+        <v>-50.346041183802321</v>
       </c>
     </row>
     <row r="489" spans="2:4">
@@ -14885,10 +14885,10 @@
         <v>883</v>
       </c>
       <c r="C489">
-        <v>-5.9998142531104177</v>
+        <v>-1.8224438009213897</v>
       </c>
       <c r="D489">
-        <v>-38.133424249380312</v>
+        <v>-46.302133663503504</v>
       </c>
     </row>
     <row r="490" spans="2:4">
@@ -14896,10 +14896,10 @@
         <v>884</v>
       </c>
       <c r="C490">
-        <v>-4.6375432587986198</v>
+        <v>-2.692908965809846</v>
       </c>
       <c r="D490">
-        <v>-40.426446322118963</v>
+        <v>-43.461814021584082</v>
       </c>
     </row>
     <row r="491" spans="2:4">
@@ -14907,10 +14907,10 @@
         <v>885</v>
       </c>
       <c r="C491">
-        <v>3.4859879388010531</v>
+        <v>-9.7708487803103203</v>
       </c>
       <c r="D491">
-        <v>-60.164562445002161</v>
+        <v>-36.614719032644885</v>
       </c>
     </row>
     <row r="492" spans="2:4">
@@ -14918,10 +14918,10 @@
         <v>886</v>
       </c>
       <c r="C492">
-        <v>-16.938961091173553</v>
+        <v>-4.6375432587986198</v>
       </c>
       <c r="D492">
-        <v>-39.460454361766544</v>
+        <v>-40.426446322118963</v>
       </c>
     </row>
     <row r="493" spans="2:4">
@@ -14929,10 +14929,10 @@
         <v>887</v>
       </c>
       <c r="C493">
-        <v>-17.959343811553321</v>
+        <v>-5.781767828716001</v>
       </c>
       <c r="D493">
-        <v>-40.491165386460189</v>
+        <v>-36.456336218936713</v>
       </c>
     </row>
     <row r="494" spans="2:4">
@@ -14940,10 +14940,10 @@
         <v>888</v>
       </c>
       <c r="C494">
-        <v>-19.925989442115782</v>
+        <v>-5.9998142531104177</v>
       </c>
       <c r="D494">
-        <v>-40.083674981348743</v>
+        <v>-38.133424249380312</v>
       </c>
     </row>
     <row r="495" spans="2:4">
@@ -14951,10 +14951,10 @@
         <v>889</v>
       </c>
       <c r="C495">
-        <v>-21.946540389185209</v>
+        <v>3.4859879388010531</v>
       </c>
       <c r="D495">
-        <v>-41.379690587979908</v>
+        <v>-60.164562445002161</v>
       </c>
     </row>
     <row r="496" spans="2:4">
@@ -14962,10 +14962,10 @@
         <v>890</v>
       </c>
       <c r="C496">
-        <v>-28.405295728661457</v>
+        <v>-16.938961091173553</v>
       </c>
       <c r="D496">
-        <v>-48.964568810395107</v>
+        <v>-39.460454361766544</v>
       </c>
     </row>
     <row r="497" spans="2:4">
@@ -14973,10 +14973,10 @@
         <v>891</v>
       </c>
       <c r="C497">
-        <v>-23.346618682710911</v>
+        <v>-17.959343811553321</v>
       </c>
       <c r="D497">
-        <v>-44.465694962786102</v>
+        <v>-40.491165386460189</v>
       </c>
     </row>
     <row r="498" spans="2:4">
@@ -14984,10 +14984,10 @@
         <v>892</v>
       </c>
       <c r="C498">
-        <v>-10.07503066804068</v>
+        <v>-19.925989442115782</v>
       </c>
       <c r="D498">
-        <v>-46.302133663503497</v>
+        <v>-40.083674981348743</v>
       </c>
     </row>
     <row r="499" spans="2:4">
@@ -14995,10 +14995,10 @@
         <v>893</v>
       </c>
       <c r="C499">
-        <v>-12.161321658886941</v>
+        <v>-21.946540389185209</v>
       </c>
       <c r="D499">
-        <v>-48.351086012993882</v>
+        <v>-41.379690587979908</v>
       </c>
     </row>
     <row r="500" spans="2:4">
@@ -15006,10 +15006,10 @@
         <v>894</v>
       </c>
       <c r="C500">
-        <v>-12.570833610225796</v>
+        <v>-28.405295728661457</v>
       </c>
       <c r="D500">
-        <v>-46.393783754618518</v>
+        <v>-48.964568810395107</v>
       </c>
     </row>
     <row r="501" spans="2:4">
@@ -15017,10 +15017,10 @@
         <v>895</v>
       </c>
       <c r="C501">
-        <v>-6.7466636356287859</v>
+        <v>-23.346618682710911</v>
       </c>
       <c r="D501">
-        <v>-44.602024473319695</v>
+        <v>-44.465694962786102</v>
       </c>
     </row>
     <row r="502" spans="2:4">
@@ -15028,10 +15028,10 @@
         <v>896</v>
       </c>
       <c r="C502">
-        <v>-7.1390141864693932</v>
+        <v>-10.07503066804068</v>
       </c>
       <c r="D502">
-        <v>-43.51138838905085</v>
+        <v>-46.302133663503497</v>
       </c>
     </row>
     <row r="503" spans="2:4">
@@ -15039,10 +15039,10 @@
         <v>897</v>
       </c>
       <c r="C503">
-        <v>-9.9467452632152664</v>
+        <v>-12.161321658886941</v>
       </c>
       <c r="D503">
-        <v>-44.738353983853301</v>
+        <v>-48.351086012993882</v>
       </c>
     </row>
     <row r="504" spans="2:4">
@@ -15050,10 +15050,10 @@
         <v>898</v>
       </c>
       <c r="C504">
-        <v>-8.3856424144456074</v>
+        <v>-12.570833610225796</v>
       </c>
       <c r="D504">
-        <v>-42.076964843436379</v>
+        <v>-46.393783754618518</v>
       </c>
     </row>
     <row r="505" spans="2:4">
@@ -15061,10 +15061,10 @@
         <v>899</v>
       </c>
       <c r="C505">
-        <v>-16.211569620513998</v>
+        <v>-6.7466636356287859</v>
       </c>
       <c r="D505">
-        <v>-45.083187451673609</v>
+        <v>-44.602024473319695</v>
       </c>
     </row>
     <row r="506" spans="2:4">
@@ -15072,10 +15072,10 @@
         <v>900</v>
       </c>
       <c r="C506">
-        <v>-13.664261940654852</v>
+        <v>-7.1390141864693932</v>
       </c>
       <c r="D506">
-        <v>-45.147342515454127</v>
+        <v>-43.51138838905085</v>
       </c>
     </row>
     <row r="507" spans="2:4">
@@ -15083,10 +15083,10 @@
         <v>901</v>
       </c>
       <c r="C507">
-        <v>-16.435769935280067</v>
+        <v>-9.9467452632152664</v>
       </c>
       <c r="D507">
-        <v>-43.485420863234928</v>
+        <v>-44.738353983853301</v>
       </c>
     </row>
     <row r="508" spans="2:4">
@@ -15094,10 +15094,10 @@
         <v>902</v>
       </c>
       <c r="C508">
-        <v>-12.779604408947565</v>
+        <v>-8.3856424144456074</v>
       </c>
       <c r="D508">
-        <v>-43.511388389050857</v>
+        <v>-42.076964843436379</v>
       </c>
     </row>
     <row r="509" spans="2:4">
@@ -15105,10 +15105,10 @@
         <v>903</v>
       </c>
       <c r="C509">
-        <v>-19.647628377153421</v>
+        <v>-16.211569620513998</v>
       </c>
       <c r="D509">
-        <v>-47.302647158175901</v>
+        <v>-45.083187451673609</v>
       </c>
     </row>
     <row r="510" spans="2:4">
@@ -15116,10 +15116,10 @@
         <v>904</v>
       </c>
       <c r="C510">
-        <v>-17.286425777158033</v>
+        <v>-13.664261940654852</v>
       </c>
       <c r="D510">
-        <v>-49.212440647728947</v>
+        <v>-45.147342515454127</v>
       </c>
     </row>
     <row r="511" spans="2:4">
@@ -15127,10 +15127,10 @@
         <v>905</v>
       </c>
       <c r="C511">
-        <v>-16.99812690457648</v>
+        <v>-16.244920375690491</v>
       </c>
       <c r="D511">
-        <v>-47.902633675712288</v>
+        <v>-43.440259948772457</v>
       </c>
     </row>
     <row r="512" spans="2:4">
@@ -15138,10 +15138,10 @@
         <v>906</v>
       </c>
       <c r="C512">
-        <v>-16.921666468794236</v>
+        <v>-12.779604408947565</v>
       </c>
       <c r="D512">
-        <v>-50.306890144879851</v>
+        <v>-43.511388389050857</v>
       </c>
     </row>
     <row r="513" spans="2:4">
@@ -15149,10 +15149,10 @@
         <v>907</v>
       </c>
       <c r="C513">
-        <v>-20.96092160671942</v>
+        <v>-19.647628377153421</v>
       </c>
       <c r="D513">
-        <v>-47.995114513267239</v>
+        <v>-47.302647158175901</v>
       </c>
     </row>
     <row r="514" spans="2:4">
@@ -15160,10 +15160,10 @@
         <v>908</v>
       </c>
       <c r="C514">
-        <v>-19.243469523217691</v>
+        <v>-17.286425777158033</v>
       </c>
       <c r="D514">
-        <v>-49.57805160779634</v>
+        <v>-49.212440647728947</v>
       </c>
     </row>
     <row r="515" spans="2:4">
@@ -15171,10 +15171,10 @@
         <v>909</v>
       </c>
       <c r="C515">
-        <v>-20.2552049324078</v>
+        <v>-16.99812690457648</v>
       </c>
       <c r="D515">
-        <v>-50.430111048631375</v>
+        <v>-47.902633675712288</v>
       </c>
     </row>
     <row r="516" spans="2:4">
@@ -15182,10 +15182,10 @@
         <v>910</v>
       </c>
       <c r="C516">
-        <v>-33.049576460325305</v>
+        <v>-29.884660564910089</v>
       </c>
       <c r="D516">
-        <v>-51.036372670639899</v>
+        <v>-48.041622626778846</v>
       </c>
     </row>
     <row r="517" spans="2:4">
@@ -15193,10 +15193,10 @@
         <v>911</v>
       </c>
       <c r="C517">
-        <v>-33.257111928877123</v>
+        <v>-29.986856060787883</v>
       </c>
       <c r="D517">
-        <v>-52.989782771191962</v>
+        <v>-49.136498542094962</v>
       </c>
     </row>
     <row r="518" spans="2:4">
@@ -15204,10 +15204,10 @@
         <v>912</v>
       </c>
       <c r="C518">
-        <v>-34.201398310787894</v>
+        <v>-31.554826954684241</v>
       </c>
       <c r="D518">
-        <v>-52.01882304474109</v>
+        <v>-50.322310995228015</v>
       </c>
     </row>
     <row r="519" spans="2:4">
@@ -15215,10 +15215,10 @@
         <v>913</v>
       </c>
       <c r="C519">
-        <v>-31.45847120142804</v>
+        <v>-32.987315819759758</v>
       </c>
       <c r="D519">
-        <v>-50.303843882932888</v>
+        <v>-50.954501806131468</v>
       </c>
     </row>
     <row r="520" spans="2:4">
@@ -15226,10 +15226,10 @@
         <v>914</v>
       </c>
       <c r="C520">
-        <v>-29.986856060787883</v>
+        <v>-33.916613528941788</v>
       </c>
       <c r="D520">
-        <v>-49.136498542094962</v>
+        <v>-52.168201464195072</v>
       </c>
     </row>
     <row r="521" spans="2:4">
@@ -15237,10 +15237,10 @@
         <v>915</v>
       </c>
       <c r="C521">
-        <v>-23.764285867340291</v>
+        <v>-26.152481055453244</v>
       </c>
       <c r="D521">
-        <v>-42.595534417519154</v>
+        <v>-47.537470461121664</v>
       </c>
     </row>
     <row r="522" spans="2:4">
@@ -15248,10 +15248,10 @@
         <v>916</v>
       </c>
       <c r="C522">
-        <v>-25.208194673542479</v>
+        <v>-27.051801419177785</v>
       </c>
       <c r="D522">
-        <v>-44.736625096359532</v>
+        <v>-48.097639534074077</v>
       </c>
     </row>
     <row r="523" spans="2:4">
@@ -15259,10 +15259,10 @@
         <v>917</v>
       </c>
       <c r="C523">
-        <v>-23.51447465519459</v>
+        <v>-27.26164283738018</v>
       </c>
       <c r="D523">
-        <v>-43.653631555318178</v>
+        <v>-46.734561456556527</v>
       </c>
     </row>
     <row r="524" spans="2:4">
@@ -15270,10 +15270,10 @@
         <v>918</v>
       </c>
       <c r="C524">
-        <v>-24.376323337097279</v>
+        <v>-28.351728126743261</v>
       </c>
       <c r="D524">
-        <v>-45.170756127897661</v>
+        <v>-47.557840245592665</v>
       </c>
     </row>
     <row r="525" spans="2:4">
@@ -15281,10 +15281,10 @@
         <v>919</v>
       </c>
       <c r="C525">
-        <v>-29.884660564910089</v>
+        <v>-24.263908291631708</v>
       </c>
       <c r="D525">
-        <v>-48.041622626778846</v>
+        <v>-45.120741032098337</v>
       </c>
     </row>
     <row r="526" spans="2:4">
@@ -15292,10 +15292,10 @@
         <v>920</v>
       </c>
       <c r="C526">
-        <v>-28.351728126743261</v>
+        <v>-23.51447465519459</v>
       </c>
       <c r="D526">
-        <v>-47.557840245592665</v>
+        <v>-43.653631555318178</v>
       </c>
     </row>
     <row r="527" spans="2:4">
@@ -15303,10 +15303,10 @@
         <v>921</v>
       </c>
       <c r="C527">
-        <v>-25.291702993031183</v>
+        <v>-24.78851183713769</v>
       </c>
       <c r="D527">
-        <v>-46.64119994439779</v>
+        <v>-44.400523652588085</v>
       </c>
     </row>
     <row r="528" spans="2:4">
@@ -15314,10 +15314,10 @@
         <v>922</v>
       </c>
       <c r="C528">
-        <v>-26.87193734643288</v>
+        <v>-25.163228655356249</v>
       </c>
       <c r="D528">
-        <v>-46.585183037102553</v>
+        <v>-46.921284480874007</v>
       </c>
     </row>
     <row r="529" spans="2:4">
@@ -15325,10 +15325,10 @@
         <v>923</v>
       </c>
       <c r="C529">
-        <v>-26.152481055453244</v>
+        <v>-25.837718928149656</v>
       </c>
       <c r="D529">
-        <v>-47.537470461121664</v>
+        <v>-45.894307847127891</v>
       </c>
     </row>
     <row r="530" spans="2:4">
@@ -15336,10 +15336,10 @@
         <v>924</v>
       </c>
       <c r="C530">
-        <v>-27.051801419177785</v>
+        <v>4.7391734384846727</v>
       </c>
       <c r="D530">
-        <v>-48.097639534074077</v>
+        <v>-50.469021942906032</v>
       </c>
     </row>
     <row r="531" spans="2:4">
@@ -15347,10 +15347,10 @@
         <v>925</v>
       </c>
       <c r="C531">
-        <v>4.7391734384846727</v>
+        <v>3.0368884642917968</v>
       </c>
       <c r="D531">
-        <v>-50.469021942906032</v>
+        <v>-49.28199700260209</v>
       </c>
     </row>
     <row r="532" spans="2:4">
@@ -15358,10 +15358,10 @@
         <v>926</v>
       </c>
       <c r="C532">
-        <v>3.0368884642917968</v>
+        <v>-15.945194927179701</v>
       </c>
       <c r="D532">
-        <v>-49.28199700260209</v>
+        <v>-37.958579313635177</v>
       </c>
     </row>
     <row r="533" spans="2:4">
@@ -15369,10 +15369,10 @@
         <v>927</v>
       </c>
       <c r="C533">
-        <v>-13.022403745074952</v>
+        <v>-17.331647154588367</v>
       </c>
       <c r="D533">
-        <v>-37.958579313635177</v>
+        <v>-38.051940825793913</v>
       </c>
     </row>
     <row r="534" spans="2:4">
@@ -15380,10 +15380,10 @@
         <v>928</v>
       </c>
       <c r="C534">
-        <v>-10.92398956305103</v>
+        <v>-19.767306473009</v>
       </c>
       <c r="D534">
-        <v>-36.371433606936641</v>
+        <v>-39.639086532492456</v>
       </c>
     </row>
     <row r="535" spans="2:4">
@@ -15391,10 +15391,10 @@
         <v>929</v>
       </c>
       <c r="C535">
-        <v>-15.945194927179701</v>
+        <v>-19.285527706728001</v>
       </c>
       <c r="D535">
-        <v>-37.958579313635177</v>
+        <v>-38.238663850111386</v>
       </c>
     </row>
     <row r="536" spans="2:4">
@@ -15402,10 +15402,10 @@
         <v>930</v>
       </c>
       <c r="C536">
-        <v>-17.331647154588367</v>
+        <v>-23.764285867340291</v>
       </c>
       <c r="D536">
-        <v>-38.051940825793913</v>
+        <v>-42.595534417519154</v>
       </c>
     </row>
     <row r="537" spans="2:4">
@@ -15413,10 +15413,10 @@
         <v>931</v>
       </c>
       <c r="C537">
-        <v>-19.767306473009</v>
+        <v>-21.790777291389219</v>
       </c>
       <c r="D537">
-        <v>-39.639086532492456</v>
+        <v>-40.19925560544489</v>
       </c>
     </row>
     <row r="538" spans="2:4">
@@ -15424,10 +15424,10 @@
         <v>932</v>
       </c>
       <c r="C538">
-        <v>-19.285527706728001</v>
+        <v>-23.014852230903177</v>
       </c>
       <c r="D538">
-        <v>-38.238663850111386</v>
+        <v>-41.288473247296828</v>
       </c>
     </row>
     <row r="539" spans="2:4">
@@ -15435,10 +15435,10 @@
         <v>933</v>
       </c>
       <c r="C539">
-        <v>-21.790777291389219</v>
+        <v>0.79715251082544769</v>
       </c>
       <c r="D539">
-        <v>-40.19925560544489</v>
+        <v>-46.678544549261268</v>
       </c>
     </row>
     <row r="540" spans="2:4">
@@ -15446,10 +15446,10 @@
         <v>934</v>
       </c>
       <c r="C540">
-        <v>-23.014852230903177</v>
+        <v>-0.78691353334900216</v>
       </c>
       <c r="D540">
-        <v>-41.288473247296828</v>
+        <v>-44.223628155866265</v>
       </c>
     </row>
     <row r="541" spans="2:4">
@@ -15457,10 +15457,10 @@
         <v>935</v>
       </c>
       <c r="C541">
-        <v>0.79715251082544769</v>
+        <v>-13.022403745074952</v>
       </c>
       <c r="D541">
-        <v>-46.678544549261268</v>
+        <v>-37.958579313635177</v>
       </c>
     </row>
     <row r="542" spans="2:4">
@@ -15468,10 +15468,10 @@
         <v>936</v>
       </c>
       <c r="C542">
-        <v>-0.78691353334900216</v>
+        <v>-10.610590042359147</v>
       </c>
       <c r="D542">
-        <v>-44.223628155866265</v>
+        <v>-36.099836480656677</v>
       </c>
     </row>
     <row r="543" spans="2:4">
@@ -15479,10 +15479,10 @@
         <v>937</v>
       </c>
       <c r="C543">
-        <v>-7.5856033643766096</v>
+        <v>-7.2267836232945966</v>
       </c>
       <c r="D543">
-        <v>-34.521178184154373</v>
+        <v>-34.441962355656052</v>
       </c>
     </row>
     <row r="544" spans="2:4">
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428515DF-F61B-452E-BB23-A760B3D0F52C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDBA3FDC-4E2B-407A-AC35-F17A515F8387}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22033,7 +22033,7 @@
         <v>941</v>
       </c>
       <c r="H334" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
     </row>
     <row r="335" spans="2:8">
@@ -22113,7 +22113,7 @@
         <v>941</v>
       </c>
       <c r="H338" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
     </row>
     <row r="339" spans="2:8">
@@ -22133,7 +22133,7 @@
         <v>941</v>
       </c>
       <c r="H339" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
     </row>
     <row r="340" spans="2:8">
@@ -22153,7 +22153,7 @@
         <v>941</v>
       </c>
       <c r="H340" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
     </row>
     <row r="341" spans="2:8">
@@ -22173,7 +22173,7 @@
         <v>941</v>
       </c>
       <c r="H341" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
     </row>
     <row r="342" spans="2:8">
@@ -22193,7 +22193,7 @@
         <v>941</v>
       </c>
       <c r="H342" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
     </row>
     <row r="343" spans="2:8">
@@ -22213,7 +22213,7 @@
         <v>941</v>
       </c>
       <c r="H343" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
     </row>
     <row r="344" spans="2:8">
@@ -22233,7 +22233,7 @@
         <v>941</v>
       </c>
       <c r="H344" t="s">
-        <v>945</v>
+        <v>953</v>
       </c>
     </row>
     <row r="345" spans="2:8">
@@ -22253,7 +22253,7 @@
         <v>941</v>
       </c>
       <c r="H345" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="346" spans="2:8">
@@ -22273,7 +22273,7 @@
         <v>941</v>
       </c>
       <c r="H346" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
     </row>
     <row r="347" spans="2:8">
@@ -22293,7 +22293,7 @@
         <v>941</v>
       </c>
       <c r="H347" t="s">
-        <v>969</v>
+        <v>942</v>
       </c>
     </row>
     <row r="348" spans="2:8">
@@ -22313,7 +22313,7 @@
         <v>941</v>
       </c>
       <c r="H348" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="349" spans="2:8">
@@ -22333,7 +22333,7 @@
         <v>941</v>
       </c>
       <c r="H349" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="350" spans="2:8">
@@ -22353,7 +22353,7 @@
         <v>941</v>
       </c>
       <c r="H350" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="351" spans="2:8">
@@ -22373,7 +22373,7 @@
         <v>941</v>
       </c>
       <c r="H351" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="352" spans="2:8">
@@ -22393,7 +22393,7 @@
         <v>941</v>
       </c>
       <c r="H352" t="s">
-        <v>951</v>
+        <v>942</v>
       </c>
     </row>
     <row r="353" spans="2:8">
@@ -22413,7 +22413,7 @@
         <v>941</v>
       </c>
       <c r="H353" t="s">
-        <v>951</v>
+        <v>942</v>
       </c>
     </row>
     <row r="354" spans="2:8">
@@ -22433,7 +22433,7 @@
         <v>941</v>
       </c>
       <c r="H354" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
     </row>
     <row r="355" spans="2:8">
@@ -22453,7 +22453,7 @@
         <v>941</v>
       </c>
       <c r="H355" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
     <row r="356" spans="2:8">
@@ -22473,7 +22473,7 @@
         <v>941</v>
       </c>
       <c r="H356" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="357" spans="2:8">
@@ -22493,7 +22493,7 @@
         <v>941</v>
       </c>
       <c r="H357" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="358" spans="2:8">
@@ -22513,7 +22513,7 @@
         <v>941</v>
       </c>
       <c r="H358" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="359" spans="2:8">
@@ -22533,7 +22533,7 @@
         <v>941</v>
       </c>
       <c r="H359" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
     </row>
     <row r="360" spans="2:8">
@@ -22553,7 +22553,7 @@
         <v>941</v>
       </c>
       <c r="H360" t="s">
-        <v>950</v>
+        <v>968</v>
       </c>
     </row>
     <row r="361" spans="2:8">
@@ -22573,7 +22573,7 @@
         <v>941</v>
       </c>
       <c r="H361" t="s">
-        <v>947</v>
+        <v>968</v>
       </c>
     </row>
     <row r="362" spans="2:8">
@@ -22593,7 +22593,7 @@
         <v>941</v>
       </c>
       <c r="H362" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
     </row>
     <row r="363" spans="2:8">
@@ -22613,7 +22613,7 @@
         <v>941</v>
       </c>
       <c r="H363" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
     </row>
     <row r="364" spans="2:8">
@@ -22633,7 +22633,7 @@
         <v>941</v>
       </c>
       <c r="H364" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
     </row>
     <row r="365" spans="2:8">
@@ -22653,7 +22653,7 @@
         <v>941</v>
       </c>
       <c r="H365" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="366" spans="2:8">
@@ -22673,7 +22673,7 @@
         <v>941</v>
       </c>
       <c r="H366" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
     <row r="367" spans="2:8">
@@ -22693,7 +22693,7 @@
         <v>941</v>
       </c>
       <c r="H367" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
     <row r="368" spans="2:8">
@@ -22713,7 +22713,7 @@
         <v>941</v>
       </c>
       <c r="H368" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="369" spans="2:8">
@@ -22733,7 +22733,7 @@
         <v>941</v>
       </c>
       <c r="H369" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
     </row>
     <row r="370" spans="2:8">
@@ -22753,7 +22753,7 @@
         <v>941</v>
       </c>
       <c r="H370" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="371" spans="2:8">
@@ -22773,7 +22773,7 @@
         <v>941</v>
       </c>
       <c r="H371" t="s">
-        <v>956</v>
+        <v>947</v>
       </c>
     </row>
     <row r="372" spans="2:8">
@@ -22793,7 +22793,7 @@
         <v>941</v>
       </c>
       <c r="H372" t="s">
-        <v>956</v>
+        <v>949</v>
       </c>
     </row>
     <row r="373" spans="2:8">
@@ -22813,7 +22813,7 @@
         <v>941</v>
       </c>
       <c r="H373" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
     </row>
     <row r="374" spans="2:8">
@@ -22833,7 +22833,7 @@
         <v>941</v>
       </c>
       <c r="H374" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
     </row>
     <row r="375" spans="2:8">
@@ -22853,7 +22853,7 @@
         <v>941</v>
       </c>
       <c r="H375" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
     </row>
     <row r="376" spans="2:8">
@@ -22873,7 +22873,7 @@
         <v>941</v>
       </c>
       <c r="H376" t="s">
-        <v>944</v>
+        <v>952</v>
       </c>
     </row>
     <row r="377" spans="2:8">
@@ -22893,7 +22893,7 @@
         <v>941</v>
       </c>
       <c r="H377" t="s">
-        <v>944</v>
+        <v>952</v>
       </c>
     </row>
     <row r="378" spans="2:8">
@@ -22913,7 +22913,7 @@
         <v>941</v>
       </c>
       <c r="H378" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="379" spans="2:8">
@@ -22933,7 +22933,7 @@
         <v>941</v>
       </c>
       <c r="H379" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
     </row>
     <row r="380" spans="2:8">
@@ -22953,7 +22953,7 @@
         <v>941</v>
       </c>
       <c r="H380" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
     </row>
     <row r="381" spans="2:8">
@@ -22973,7 +22973,7 @@
         <v>941</v>
       </c>
       <c r="H381" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="382" spans="2:8">
@@ -22993,7 +22993,7 @@
         <v>941</v>
       </c>
       <c r="H382" t="s">
-        <v>968</v>
+        <v>952</v>
       </c>
     </row>
     <row r="383" spans="2:8">
@@ -23013,7 +23013,7 @@
         <v>941</v>
       </c>
       <c r="H383" t="s">
-        <v>952</v>
+        <v>969</v>
       </c>
     </row>
     <row r="384" spans="2:8">
@@ -23033,7 +23033,7 @@
         <v>941</v>
       </c>
       <c r="H384" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
     </row>
     <row r="385" spans="2:8">
@@ -23053,7 +23053,7 @@
         <v>941</v>
       </c>
       <c r="H385" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
     </row>
     <row r="386" spans="2:8">
@@ -23073,7 +23073,7 @@
         <v>941</v>
       </c>
       <c r="H386" t="s">
-        <v>952</v>
+        <v>970</v>
       </c>
     </row>
     <row r="387" spans="2:8">
@@ -23093,7 +23093,7 @@
         <v>941</v>
       </c>
       <c r="H387" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
     </row>
     <row r="388" spans="2:8">
@@ -23113,7 +23113,7 @@
         <v>941</v>
       </c>
       <c r="H388" t="s">
-        <v>968</v>
+        <v>949</v>
       </c>
     </row>
     <row r="389" spans="2:8">
@@ -23133,7 +23133,7 @@
         <v>941</v>
       </c>
       <c r="H389" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
     </row>
     <row r="390" spans="2:8">
@@ -23173,7 +23173,7 @@
         <v>941</v>
       </c>
       <c r="H391" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
     </row>
     <row r="392" spans="2:8">
@@ -23213,7 +23213,7 @@
         <v>941</v>
       </c>
       <c r="H393" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="394" spans="2:8">
@@ -23233,7 +23233,7 @@
         <v>941</v>
       </c>
       <c r="H394" t="s">
-        <v>952</v>
+        <v>971</v>
       </c>
     </row>
     <row r="395" spans="2:8">
@@ -23253,7 +23253,7 @@
         <v>941</v>
       </c>
       <c r="H395" t="s">
-        <v>952</v>
+        <v>971</v>
       </c>
     </row>
     <row r="396" spans="2:8">
@@ -23293,7 +23293,7 @@
         <v>941</v>
       </c>
       <c r="H397" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="398" spans="2:8">
@@ -23313,7 +23313,7 @@
         <v>941</v>
       </c>
       <c r="H398" t="s">
-        <v>947</v>
+        <v>956</v>
       </c>
     </row>
     <row r="399" spans="2:8">
@@ -23333,7 +23333,7 @@
         <v>941</v>
       </c>
       <c r="H399" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
     </row>
     <row r="400" spans="2:8">
@@ -23353,7 +23353,7 @@
         <v>941</v>
       </c>
       <c r="H400" t="s">
-        <v>947</v>
+        <v>956</v>
       </c>
     </row>
     <row r="401" spans="2:8">
@@ -23373,7 +23373,7 @@
         <v>941</v>
       </c>
       <c r="H401" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
     </row>
     <row r="402" spans="2:8">
@@ -23393,7 +23393,7 @@
         <v>941</v>
       </c>
       <c r="H402" t="s">
-        <v>947</v>
+        <v>950</v>
       </c>
     </row>
     <row r="403" spans="2:8">
@@ -23413,7 +23413,7 @@
         <v>941</v>
       </c>
       <c r="H403" t="s">
-        <v>947</v>
+        <v>954</v>
       </c>
     </row>
     <row r="404" spans="2:8">
@@ -23433,7 +23433,7 @@
         <v>941</v>
       </c>
       <c r="H404" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
     </row>
     <row r="405" spans="2:8">
@@ -23453,7 +23453,7 @@
         <v>941</v>
       </c>
       <c r="H405" t="s">
-        <v>948</v>
+        <v>957</v>
       </c>
     </row>
     <row r="406" spans="2:8">
@@ -23473,7 +23473,7 @@
         <v>941</v>
       </c>
       <c r="H406" t="s">
-        <v>970</v>
+        <v>957</v>
       </c>
     </row>
     <row r="407" spans="2:8">
@@ -23493,7 +23493,7 @@
         <v>941</v>
       </c>
       <c r="H407" t="s">
-        <v>970</v>
+        <v>960</v>
       </c>
     </row>
     <row r="408" spans="2:8">
@@ -23513,7 +23513,7 @@
         <v>941</v>
       </c>
       <c r="H408" t="s">
-        <v>949</v>
+        <v>957</v>
       </c>
     </row>
     <row r="409" spans="2:8">
@@ -23533,7 +23533,7 @@
         <v>941</v>
       </c>
       <c r="H409" t="s">
-        <v>949</v>
+        <v>960</v>
       </c>
     </row>
     <row r="410" spans="2:8">
@@ -23553,7 +23553,7 @@
         <v>941</v>
       </c>
       <c r="H410" t="s">
-        <v>949</v>
+        <v>961</v>
       </c>
     </row>
     <row r="411" spans="2:8">
@@ -23573,7 +23573,7 @@
         <v>941</v>
       </c>
       <c r="H411" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
     <row r="412" spans="2:8">
@@ -23593,7 +23593,7 @@
         <v>941</v>
       </c>
       <c r="H412" t="s">
-        <v>952</v>
+        <v>961</v>
       </c>
     </row>
     <row r="413" spans="2:8">
@@ -23613,7 +23613,7 @@
         <v>941</v>
       </c>
       <c r="H413" t="s">
-        <v>952</v>
+        <v>961</v>
       </c>
     </row>
     <row r="414" spans="2:8">
@@ -23633,7 +23633,7 @@
         <v>941</v>
       </c>
       <c r="H414" t="s">
-        <v>949</v>
+        <v>958</v>
       </c>
     </row>
     <row r="415" spans="2:8">
@@ -23653,7 +23653,7 @@
         <v>941</v>
       </c>
       <c r="H415" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
     </row>
     <row r="416" spans="2:8">
@@ -23673,7 +23673,7 @@
         <v>941</v>
       </c>
       <c r="H416" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
     </row>
     <row r="417" spans="2:8">
@@ -23693,7 +23693,7 @@
         <v>941</v>
       </c>
       <c r="H417" t="s">
-        <v>949</v>
+        <v>963</v>
       </c>
     </row>
     <row r="418" spans="2:8">
@@ -23713,7 +23713,7 @@
         <v>941</v>
       </c>
       <c r="H418" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
     </row>
     <row r="419" spans="2:8">
@@ -23733,7 +23733,7 @@
         <v>941</v>
       </c>
       <c r="H419" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
     </row>
     <row r="420" spans="2:8">
@@ -23753,7 +23753,7 @@
         <v>941</v>
       </c>
       <c r="H420" t="s">
-        <v>957</v>
+        <v>967</v>
       </c>
     </row>
     <row r="421" spans="2:8">
@@ -23773,7 +23773,7 @@
         <v>941</v>
       </c>
       <c r="H421" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="422" spans="2:8">
@@ -23793,7 +23793,7 @@
         <v>941</v>
       </c>
       <c r="H422" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
     </row>
     <row r="423" spans="2:8">
@@ -23813,7 +23813,7 @@
         <v>941</v>
       </c>
       <c r="H423" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
     </row>
     <row r="424" spans="2:8">
@@ -23833,7 +23833,7 @@
         <v>941</v>
       </c>
       <c r="H424" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
     </row>
     <row r="425" spans="2:8">
@@ -23853,7 +23853,7 @@
         <v>941</v>
       </c>
       <c r="H425" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
     </row>
     <row r="426" spans="2:8">
@@ -23873,7 +23873,7 @@
         <v>941</v>
       </c>
       <c r="H426" t="s">
-        <v>961</v>
+        <v>950</v>
       </c>
     </row>
     <row r="427" spans="2:8">
@@ -23893,7 +23893,7 @@
         <v>941</v>
       </c>
       <c r="H427" t="s">
-        <v>956</v>
+        <v>949</v>
       </c>
     </row>
     <row r="428" spans="2:8">
@@ -23913,7 +23913,7 @@
         <v>941</v>
       </c>
       <c r="H428" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="429" spans="2:8">
@@ -23953,7 +23953,7 @@
         <v>941</v>
       </c>
       <c r="H430" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
     </row>
     <row r="431" spans="2:8">
@@ -23973,7 +23973,7 @@
         <v>941</v>
       </c>
       <c r="H431" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
     </row>
     <row r="432" spans="2:8">
@@ -23993,7 +23993,7 @@
         <v>941</v>
       </c>
       <c r="H432" t="s">
-        <v>957</v>
+        <v>947</v>
       </c>
     </row>
     <row r="433" spans="2:8">
@@ -24013,7 +24013,7 @@
         <v>941</v>
       </c>
       <c r="H433" t="s">
-        <v>956</v>
+        <v>946</v>
       </c>
     </row>
     <row r="434" spans="2:8">
@@ -24033,7 +24033,7 @@
         <v>941</v>
       </c>
       <c r="H434" t="s">
-        <v>956</v>
+        <v>969</v>
       </c>
     </row>
     <row r="435" spans="2:8">
@@ -24053,7 +24053,7 @@
         <v>941</v>
       </c>
       <c r="H435" t="s">
-        <v>963</v>
+        <v>946</v>
       </c>
     </row>
     <row r="436" spans="2:8">
@@ -24073,7 +24073,7 @@
         <v>941</v>
       </c>
       <c r="H436" t="s">
-        <v>956</v>
+        <v>946</v>
       </c>
     </row>
     <row r="437" spans="2:8">
@@ -24093,7 +24093,7 @@
         <v>941</v>
       </c>
       <c r="H437" t="s">
-        <v>958</v>
+        <v>946</v>
       </c>
     </row>
     <row r="438" spans="2:8">
@@ -24113,7 +24113,7 @@
         <v>941</v>
       </c>
       <c r="H438" t="s">
-        <v>960</v>
+        <v>953</v>
       </c>
     </row>
     <row r="439" spans="2:8">
@@ -24133,7 +24133,7 @@
         <v>941</v>
       </c>
       <c r="H439" t="s">
-        <v>960</v>
+        <v>944</v>
       </c>
     </row>
     <row r="440" spans="2:8">
@@ -24153,7 +24153,7 @@
         <v>941</v>
       </c>
       <c r="H440" t="s">
-        <v>952</v>
+        <v>944</v>
       </c>
     </row>
     <row r="441" spans="2:8">
@@ -24173,7 +24173,7 @@
         <v>941</v>
       </c>
       <c r="H441" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
     </row>
     <row r="442" spans="2:8">
@@ -24193,7 +24193,7 @@
         <v>941</v>
       </c>
       <c r="H442" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="443" spans="2:8">
@@ -24213,7 +24213,7 @@
         <v>941</v>
       </c>
       <c r="H443" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="444" spans="2:8">
@@ -24233,7 +24233,7 @@
         <v>941</v>
       </c>
       <c r="H444" t="s">
-        <v>971</v>
+        <v>953</v>
       </c>
     </row>
     <row r="445" spans="2:8">
@@ -24253,7 +24253,7 @@
         <v>941</v>
       </c>
       <c r="H445" t="s">
-        <v>971</v>
+        <v>953</v>
       </c>
     </row>
     <row r="446" spans="2:8">
@@ -24273,7 +24273,7 @@
         <v>941</v>
       </c>
       <c r="H446" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="447" spans="2:8">
@@ -24293,7 +24293,7 @@
         <v>941</v>
       </c>
       <c r="H447" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
     </row>
     <row r="448" spans="2:8">
@@ -24313,7 +24313,7 @@
         <v>941</v>
       </c>
       <c r="H448" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
     </row>
     <row r="449" spans="2:8">
@@ -24333,7 +24333,7 @@
         <v>941</v>
       </c>
       <c r="H449" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="450" spans="2:8">
@@ -24353,7 +24353,7 @@
         <v>941</v>
       </c>
       <c r="H450" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
     </row>
     <row r="451" spans="2:8">
@@ -24373,7 +24373,7 @@
         <v>941</v>
       </c>
       <c r="H451" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
     </row>
     <row r="452" spans="2:8">
@@ -24393,7 +24393,7 @@
         <v>941</v>
       </c>
       <c r="H452" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
     </row>
     <row r="453" spans="2:8">
@@ -24413,7 +24413,7 @@
         <v>941</v>
       </c>
       <c r="H453" t="s">
-        <v>954</v>
+        <v>946</v>
       </c>
     </row>
     <row r="454" spans="2:8">
@@ -24433,7 +24433,7 @@
         <v>941</v>
       </c>
       <c r="H454" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="455" spans="2:8">
@@ -24453,7 +24453,7 @@
         <v>941</v>
       </c>
       <c r="H455" t="s">
-        <v>951</v>
+        <v>943</v>
       </c>
     </row>
     <row r="456" spans="2:8">
@@ -24473,7 +24473,7 @@
         <v>941</v>
       </c>
       <c r="H456" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="457" spans="2:8">
@@ -24493,7 +24493,7 @@
         <v>941</v>
       </c>
       <c r="H457" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="458" spans="2:8">
@@ -24513,7 +24513,7 @@
         <v>941</v>
       </c>
       <c r="H458" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="459" spans="2:8">
@@ -24633,7 +24633,7 @@
         <v>941</v>
       </c>
       <c r="H464" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
     </row>
     <row r="465" spans="2:8">
@@ -24673,7 +24673,7 @@
         <v>941</v>
       </c>
       <c r="H466" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
     </row>
     <row r="467" spans="2:8">
@@ -24693,7 +24693,7 @@
         <v>941</v>
       </c>
       <c r="H467" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
     </row>
     <row r="468" spans="2:8">
@@ -24713,7 +24713,7 @@
         <v>941</v>
       </c>
       <c r="H468" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
     </row>
     <row r="469" spans="2:8">
@@ -24733,7 +24733,7 @@
         <v>941</v>
       </c>
       <c r="H469" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
     </row>
     <row r="470" spans="2:8">
@@ -24793,7 +24793,7 @@
         <v>941</v>
       </c>
       <c r="H472" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="473" spans="2:8">
@@ -24813,7 +24813,7 @@
         <v>941</v>
       </c>
       <c r="H473" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="474" spans="2:8">
@@ -24833,7 +24833,7 @@
         <v>941</v>
       </c>
       <c r="H474" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
     </row>
     <row r="475" spans="2:8">
@@ -24853,7 +24853,7 @@
         <v>941</v>
       </c>
       <c r="H475" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
     </row>
     <row r="476" spans="2:8">
@@ -24873,7 +24873,7 @@
         <v>941</v>
       </c>
       <c r="H476" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="477" spans="2:8">
@@ -24893,7 +24893,7 @@
         <v>941</v>
       </c>
       <c r="H477" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
     </row>
     <row r="478" spans="2:8">
@@ -24913,7 +24913,7 @@
         <v>941</v>
       </c>
       <c r="H478" t="s">
-        <v>960</v>
+        <v>946</v>
       </c>
     </row>
     <row r="479" spans="2:8">
@@ -24933,7 +24933,7 @@
         <v>941</v>
       </c>
       <c r="H479" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
     </row>
     <row r="480" spans="2:8">
@@ -24953,7 +24953,7 @@
         <v>941</v>
       </c>
       <c r="H480" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="481" spans="2:8">
@@ -24993,7 +24993,7 @@
         <v>941</v>
       </c>
       <c r="H482" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
     </row>
     <row r="483" spans="2:8">
@@ -25033,7 +25033,7 @@
         <v>941</v>
       </c>
       <c r="H484" t="s">
-        <v>969</v>
+        <v>953</v>
       </c>
     </row>
     <row r="485" spans="2:8">
@@ -25053,7 +25053,7 @@
         <v>941</v>
       </c>
       <c r="H485" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
     </row>
     <row r="486" spans="2:8">
@@ -25073,7 +25073,7 @@
         <v>941</v>
       </c>
       <c r="H486" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
     </row>
     <row r="487" spans="2:8">
@@ -25093,7 +25093,7 @@
         <v>941</v>
       </c>
       <c r="H487" t="s">
-        <v>962</v>
+        <v>956</v>
       </c>
     </row>
     <row r="488" spans="2:8">
@@ -25113,7 +25113,7 @@
         <v>941</v>
       </c>
       <c r="H488" t="s">
-        <v>958</v>
+        <v>969</v>
       </c>
     </row>
     <row r="489" spans="2:8">
@@ -25133,7 +25133,7 @@
         <v>941</v>
       </c>
       <c r="H489" t="s">
-        <v>965</v>
+        <v>949</v>
       </c>
     </row>
     <row r="490" spans="2:8">
@@ -25153,7 +25153,7 @@
         <v>941</v>
       </c>
       <c r="H490" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
     </row>
     <row r="491" spans="2:8">
@@ -25173,7 +25173,7 @@
         <v>941</v>
       </c>
       <c r="H491" t="s">
-        <v>971</v>
+        <v>962</v>
       </c>
     </row>
     <row r="492" spans="2:8">
@@ -25193,7 +25193,7 @@
         <v>941</v>
       </c>
       <c r="H492" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
     </row>
     <row r="493" spans="2:8">
@@ -25213,7 +25213,7 @@
         <v>941</v>
       </c>
       <c r="H493" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
     </row>
     <row r="494" spans="2:8">
@@ -25233,7 +25233,7 @@
         <v>941</v>
       </c>
       <c r="H494" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
     </row>
     <row r="495" spans="2:8">
@@ -25253,7 +25253,7 @@
         <v>941</v>
       </c>
       <c r="H495" t="s">
-        <v>944</v>
+        <v>971</v>
       </c>
     </row>
     <row r="496" spans="2:8">
@@ -25273,7 +25273,7 @@
         <v>941</v>
       </c>
       <c r="H496" t="s">
-        <v>945</v>
+        <v>956</v>
       </c>
     </row>
     <row r="497" spans="2:8">
@@ -25293,7 +25293,7 @@
         <v>941</v>
       </c>
       <c r="H497" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="498" spans="2:8">
@@ -25313,7 +25313,7 @@
         <v>941</v>
       </c>
       <c r="H498" t="s">
-        <v>961</v>
+        <v>969</v>
       </c>
     </row>
     <row r="499" spans="2:8">
@@ -25333,7 +25333,7 @@
         <v>941</v>
       </c>
       <c r="H499" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
     </row>
     <row r="500" spans="2:8">
@@ -25353,7 +25353,7 @@
         <v>941</v>
       </c>
       <c r="H500" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
     </row>
     <row r="501" spans="2:8">
@@ -25373,7 +25373,7 @@
         <v>941</v>
       </c>
       <c r="H501" t="s">
-        <v>961</v>
+        <v>969</v>
       </c>
     </row>
     <row r="502" spans="2:8">
@@ -25393,7 +25393,7 @@
         <v>941</v>
       </c>
       <c r="H502" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
     </row>
     <row r="503" spans="2:8">
@@ -25413,7 +25413,7 @@
         <v>941</v>
       </c>
       <c r="H503" t="s">
-        <v>957</v>
+        <v>950</v>
       </c>
     </row>
     <row r="504" spans="2:8">
@@ -25433,7 +25433,7 @@
         <v>941</v>
       </c>
       <c r="H504" t="s">
-        <v>957</v>
+        <v>950</v>
       </c>
     </row>
     <row r="505" spans="2:8">
@@ -25453,7 +25453,7 @@
         <v>941</v>
       </c>
       <c r="H505" t="s">
-        <v>953</v>
+        <v>961</v>
       </c>
     </row>
     <row r="506" spans="2:8">
@@ -25473,7 +25473,7 @@
         <v>941</v>
       </c>
       <c r="H506" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
     </row>
     <row r="507" spans="2:8">
@@ -25493,7 +25493,7 @@
         <v>941</v>
       </c>
       <c r="H507" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
     </row>
     <row r="508" spans="2:8">
@@ -25513,7 +25513,7 @@
         <v>941</v>
       </c>
       <c r="H508" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
     </row>
     <row r="509" spans="2:8">
@@ -25553,7 +25553,7 @@
         <v>941</v>
       </c>
       <c r="H510" t="s">
-        <v>954</v>
+        <v>956</v>
       </c>
     </row>
     <row r="511" spans="2:8">
@@ -25573,7 +25573,7 @@
         <v>941</v>
       </c>
       <c r="H511" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="512" spans="2:8">
@@ -25593,7 +25593,7 @@
         <v>941</v>
       </c>
       <c r="H512" t="s">
-        <v>954</v>
+        <v>956</v>
       </c>
     </row>
     <row r="513" spans="2:8">
@@ -25613,7 +25613,7 @@
         <v>941</v>
       </c>
       <c r="H513" t="s">
-        <v>946</v>
+        <v>953</v>
       </c>
     </row>
     <row r="514" spans="2:8">
@@ -25633,7 +25633,7 @@
         <v>941</v>
       </c>
       <c r="H514" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
     </row>
     <row r="515" spans="2:8">
@@ -25653,7 +25653,7 @@
         <v>941</v>
       </c>
       <c r="H515" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
     </row>
     <row r="516" spans="2:8">
@@ -25693,7 +25693,7 @@
         <v>941</v>
       </c>
       <c r="H517" t="s">
-        <v>943</v>
+        <v>969</v>
       </c>
     </row>
     <row r="518" spans="2:8">

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 02:55
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1000DCAD-328F-4029-8183-DAF5D97200A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{07240575-053D-4FCF-A488-1F7F1C432133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2885D707-9737-44B0-ADA4-9B3309D6D3F3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{975D951B-D28E-4333-82F4-964C44C14D5F}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDBA3FDC-4E2B-407A-AC35-F17A515F8387}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3EE21C4-9BC9-463B-91F6-8F3AB24D2584}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 03:14
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{07240575-053D-4FCF-A488-1F7F1C432133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D07C8983-1018-4764-AD9D-80B72AD1517C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2996,10 +2996,10 @@
     <t>Unknown</t>
   </si>
   <si>
+    <t>Roraima</t>
+  </si>
+  <si>
     <t>Amapá</t>
-  </si>
-  <si>
-    <t>Roraima</t>
   </si>
   <si>
     <t>~geolocation</t>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{975D951B-D28E-4333-82F4-964C44C14D5F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9B6772F-99C1-4281-95F0-F7139F5DC23A}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -13158,10 +13158,10 @@
         <v>726</v>
       </c>
       <c r="C332">
-        <v>-29.91778906765273</v>
+        <v>-30.38909064864206</v>
       </c>
       <c r="D332">
-        <v>-55.756257153342048</v>
+        <v>-51.498693829725681</v>
       </c>
     </row>
     <row r="333" spans="2:4">
@@ -13169,10 +13169,10 @@
         <v>727</v>
       </c>
       <c r="C333">
-        <v>-31.925049565997167</v>
+        <v>-27.638228359602291</v>
       </c>
       <c r="D333">
-        <v>-52.988639879938802</v>
+        <v>-53.455423275031549</v>
       </c>
     </row>
     <row r="334" spans="2:4">
@@ -13180,10 +13180,10 @@
         <v>728</v>
       </c>
       <c r="C334">
-        <v>-27.026337837617159</v>
+        <v>-28.838896618314362</v>
       </c>
       <c r="D334">
-        <v>-52.999922322189846</v>
+        <v>-50.912133246589491</v>
       </c>
     </row>
     <row r="335" spans="2:4">
@@ -13191,10 +13191,10 @@
         <v>729</v>
       </c>
       <c r="C335">
-        <v>-29.154729365098586</v>
+        <v>-31.97045859914089</v>
       </c>
       <c r="D335">
-        <v>-51.473031804213456</v>
+        <v>-52.97655154895552</v>
       </c>
     </row>
     <row r="336" spans="2:4">
@@ -13202,10 +13202,10 @@
         <v>730</v>
       </c>
       <c r="C336">
-        <v>-28.474474218178731</v>
+        <v>-30.08663379997256</v>
       </c>
       <c r="D336">
-        <v>-50.264942603177197</v>
+        <v>-56.101122318328237</v>
       </c>
     </row>
     <row r="337" spans="2:4">
@@ -13213,10 +13213,10 @@
         <v>731</v>
       </c>
       <c r="C337">
-        <v>-30.38909064864206</v>
+        <v>-29.304616092385999</v>
       </c>
       <c r="D337">
-        <v>-51.498693829725681</v>
+        <v>-54.397552267215872</v>
       </c>
     </row>
     <row r="338" spans="2:4">
@@ -13224,10 +13224,10 @@
         <v>732</v>
       </c>
       <c r="C338">
-        <v>-28.657105430504327</v>
+        <v>-22.452651416389497</v>
       </c>
       <c r="D338">
-        <v>-53.981494798031832</v>
+        <v>-55.248710057848974</v>
       </c>
     </row>
     <row r="339" spans="2:4">
@@ -13235,10 +13235,10 @@
         <v>733</v>
       </c>
       <c r="C339">
-        <v>-18.339825503898322</v>
+        <v>-20.694456313764</v>
       </c>
       <c r="D339">
-        <v>-56.661942712831042</v>
+        <v>-57.447293910263937</v>
       </c>
     </row>
     <row r="340" spans="2:4">
@@ -13246,10 +13246,10 @@
         <v>734</v>
       </c>
       <c r="C340">
-        <v>-15.393254216021999</v>
+        <v>-21.99347461692167</v>
       </c>
       <c r="D340">
-        <v>-59.870929653083621</v>
+        <v>-50.600522936798384</v>
       </c>
     </row>
     <row r="341" spans="2:4">
@@ -13257,10 +13257,10 @@
         <v>735</v>
       </c>
       <c r="C341">
-        <v>-15.80297747383729</v>
+        <v>-20.12208185225121</v>
       </c>
       <c r="D341">
-        <v>-57.273493715548582</v>
+        <v>-55.537086265594233</v>
       </c>
     </row>
     <row r="342" spans="2:4">
@@ -13268,10 +13268,10 @@
         <v>736</v>
       </c>
       <c r="C342">
-        <v>-20.583933777481352</v>
+        <v>-20.846722195452809</v>
       </c>
       <c r="D342">
-        <v>-52.781795105336087</v>
+        <v>-53.197275518390882</v>
       </c>
     </row>
     <row r="343" spans="2:4">
@@ -13279,10 +13279,10 @@
         <v>737</v>
       </c>
       <c r="C343">
-        <v>-22.44729831898637</v>
+        <v>-25.807259122346117</v>
       </c>
       <c r="D343">
-        <v>-51.009511468399197</v>
+        <v>-49.206932384677074</v>
       </c>
     </row>
     <row r="344" spans="2:4">
@@ -13290,10 +13290,10 @@
         <v>738</v>
       </c>
       <c r="C344">
-        <v>-19.830741226253327</v>
+        <v>-27.011349164888419</v>
       </c>
       <c r="D344">
-        <v>-49.754339767969107</v>
+        <v>-51.036777370505931</v>
       </c>
     </row>
     <row r="345" spans="2:4">
@@ -13301,10 +13301,10 @@
         <v>739</v>
       </c>
       <c r="C345">
-        <v>-18.476312794026995</v>
+        <v>-26.775277569410729</v>
       </c>
       <c r="D345">
-        <v>-52.914440034503912</v>
+        <v>-49.987040139397152</v>
       </c>
     </row>
     <row r="346" spans="2:4">
@@ -13312,10 +13312,10 @@
         <v>740</v>
       </c>
       <c r="C346">
-        <v>-24.294116923063548</v>
+        <v>-25.891286530067848</v>
       </c>
       <c r="D346">
-        <v>-50.133107472111739</v>
+        <v>-53.178390045070209</v>
       </c>
     </row>
     <row r="347" spans="2:4">
@@ -13323,10 +13323,10 @@
         <v>741</v>
       </c>
       <c r="C347">
-        <v>-25.807259122346117</v>
+        <v>-24.294116923063548</v>
       </c>
       <c r="D347">
-        <v>-49.206932384677074</v>
+        <v>-50.133107472111739</v>
       </c>
     </row>
     <row r="348" spans="2:4">
@@ -13334,10 +13334,10 @@
         <v>742</v>
       </c>
       <c r="C348">
-        <v>-27.011349164888419</v>
+        <v>-22.925062262215032</v>
       </c>
       <c r="D348">
-        <v>-51.036777370505931</v>
+        <v>-52.543218461902271</v>
       </c>
     </row>
     <row r="349" spans="2:4">
@@ -13345,10 +13345,10 @@
         <v>743</v>
       </c>
       <c r="C349">
-        <v>-26.775277569410729</v>
+        <v>-24.223456037342338</v>
       </c>
       <c r="D349">
-        <v>-49.987040139397152</v>
+        <v>-52.999922322189867</v>
       </c>
     </row>
     <row r="350" spans="2:4">
@@ -13356,10 +13356,10 @@
         <v>744</v>
       </c>
       <c r="C350">
-        <v>-20.883707232056199</v>
+        <v>-24.408316334330163</v>
       </c>
       <c r="D350">
-        <v>-56.760138094544068</v>
+        <v>-47.813341832555771</v>
       </c>
     </row>
     <row r="351" spans="2:4">
@@ -13367,10 +13367,10 @@
         <v>745</v>
       </c>
       <c r="C351">
-        <v>-22.955414324490736</v>
+        <v>-26.606655001212371</v>
       </c>
       <c r="D351">
-        <v>-54.352311066683242</v>
+        <v>-48.419250768260682</v>
       </c>
     </row>
     <row r="352" spans="2:4">
@@ -13378,10 +13378,10 @@
         <v>746</v>
       </c>
       <c r="C352">
-        <v>-24.223456037342338</v>
+        <v>-23.045346360863192</v>
       </c>
       <c r="D352">
-        <v>-52.127413454774775</v>
+        <v>-47.132300188823429</v>
       </c>
     </row>
     <row r="353" spans="2:4">
@@ -13389,10 +13389,10 @@
         <v>747</v>
       </c>
       <c r="C353">
-        <v>-25.236262066013079</v>
+        <v>-20.761072637002851</v>
       </c>
       <c r="D353">
-        <v>-53.353080673286442</v>
+        <v>-47.873932726126263</v>
       </c>
     </row>
     <row r="354" spans="2:4">
@@ -13400,10 +13400,10 @@
         <v>748</v>
       </c>
       <c r="C354">
-        <v>-11.677936963385005</v>
+        <v>-22.110053182589667</v>
       </c>
       <c r="D354">
-        <v>-64.778792032293467</v>
+        <v>-45.69266055758856</v>
       </c>
     </row>
     <row r="355" spans="2:4">
@@ -13411,10 +13411,10 @@
         <v>749</v>
       </c>
       <c r="C355">
-        <v>-9.4786898920949962</v>
+        <v>-21.435562909796261</v>
       </c>
       <c r="D355">
-        <v>-65.224961339494342</v>
+        <v>-41.60277524158036</v>
       </c>
     </row>
     <row r="356" spans="2:4">
@@ -13422,10 +13422,10 @@
         <v>750</v>
       </c>
       <c r="C356">
-        <v>-5.5625584900581444</v>
+        <v>-22.309902152306229</v>
       </c>
       <c r="D356">
-        <v>-67.341786830325262</v>
+        <v>-43.178138474413146</v>
       </c>
     </row>
     <row r="357" spans="2:4">
@@ -13433,10 +13433,10 @@
         <v>751</v>
       </c>
       <c r="C357">
-        <v>-6.665203457755184</v>
+        <v>-20.311412455140584</v>
       </c>
       <c r="D357">
-        <v>-64.897339432757434</v>
+        <v>-45.536855402693007</v>
       </c>
     </row>
     <row r="358" spans="2:4">
@@ -13444,10 +13444,10 @@
         <v>752</v>
       </c>
       <c r="C358">
-        <v>-5.732956032658584</v>
+        <v>-18.724376519156099</v>
       </c>
       <c r="D358">
-        <v>-72.068833227143116</v>
+        <v>-45.083187451673609</v>
       </c>
     </row>
     <row r="359" spans="2:4">
@@ -13455,10 +13455,10 @@
         <v>753</v>
       </c>
       <c r="C359">
-        <v>-4.8880682172647409</v>
+        <v>-16.80406303661487</v>
       </c>
       <c r="D359">
-        <v>-69.904781628357057</v>
+        <v>-44.765619885960028</v>
       </c>
     </row>
     <row r="360" spans="2:4">
@@ -13466,10 +13466,10 @@
         <v>754</v>
       </c>
       <c r="C360">
-        <v>-8.6973323293265334</v>
+        <v>-18.422839691319048</v>
       </c>
       <c r="D360">
-        <v>-71.665379878676774</v>
+        <v>-47.98299633455315</v>
       </c>
     </row>
     <row r="361" spans="2:4">
@@ -13477,10 +13477,10 @@
         <v>755</v>
       </c>
       <c r="C361">
-        <v>-9.9371096878896488</v>
+        <v>-16.553538078148751</v>
       </c>
       <c r="D361">
-        <v>-68.498640105424712</v>
+        <v>-47.289663395267937</v>
       </c>
     </row>
     <row r="362" spans="2:4">
@@ -13488,10 +13488,10 @@
         <v>756</v>
       </c>
       <c r="C362">
-        <v>-8.2830025903248714</v>
+        <v>-11.37271308236334</v>
       </c>
       <c r="D362">
-        <v>-67.369052732431996</v>
+        <v>-47.659110467103602</v>
       </c>
     </row>
     <row r="363" spans="2:4">
@@ -13499,10 +13499,10 @@
         <v>757</v>
       </c>
       <c r="C363">
-        <v>-7.2412898356772812</v>
+        <v>-14.235235125873496</v>
       </c>
       <c r="D363">
-        <v>-69.868427092214745</v>
+        <v>-46.419751280434447</v>
       </c>
     </row>
     <row r="364" spans="2:4">
@@ -13510,10 +13510,10 @@
         <v>758</v>
       </c>
       <c r="C364">
-        <v>-8.9613692439963994</v>
+        <v>-13.744007167415322</v>
       </c>
       <c r="D364">
-        <v>-60.961565737352473</v>
+        <v>-43.511388389050843</v>
       </c>
     </row>
     <row r="365" spans="2:4">
@@ -13521,10 +13521,10 @@
         <v>759</v>
       </c>
       <c r="C365">
-        <v>-7.4960972720659012</v>
+        <v>-9.8481659156531514</v>
       </c>
       <c r="D365">
-        <v>-63.142837905890175</v>
+        <v>-42.231988367120088</v>
       </c>
     </row>
     <row r="366" spans="2:4">
@@ -13532,10 +13532,10 @@
         <v>760</v>
       </c>
       <c r="C366">
-        <v>-9.6994321631910196</v>
+        <v>-10.291626138549251</v>
       </c>
       <c r="D366">
-        <v>-63.070128833605601</v>
+        <v>-44.982718200847508</v>
       </c>
     </row>
     <row r="367" spans="2:4">
@@ -13543,10 +13543,10 @@
         <v>761</v>
       </c>
       <c r="C367">
-        <v>-12.217529181619728</v>
+        <v>-3.7331515396395458</v>
       </c>
       <c r="D367">
-        <v>-62.541107652500472</v>
+        <v>-42.793864649400298</v>
       </c>
     </row>
     <row r="368" spans="2:4">
@@ -13554,10 +13554,10 @@
         <v>762</v>
       </c>
       <c r="C368">
-        <v>-11.361724319365733</v>
+        <v>-5.1697940863090608</v>
       </c>
       <c r="D368">
-        <v>-58.340520954190247</v>
+        <v>-39.805451490463838</v>
       </c>
     </row>
     <row r="369" spans="2:4">
@@ -13565,10 +13565,10 @@
         <v>763</v>
       </c>
       <c r="C369">
-        <v>-11.318208817895188</v>
+        <v>-1.8648877852558583</v>
       </c>
       <c r="D369">
-        <v>-60.620741961018453</v>
+        <v>-46.694523937323893</v>
       </c>
     </row>
     <row r="370" spans="2:4">
@@ -13576,10 +13576,10 @@
         <v>764</v>
       </c>
       <c r="C370">
-        <v>-13.140515870705434</v>
+        <v>-4.4813301436711441</v>
       </c>
       <c r="D370">
-        <v>-59.813527753911572</v>
+        <v>-46.448669661456734</v>
       </c>
     </row>
     <row r="371" spans="2:4">
@@ -13587,10 +13587,10 @@
         <v>765</v>
       </c>
       <c r="C371">
-        <v>-9.4615474218187234</v>
+        <v>-6.3505344277977391</v>
       </c>
       <c r="D371">
-        <v>-56.898066778221747</v>
+        <v>-47.432484787255532</v>
       </c>
     </row>
     <row r="372" spans="2:4">
@@ -13598,10 +13598,10 @@
         <v>766</v>
       </c>
       <c r="C372">
-        <v>-7.3252264029582399</v>
+        <v>-8.2916499015145302</v>
       </c>
       <c r="D372">
-        <v>-56.817148617130833</v>
+        <v>-47.16082451718124</v>
       </c>
     </row>
     <row r="373" spans="2:4">
@@ -13609,10 +13609,10 @@
         <v>767</v>
       </c>
       <c r="C373">
-        <v>-5.9035507946370318</v>
+        <v>-7.2525313402238396</v>
       </c>
       <c r="D373">
-        <v>-53.440721072915188</v>
+        <v>-41.875434262647573</v>
       </c>
     </row>
     <row r="374" spans="2:4">
@@ -13620,10 +13620,10 @@
         <v>768</v>
       </c>
       <c r="C374">
-        <v>-4.1645241064499992</v>
+        <v>-6.4537032141124584</v>
       </c>
       <c r="D374">
-        <v>-55.40923658107468</v>
+        <v>-43.874933750473801</v>
       </c>
     </row>
     <row r="375" spans="2:4">
@@ -13631,10 +13631,10 @@
         <v>769</v>
       </c>
       <c r="C375">
-        <v>-5.7536640673496082</v>
+        <v>-16.114584091092727</v>
       </c>
       <c r="D375">
-        <v>-56.712629325721743</v>
+        <v>-39.754752987680362</v>
       </c>
     </row>
     <row r="376" spans="2:4">
@@ -13642,10 +13642,10 @@
         <v>770</v>
       </c>
       <c r="C376">
-        <v>-4.0178435123665857</v>
+        <v>-15.225600743043184</v>
       </c>
       <c r="D376">
-        <v>-62.982450246438873</v>
+        <v>-41.781413910555422</v>
       </c>
     </row>
     <row r="377" spans="2:4">
@@ -13653,10 +13653,10 @@
         <v>771</v>
       </c>
       <c r="C377">
-        <v>-7.0291424678243146</v>
+        <v>-19.906718291464539</v>
       </c>
       <c r="D377">
-        <v>-60.416247695218047</v>
+        <v>-43.238729367983645</v>
       </c>
     </row>
     <row r="378" spans="2:4">
@@ -13664,10 +13664,10 @@
         <v>772</v>
       </c>
       <c r="C378">
-        <v>-5.6412490218840405</v>
+        <v>-18.380518733026125</v>
       </c>
       <c r="D378">
-        <v>-61.688656460198366</v>
+        <v>-42.805682687465122</v>
       </c>
     </row>
     <row r="379" spans="2:4">
@@ -13675,10 +13675,10 @@
         <v>773</v>
       </c>
       <c r="C379">
-        <v>-1.7935886020853082</v>
+        <v>-17.788319212468952</v>
       </c>
       <c r="D379">
-        <v>-56.797318870144117</v>
+        <v>-41.208934433372157</v>
       </c>
     </row>
     <row r="380" spans="2:4">
@@ -13686,10 +13686,10 @@
         <v>774</v>
       </c>
       <c r="C380">
-        <v>-3.3742122716617691</v>
+        <v>-19.648755345027759</v>
       </c>
       <c r="D380">
-        <v>-57.663689958729989</v>
+        <v>-40.641293430448606</v>
       </c>
     </row>
     <row r="381" spans="2:4">
@@ -13697,10 +13697,10 @@
         <v>775</v>
       </c>
       <c r="C381">
-        <v>-2.6247786352246538</v>
+        <v>-5.6391672617828261</v>
       </c>
       <c r="D381">
-        <v>-60.182539962874714</v>
+        <v>-37.593677783666159</v>
       </c>
     </row>
     <row r="382" spans="2:4">
@@ -13708,10 +13708,10 @@
         <v>776</v>
       </c>
       <c r="C382">
-        <v>-4.4076418124329484</v>
+        <v>-7.925318354752612</v>
       </c>
       <c r="D382">
-        <v>-60.100537249771811</v>
+        <v>-36.204126624449543</v>
       </c>
     </row>
     <row r="383" spans="2:4">
@@ -13719,10 +13719,10 @@
         <v>777</v>
       </c>
       <c r="C383">
-        <v>-1.844333951762555</v>
+        <v>-13.093183219983089</v>
       </c>
       <c r="D383">
-        <v>-49.867164190479677</v>
+        <v>-40.268181085830321</v>
       </c>
     </row>
     <row r="384" spans="2:4">
@@ -13730,10 +13730,10 @@
         <v>778</v>
       </c>
       <c r="C384">
-        <v>-4.2893101856270874</v>
+        <v>-11.344659416828264</v>
       </c>
       <c r="D384">
-        <v>-49.91170014673385</v>
+        <v>-41.330116220513162</v>
       </c>
     </row>
     <row r="385" spans="2:4">
@@ -13741,10 +13741,10 @@
         <v>779</v>
       </c>
       <c r="C385">
-        <v>-6.139363964722846</v>
+        <v>-8.9125268449320494</v>
       </c>
       <c r="D385">
-        <v>-50.544110725543099</v>
+        <v>-39.775959800430037</v>
       </c>
     </row>
     <row r="386" spans="2:4">
@@ -13752,10 +13752,10 @@
         <v>780</v>
       </c>
       <c r="C386">
-        <v>1.7083103899935743</v>
+        <v>-11.146909700995275</v>
       </c>
       <c r="D386">
-        <v>-50.91449393075456</v>
+        <v>-38.551590958209175</v>
       </c>
     </row>
     <row r="387" spans="2:4">
@@ -13763,10 +13763,10 @@
         <v>781</v>
       </c>
       <c r="C387">
-        <v>1.1759205209921435</v>
+        <v>-2.6247786352246538</v>
       </c>
       <c r="D387">
-        <v>-55.15782371749323</v>
+        <v>-60.182539962874714</v>
       </c>
     </row>
     <row r="388" spans="2:4">
@@ -13774,10 +13774,10 @@
         <v>782</v>
       </c>
       <c r="C388">
-        <v>-1.9586154028361076</v>
+        <v>-4.5452023285947609</v>
       </c>
       <c r="D388">
-        <v>-52.175886169631163</v>
+        <v>-60.484412450484839</v>
       </c>
     </row>
     <row r="389" spans="2:4">
@@ -13785,10 +13785,10 @@
         <v>783</v>
       </c>
       <c r="C389">
-        <v>-2.5498352715809425</v>
+        <v>-6.6417429265275896</v>
       </c>
       <c r="D389">
-        <v>-54.230296154755656</v>
+        <v>-60.416247695218033</v>
       </c>
     </row>
     <row r="390" spans="2:4">
@@ -13796,10 +13796,10 @@
         <v>784</v>
       </c>
       <c r="C390">
-        <v>0.78173789403495986</v>
+        <v>-3.7114574080584712</v>
       </c>
       <c r="D390">
-        <v>-68.596018327234432</v>
+        <v>-63.097394735712321</v>
       </c>
     </row>
     <row r="391" spans="2:4">
@@ -13807,10 +13807,10 @@
         <v>785</v>
       </c>
       <c r="C391">
-        <v>-2.4655239874817667</v>
+        <v>-5.4051774264063503</v>
       </c>
       <c r="D391">
-        <v>-68.800512593034838</v>
+        <v>-62.461190353222165</v>
       </c>
     </row>
     <row r="392" spans="2:4">
@@ -13818,10 +13818,10 @@
         <v>786</v>
       </c>
       <c r="C392">
-        <v>0.68425911335153089</v>
+        <v>-7.8065769214469913</v>
       </c>
       <c r="D392">
-        <v>-64.778792032293467</v>
+        <v>-57.97530026852111</v>
       </c>
     </row>
     <row r="393" spans="2:4">
@@ -13829,10 +13829,10 @@
         <v>787</v>
       </c>
       <c r="C393">
-        <v>-2.5948012897671693</v>
+        <v>-6.4000505787766198</v>
       </c>
       <c r="D393">
-        <v>-66.033023529202637</v>
+        <v>-55.917373847609042</v>
       </c>
     </row>
     <row r="394" spans="2:4">
@@ -13840,10 +13840,10 @@
         <v>788</v>
       </c>
       <c r="C394">
-        <v>3.4177977134197421</v>
+        <v>-8.414153476701367</v>
       </c>
       <c r="D394">
-        <v>-60.883663159904685</v>
+        <v>-55.803765922164359</v>
       </c>
     </row>
     <row r="395" spans="2:4">
@@ -13851,10 +13851,10 @@
         <v>789</v>
       </c>
       <c r="C395">
-        <v>1.0871220817168219</v>
+        <v>1.1598612287827772</v>
       </c>
       <c r="D395">
-        <v>-60.640790418449861</v>
+        <v>-56.008260187964773</v>
       </c>
     </row>
     <row r="396" spans="2:4">
@@ -13862,10 +13862,10 @@
         <v>790</v>
       </c>
       <c r="C396">
-        <v>-0.2265909986258858</v>
+        <v>-1.9768811688854704</v>
       </c>
       <c r="D396">
-        <v>-62.688406204111487</v>
+        <v>-56.933248587391709</v>
       </c>
     </row>
     <row r="397" spans="2:4">
@@ -13873,10 +13873,10 @@
         <v>791</v>
       </c>
       <c r="C397">
-        <v>-1.1687361415754016</v>
+        <v>-4.2735326353863066</v>
       </c>
       <c r="D397">
-        <v>-61.078419603524146</v>
+        <v>-54.932771827088544</v>
       </c>
     </row>
     <row r="398" spans="2:4">
@@ -13884,10 +13884,10 @@
         <v>792</v>
       </c>
       <c r="C398">
-        <v>-11.767868999757455</v>
+        <v>-4.2977079139810526</v>
       </c>
       <c r="D398">
-        <v>-41.875434262647573</v>
+        <v>-57.689657484545911</v>
       </c>
     </row>
     <row r="399" spans="2:4">
@@ -13895,10 +13895,10 @@
         <v>793</v>
       </c>
       <c r="C399">
-        <v>-9.4895907449886234</v>
+        <v>-2.9745143322286411</v>
       </c>
       <c r="D399">
-        <v>-42.202625087928233</v>
+        <v>-65.35440552121311</v>
       </c>
     </row>
     <row r="400" spans="2:4">
@@ -13906,10 +13906,10 @@
         <v>794</v>
       </c>
       <c r="C400">
-        <v>-12.901794675757964</v>
+        <v>1.3227765033990899E-2</v>
       </c>
       <c r="D400">
-        <v>-43.463969428865255</v>
+        <v>-65.514971389174903</v>
       </c>
     </row>
     <row r="401" spans="2:4">
@@ -13917,10 +13917,10 @@
         <v>795</v>
       </c>
       <c r="C401">
-        <v>-15.347855832276291</v>
+        <v>0.78173789403495986</v>
       </c>
       <c r="D401">
-        <v>-44.119627743739251</v>
+        <v>-68.596018327234432</v>
       </c>
     </row>
     <row r="402" spans="2:4">
@@ -13928,10 +13928,10 @@
         <v>796</v>
       </c>
       <c r="C402">
-        <v>-9.5876984210313037</v>
+        <v>-2.6247786352246534</v>
       </c>
       <c r="D402">
-        <v>-47.559961732170073</v>
+        <v>-68.440213172338886</v>
       </c>
     </row>
     <row r="403" spans="2:4">
@@ -13939,10 +13939,10 @@
         <v>797</v>
       </c>
       <c r="C403">
-        <v>-12.912458553588689</v>
+        <v>3.4177977134197421</v>
       </c>
       <c r="D403">
-        <v>-46.11404268105607</v>
+        <v>-60.883663159904685</v>
       </c>
     </row>
     <row r="404" spans="2:4">
@@ -13950,10 +13950,10 @@
         <v>798</v>
       </c>
       <c r="C404">
-        <v>-13.116849545344261</v>
+        <v>1.0871220817168219</v>
       </c>
       <c r="D404">
-        <v>-47.951835303574043</v>
+        <v>-60.640790418449861</v>
       </c>
     </row>
     <row r="405" spans="2:4">
@@ -13961,10 +13961,10 @@
         <v>799</v>
       </c>
       <c r="C405">
-        <v>-7.3611992175072203</v>
+        <v>-0.2265909986258858</v>
       </c>
       <c r="D405">
-        <v>-44.356631354359209</v>
+        <v>-62.688406204111487</v>
       </c>
     </row>
     <row r="406" spans="2:4">
@@ -13972,10 +13972,10 @@
         <v>800</v>
       </c>
       <c r="C406">
-        <v>-10.408431240638969</v>
+        <v>-1.1687361415754016</v>
       </c>
       <c r="D406">
-        <v>-44.982478921320464</v>
+        <v>-61.078419603524146</v>
       </c>
     </row>
     <row r="407" spans="2:4">
@@ -13983,10 +13983,10 @@
         <v>801</v>
       </c>
       <c r="C407">
-        <v>-4.303509980843792</v>
+        <v>-10.999699522409411</v>
       </c>
       <c r="D407">
-        <v>-39.460454361766537</v>
+        <v>-54.417749231739357</v>
       </c>
     </row>
     <row r="408" spans="2:4">
@@ -13994,10 +13994,10 @@
         <v>802</v>
       </c>
       <c r="C408">
-        <v>-4.191776238684076</v>
+        <v>-11.205793772429621</v>
       </c>
       <c r="D408">
-        <v>-42.602524985493474</v>
+        <v>-52.372806573735268</v>
       </c>
     </row>
     <row r="409" spans="2:4">
@@ -14005,10 +14005,10 @@
         <v>803</v>
       </c>
       <c r="C409">
-        <v>-6.4930091740654543</v>
+        <v>-11.243265454251476</v>
       </c>
       <c r="D409">
-        <v>-40.721876865824747</v>
+        <v>-49.934023107522975</v>
       </c>
     </row>
     <row r="410" spans="2:4">
@@ -14016,10 +14016,10 @@
         <v>804</v>
       </c>
       <c r="C410">
-        <v>-1.9811473945198379</v>
+        <v>-13.566509727206537</v>
       </c>
       <c r="D410">
-        <v>-46.141746004052202</v>
+        <v>-49.683397138663217</v>
       </c>
     </row>
     <row r="411" spans="2:4">
@@ -14027,10 +14027,10 @@
         <v>805</v>
       </c>
       <c r="C411">
-        <v>-6.5030977037867244</v>
+        <v>-16.264470818380147</v>
       </c>
       <c r="D411">
-        <v>-47.533108949792243</v>
+        <v>-49.393032986357873</v>
       </c>
     </row>
     <row r="412" spans="2:4">
@@ -14038,10 +14038,10 @@
         <v>806</v>
       </c>
       <c r="C412">
-        <v>-4.1063512857195654</v>
+        <v>-14.384073694228841</v>
       </c>
       <c r="D412">
-        <v>-47.265693371437855</v>
+        <v>-51.509386340355761</v>
       </c>
     </row>
     <row r="413" spans="2:4">
@@ -14049,10 +14049,10 @@
         <v>807</v>
       </c>
       <c r="C413">
-        <v>-5.2400436009983089</v>
+        <v>-8.6951910903652845</v>
       </c>
       <c r="D413">
-        <v>-44.451591909972265</v>
+        <v>-51.168562564021748</v>
       </c>
     </row>
     <row r="414" spans="2:4">
@@ -14060,10 +14060,10 @@
         <v>808</v>
       </c>
       <c r="C414">
-        <v>-6.8526180462974819</v>
+        <v>-8.2743552791352126</v>
       </c>
       <c r="D414">
-        <v>-36.41285180609411</v>
+        <v>-49.572808165083501</v>
       </c>
     </row>
     <row r="415" spans="2:4">
@@ -14071,10 +14071,10 @@
         <v>809</v>
       </c>
       <c r="C415">
-        <v>-8.6347528938784208</v>
+        <v>-6.1833796443712101</v>
       </c>
       <c r="D415">
-        <v>-39.518253048260057</v>
+        <v>-52.711431486996162</v>
       </c>
     </row>
     <row r="416" spans="2:4">
@@ -14082,10 +14082,10 @@
         <v>810</v>
       </c>
       <c r="C416">
-        <v>-11.717906757328317</v>
+        <v>-4.9139577428871144</v>
       </c>
       <c r="D416">
-        <v>-38.724707796982003</v>
+        <v>-49.972580948886019</v>
       </c>
     </row>
     <row r="417" spans="2:4">
@@ -14093,10 +14093,10 @@
         <v>811</v>
       </c>
       <c r="C417">
-        <v>-9.9551763916251836</v>
+        <v>-2.7318405832870987</v>
       </c>
       <c r="D417">
-        <v>-37.325436848588453</v>
+        <v>-53.976301292868648</v>
       </c>
     </row>
     <row r="418" spans="2:4">
@@ -14104,10 +14104,10 @@
         <v>812</v>
       </c>
       <c r="C418">
-        <v>-17.538508000323247</v>
+        <v>-2.5337759793715762</v>
       </c>
       <c r="D418">
-        <v>-41.60277524158036</v>
+        <v>-51.90539110904863</v>
       </c>
     </row>
     <row r="419" spans="2:4">
@@ -14115,10 +14115,10 @@
         <v>813</v>
       </c>
       <c r="C419">
-        <v>-18.921553711202652</v>
+        <v>-1.6016388011322449</v>
       </c>
       <c r="D419">
-        <v>-42.519901039715528</v>
+        <v>-49.699562693271943</v>
       </c>
     </row>
     <row r="420" spans="2:4">
@@ -14126,10 +14126,10 @@
         <v>814</v>
       </c>
       <c r="C420">
-        <v>-19.648755345027759</v>
+        <v>3.103035586116154</v>
       </c>
       <c r="D420">
-        <v>-40.641293430448606</v>
+        <v>-51.262694845104477</v>
       </c>
     </row>
     <row r="421" spans="2:4">
@@ -14137,10 +14137,10 @@
         <v>815</v>
       </c>
       <c r="C421">
-        <v>-12.506596441388329</v>
+        <v>0.35845074336695881</v>
       </c>
       <c r="D421">
-        <v>-40.258955780606243</v>
+        <v>-51.462477261462482</v>
       </c>
     </row>
     <row r="422" spans="2:4">
@@ -14148,10 +14148,10 @@
         <v>816</v>
       </c>
       <c r="C422">
-        <v>-15.023408716440285</v>
+        <v>-8.7156301895408426</v>
       </c>
       <c r="D422">
-        <v>-41.635494324108421</v>
+        <v>-71.752253055951869</v>
       </c>
     </row>
     <row r="423" spans="2:4">
@@ -14159,10 +14159,10 @@
         <v>817</v>
       </c>
       <c r="C423">
-        <v>-16.039640727449015</v>
+        <v>-4.7231928172485764</v>
       </c>
       <c r="D423">
-        <v>-39.733113382833757</v>
+        <v>-69.868427092214759</v>
       </c>
     </row>
     <row r="424" spans="2:4">
@@ -14170,10 +14170,10 @@
         <v>818</v>
       </c>
       <c r="C424">
-        <v>-11.205793772429621</v>
+        <v>-5.7973810294751082</v>
       </c>
       <c r="D424">
-        <v>-52.372806573735268</v>
+        <v>-72.110290154322939</v>
       </c>
     </row>
     <row r="425" spans="2:4">
@@ -14181,10 +14181,10 @@
         <v>819</v>
       </c>
       <c r="C425">
-        <v>-10.51524420742685</v>
+        <v>-6.8216069992724968</v>
       </c>
       <c r="D425">
-        <v>-54.437224876101297</v>
+        <v>-70.270923742361575</v>
       </c>
     </row>
     <row r="426" spans="2:4">
@@ -14192,10 +14192,10 @@
         <v>820</v>
       </c>
       <c r="C426">
-        <v>-12.032374989088204</v>
+        <v>-8.075922243414615</v>
       </c>
       <c r="D426">
-        <v>-50.039166128718826</v>
+        <v>-64.807492981879449</v>
       </c>
     </row>
     <row r="427" spans="2:4">
@@ -14203,10 +14203,10 @@
         <v>821</v>
       </c>
       <c r="C427">
-        <v>-8.6006972840319094</v>
+        <v>-5.6439255705856022</v>
       </c>
       <c r="D427">
-        <v>-50.434556576148779</v>
+        <v>-66.051200797273779</v>
       </c>
     </row>
     <row r="428" spans="2:4">
@@ -14214,10 +14214,10 @@
         <v>822</v>
       </c>
       <c r="C428">
-        <v>-16.902698173281436</v>
+        <v>-9.7806610992693646</v>
       </c>
       <c r="D428">
-        <v>-50.477386604703518</v>
+        <v>-68.648791040989394</v>
       </c>
     </row>
     <row r="429" spans="2:4">
@@ -14225,10 +14225,10 @@
         <v>823</v>
       </c>
       <c r="C429">
-        <v>-14.562185844187271</v>
+        <v>-10.993454242105772</v>
       </c>
       <c r="D429">
-        <v>-50.808263143325782</v>
+        <v>-64.930269266219682</v>
       </c>
     </row>
     <row r="430" spans="2:4">
@@ -14236,10 +14236,10 @@
         <v>824</v>
       </c>
       <c r="C430">
-        <v>-15.907048622540906</v>
+        <v>-8.4567349333171133</v>
       </c>
       <c r="D430">
-        <v>-54.263941578829673</v>
+        <v>-67.108787303231466</v>
       </c>
     </row>
     <row r="431" spans="2:4">
@@ -14247,10 +14247,10 @@
         <v>825</v>
       </c>
       <c r="C431">
-        <v>-13.566509727206531</v>
+        <v>-17.700482366908048</v>
       </c>
       <c r="D431">
-        <v>-54.076925455405352</v>
+        <v>-56.56383959110709</v>
       </c>
     </row>
     <row r="432" spans="2:4">
@@ -14258,10 +14258,10 @@
         <v>826</v>
       </c>
       <c r="C432">
-        <v>-12.986303040932638</v>
+        <v>-15.485059836485544</v>
       </c>
       <c r="D432">
-        <v>-56.282385117747381</v>
+        <v>-59.834575116941323</v>
       </c>
     </row>
     <row r="433" spans="2:4">
@@ -14269,10 +14269,10 @@
         <v>827</v>
       </c>
       <c r="C433">
-        <v>-24.317475893549901</v>
+        <v>-15.28188005060704</v>
       </c>
       <c r="D433">
-        <v>-47.675635256259191</v>
+        <v>-57.770445342639903</v>
       </c>
     </row>
     <row r="434" spans="2:4">
@@ -14280,10 +14280,10 @@
         <v>828</v>
       </c>
       <c r="C434">
-        <v>-26.606655001212371</v>
+        <v>-16.189527454736439</v>
       </c>
       <c r="D434">
-        <v>-48.419250768260682</v>
+        <v>-55.023658167444282</v>
       </c>
     </row>
     <row r="435" spans="2:4">
@@ -14291,10 +14291,10 @@
         <v>829</v>
       </c>
       <c r="C435">
-        <v>-23.369101691804023</v>
+        <v>-16.932884602229468</v>
       </c>
       <c r="D435">
-        <v>-45.747192361801993</v>
+        <v>-52.354383666906401</v>
       </c>
     </row>
     <row r="436" spans="2:4">
@@ -14302,10 +14302,10 @@
         <v>830</v>
       </c>
       <c r="C436">
-        <v>-22.709600091739361</v>
+        <v>-19.055465050628719</v>
       </c>
       <c r="D436">
-        <v>-47.764869117699376</v>
+        <v>-52.875815457428217</v>
       </c>
     </row>
     <row r="437" spans="2:4">
@@ -14313,10 +14313,10 @@
         <v>831</v>
       </c>
       <c r="C437">
-        <v>-20.761072637002851</v>
+        <v>-19.487035455059758</v>
       </c>
       <c r="D437">
-        <v>-47.873932726126263</v>
+        <v>-49.782545873596746</v>
       </c>
     </row>
     <row r="438" spans="2:4">
@@ -14324,10 +14324,10 @@
         <v>832</v>
       </c>
       <c r="C438">
-        <v>-21.990143800759729</v>
+        <v>-13.333352595870542</v>
       </c>
       <c r="D438">
-        <v>-45.801724166015447</v>
+        <v>-56.457642648612577</v>
       </c>
     </row>
     <row r="439" spans="2:4">
@@ -14335,10 +14335,10 @@
         <v>833</v>
       </c>
       <c r="C439">
-        <v>-22.309902152306229</v>
+        <v>-14.068053776206758</v>
       </c>
       <c r="D439">
-        <v>-43.178138474413146</v>
+        <v>-53.998273814712888</v>
       </c>
     </row>
     <row r="440" spans="2:4">
@@ -14346,10 +14346,10 @@
         <v>834</v>
       </c>
       <c r="C440">
-        <v>-21.093430162727142</v>
+        <v>-10.76478090175701</v>
       </c>
       <c r="D440">
-        <v>-42.065110103389983</v>
+        <v>-56.724864025385003</v>
       </c>
     </row>
     <row r="441" spans="2:4">
@@ -14357,10 +14357,10 @@
         <v>835</v>
       </c>
       <c r="C441">
-        <v>-18.422839691319048</v>
+        <v>-12.8328536410102</v>
       </c>
       <c r="D441">
-        <v>-47.98299633455315</v>
+        <v>-58.923798316744872</v>
       </c>
     </row>
     <row r="442" spans="2:4">
@@ -14368,10 +14368,10 @@
         <v>836</v>
       </c>
       <c r="C442">
-        <v>-20.311412455140584</v>
+        <v>-10.920432503170872</v>
       </c>
       <c r="D442">
-        <v>-45.536855402693007</v>
+        <v>-59.745087027975664</v>
       </c>
     </row>
     <row r="443" spans="2:4">
@@ -14379,10 +14379,10 @@
         <v>837</v>
       </c>
       <c r="C443">
-        <v>-16.558479398828556</v>
+        <v>-10.797549659949404</v>
       </c>
       <c r="D443">
-        <v>-47.370562225694478</v>
+        <v>-62.712323662099848</v>
       </c>
     </row>
     <row r="444" spans="2:4">
@@ -14390,10 +14390,10 @@
         <v>838</v>
       </c>
       <c r="C444">
-        <v>-15.76984461833165</v>
+        <v>-12.837750122119409</v>
       </c>
       <c r="D444">
-        <v>-46.074383187082653</v>
+        <v>-61.770140765344891</v>
       </c>
     </row>
     <row r="445" spans="2:4">
@@ -14401,10 +14401,10 @@
         <v>839</v>
       </c>
       <c r="C445">
-        <v>-18.724376519156099</v>
+        <v>-8.8900438358389344</v>
       </c>
       <c r="D445">
-        <v>-45.083187451673609</v>
+        <v>-60.525311303644934</v>
       </c>
     </row>
     <row r="446" spans="2:4">
@@ -14412,10 +14412,10 @@
         <v>840</v>
       </c>
       <c r="C446">
-        <v>-17.645569948385692</v>
+        <v>-8.5536314034827186</v>
       </c>
       <c r="D446">
-        <v>-43.861949987565843</v>
+        <v>-62.738898615420247</v>
       </c>
     </row>
     <row r="447" spans="2:4">
@@ -14423,10 +14423,10 @@
         <v>841</v>
       </c>
       <c r="C447">
-        <v>-23.035824145247283</v>
+        <v>-21.092401192059267</v>
       </c>
       <c r="D447">
-        <v>-49.958972298993167</v>
+        <v>-57.574853686201827</v>
       </c>
     </row>
     <row r="448" spans="2:4">
@@ -14434,10 +14434,10 @@
         <v>842</v>
       </c>
       <c r="C448">
-        <v>-23.548965764548932</v>
+        <v>-19.681888200533407</v>
       </c>
       <c r="D448">
-        <v>-46.892360250284291</v>
+        <v>-56.889857689415422</v>
       </c>
     </row>
     <row r="449" spans="2:4">
@@ -14445,10 +14445,10 @@
         <v>843</v>
       </c>
       <c r="C449">
-        <v>-23.493622972935107</v>
+        <v>-14.17968270247326</v>
       </c>
       <c r="D449">
-        <v>-48.335355684855394</v>
+        <v>-58.284549894147112</v>
       </c>
     </row>
     <row r="450" spans="2:4">
@@ -14456,10 +14456,10 @@
         <v>844</v>
       </c>
       <c r="C450">
-        <v>-19.412092091416039</v>
+        <v>-18.437828364047789</v>
       </c>
       <c r="D450">
-        <v>-44.874683494386922</v>
+        <v>-56.09914652832051</v>
       </c>
     </row>
     <row r="451" spans="2:4">
@@ -14467,10 +14467,10 @@
         <v>845</v>
       </c>
       <c r="C451">
-        <v>-20.940936709747763</v>
+        <v>-17.035316844429754</v>
       </c>
       <c r="D451">
-        <v>-44.492960864892822</v>
+        <v>-58.273926815404231</v>
       </c>
     </row>
     <row r="452" spans="2:4">
@@ -14478,10 +14478,10 @@
         <v>846</v>
       </c>
       <c r="C452">
-        <v>-20.96092160671942</v>
+        <v>-25.423338733153766</v>
       </c>
       <c r="D452">
-        <v>-47.995114513267239</v>
+        <v>-50.141307743422033</v>
       </c>
     </row>
     <row r="453" spans="2:4">
@@ -14489,10 +14489,10 @@
         <v>847</v>
       </c>
       <c r="C453">
-        <v>-21.922694773480387</v>
+        <v>-28.899921928709954</v>
       </c>
       <c r="D453">
-        <v>-48.237478087549214</v>
+        <v>-51.25490458735969</v>
       </c>
     </row>
     <row r="454" spans="2:4">
@@ -14500,10 +14500,10 @@
         <v>848</v>
       </c>
       <c r="C454">
-        <v>-27.345382442843249</v>
+        <v>-27.337352796738564</v>
       </c>
       <c r="D454">
-        <v>-51.53535386617169</v>
+        <v>-51.14584097893281</v>
       </c>
     </row>
     <row r="455" spans="2:4">
@@ -14511,10 +14511,10 @@
         <v>849</v>
       </c>
       <c r="C455">
-        <v>-28.899921928709954</v>
+        <v>-28.180465637730322</v>
       </c>
       <c r="D455">
-        <v>-51.25490458735969</v>
+        <v>-50.259699160464372</v>
       </c>
     </row>
     <row r="456" spans="2:4">
@@ -14522,10 +14522,10 @@
         <v>850</v>
       </c>
       <c r="C456">
-        <v>-28.180465637730322</v>
+        <v>-28.904918152952877</v>
       </c>
       <c r="D456">
-        <v>-50.259699160464372</v>
+        <v>-55.266021741726256</v>
       </c>
     </row>
     <row r="457" spans="2:4">
@@ -14533,10 +14533,10 @@
         <v>851</v>
       </c>
       <c r="C457">
-        <v>-25.932164728418968</v>
+        <v>-28.092488645626837</v>
       </c>
       <c r="D457">
-        <v>-49.946141286237072</v>
+        <v>-53.374532107656123</v>
       </c>
     </row>
     <row r="458" spans="2:4">
@@ -14544,10 +14544,10 @@
         <v>852</v>
       </c>
       <c r="C458">
-        <v>-25.068343852736184</v>
+        <v>-31.725863225490532</v>
       </c>
       <c r="D458">
-        <v>-51.088439079760768</v>
+        <v>-51.942844271283128</v>
       </c>
     </row>
     <row r="459" spans="2:4">
@@ -14555,10 +14555,10 @@
         <v>853</v>
       </c>
       <c r="C459">
-        <v>-28.904918152952877</v>
+        <v>-30.336189450775912</v>
       </c>
       <c r="D459">
-        <v>-55.266021741726256</v>
+        <v>-52.396864722652957</v>
       </c>
     </row>
     <row r="460" spans="2:4">
@@ -14566,10 +14566,10 @@
         <v>854</v>
       </c>
       <c r="C460">
-        <v>-28.135499619544092</v>
+        <v>-30.611440995923225</v>
       </c>
       <c r="D460">
-        <v>-53.572506266431006</v>
+        <v>-55.184602728490901</v>
       </c>
     </row>
     <row r="461" spans="2:4">
@@ -14577,10 +14577,10 @@
         <v>855</v>
       </c>
       <c r="C461">
-        <v>-31.725863225490532</v>
+        <v>-22.217115130652115</v>
       </c>
       <c r="D461">
-        <v>-51.942844271283128</v>
+        <v>-48.704893552235859</v>
       </c>
     </row>
     <row r="462" spans="2:4">
@@ -14588,10 +14588,10 @@
         <v>856</v>
       </c>
       <c r="C462">
-        <v>-30.336189450775912</v>
+        <v>-23.548965764548932</v>
       </c>
       <c r="D462">
-        <v>-52.396864722652957</v>
+        <v>-46.892360250284291</v>
       </c>
     </row>
     <row r="463" spans="2:4">
@@ -14599,10 +14599,10 @@
         <v>857</v>
       </c>
       <c r="C463">
-        <v>-30.611440995923225</v>
+        <v>-23.518988419091443</v>
       </c>
       <c r="D463">
-        <v>-55.184602728490901</v>
+        <v>-48.564668912829866</v>
       </c>
     </row>
     <row r="464" spans="2:4">
@@ -14610,10 +14610,10 @@
         <v>858</v>
       </c>
       <c r="C464">
-        <v>-14.17968270247326</v>
+        <v>-19.412092091416039</v>
       </c>
       <c r="D464">
-        <v>-58.284549894147112</v>
+        <v>-44.874683494386922</v>
       </c>
     </row>
     <row r="465" spans="2:4">
@@ -14621,10 +14621,10 @@
         <v>859</v>
       </c>
       <c r="C465">
-        <v>-21.092401192059267</v>
+        <v>-20.940936709747763</v>
       </c>
       <c r="D465">
-        <v>-57.574853686201827</v>
+        <v>-44.492960864892822</v>
       </c>
     </row>
     <row r="466" spans="2:4">
@@ -14632,10 +14632,10 @@
         <v>860</v>
       </c>
       <c r="C466">
-        <v>-17.135687420738297</v>
+        <v>-21.833339224520579</v>
       </c>
       <c r="D466">
-        <v>-58.064563638513327</v>
+        <v>-50.810260645311615</v>
       </c>
     </row>
     <row r="467" spans="2:4">
@@ -14643,10 +14643,10 @@
         <v>861</v>
       </c>
       <c r="C467">
-        <v>-18.635406322744849</v>
+        <v>-21.435562909796261</v>
       </c>
       <c r="D467">
-        <v>-55.954554623209113</v>
+        <v>-52.463692914091013</v>
       </c>
     </row>
     <row r="468" spans="2:4">
@@ -14654,10 +14654,10 @@
         <v>862</v>
       </c>
       <c r="C468">
-        <v>-19.681888200533407</v>
+        <v>-20.96092160671942</v>
       </c>
       <c r="D468">
-        <v>-56.889857689415422</v>
+        <v>-47.995114513267239</v>
       </c>
     </row>
     <row r="469" spans="2:4">
@@ -14665,10 +14665,10 @@
         <v>863</v>
       </c>
       <c r="C469">
-        <v>-21.840257073472305</v>
+        <v>-19.243469523217691</v>
       </c>
       <c r="D469">
-        <v>-51.000422834363619</v>
+        <v>-49.57805160779634</v>
       </c>
     </row>
     <row r="470" spans="2:4">
@@ -14676,10 +14676,10 @@
         <v>864</v>
       </c>
       <c r="C470">
-        <v>-23.4162089489515</v>
+        <v>-20.2552049324078</v>
       </c>
       <c r="D470">
-        <v>-52.548087372992768</v>
+        <v>-50.430111048631375</v>
       </c>
     </row>
     <row r="471" spans="2:4">
@@ -14687,10 +14687,10 @@
         <v>865</v>
       </c>
       <c r="C471">
-        <v>-25.83580897516277</v>
+        <v>-19.476329260253511</v>
       </c>
       <c r="D471">
-        <v>-53.482918302366073</v>
+        <v>-55.196775006217123</v>
       </c>
     </row>
     <row r="472" spans="2:4">
@@ -14698,10 +14698,10 @@
         <v>866</v>
       </c>
       <c r="C472">
-        <v>-21.685374121941965</v>
+        <v>-19.974167318743884</v>
       </c>
       <c r="D472">
-        <v>-55.175135401370511</v>
+        <v>-54.008760700138552</v>
       </c>
     </row>
     <row r="473" spans="2:4">
@@ -14709,10 +14709,10 @@
         <v>867</v>
       </c>
       <c r="C473">
-        <v>-23.144271600872891</v>
+        <v>-19.611941061132608</v>
       </c>
       <c r="D473">
-        <v>-54.363217427525932</v>
+        <v>-52.418249743913137</v>
       </c>
     </row>
     <row r="474" spans="2:4">
@@ -14720,10 +14720,10 @@
         <v>868</v>
       </c>
       <c r="C474">
-        <v>-15.927225681983444</v>
+        <v>-17.838281454898095</v>
       </c>
       <c r="D474">
-        <v>-49.918875384130345</v>
+        <v>-52.859697682783867</v>
       </c>
     </row>
     <row r="475" spans="2:4">
@@ -14731,10 +14731,10 @@
         <v>869</v>
       </c>
       <c r="C475">
-        <v>-17.50968362969105</v>
+        <v>-23.90869391003875</v>
       </c>
       <c r="D475">
-        <v>-50.768313103608975</v>
+        <v>-51.09130917471937</v>
       </c>
     </row>
     <row r="476" spans="2:4">
@@ -14742,10 +14742,10 @@
         <v>870</v>
       </c>
       <c r="C476">
-        <v>-20.311412455140584</v>
+        <v>-25.91717605569022</v>
       </c>
       <c r="D476">
-        <v>-52.42894225454323</v>
+        <v>-52.381895207770853</v>
       </c>
     </row>
     <row r="477" spans="2:4">
@@ -14753,10 +14753,10 @@
         <v>871</v>
       </c>
       <c r="C477">
-        <v>-19.243469523217691</v>
+        <v>-23.530032704259995</v>
       </c>
       <c r="D477">
-        <v>-49.57805160779634</v>
+        <v>-52.523486559061887</v>
       </c>
     </row>
     <row r="478" spans="2:4">
@@ -14764,10 +14764,10 @@
         <v>872</v>
       </c>
       <c r="C478">
-        <v>-20.2552049324078</v>
+        <v>-22.074080368040683</v>
       </c>
       <c r="D478">
-        <v>-50.430111048631375</v>
+        <v>-54.832190943761525</v>
       </c>
     </row>
     <row r="479" spans="2:4">
@@ -14775,10 +14775,10 @@
         <v>873</v>
       </c>
       <c r="C479">
-        <v>-18.095230130247963</v>
+        <v>-26.83148509214351</v>
       </c>
       <c r="D479">
-        <v>-53.482918302366059</v>
+        <v>-53.327113147470506</v>
       </c>
     </row>
     <row r="480" spans="2:4">
@@ -14786,10 +14786,10 @@
         <v>874</v>
       </c>
       <c r="C480">
-        <v>-19.909084924000659</v>
+        <v>-24.524018369429225</v>
       </c>
       <c r="D480">
-        <v>-54.360347332567322</v>
+        <v>-54.274244483809248</v>
       </c>
     </row>
     <row r="481" spans="2:4">
@@ -14797,10 +14797,10 @@
         <v>875</v>
       </c>
       <c r="C481">
-        <v>-11.719691123129357</v>
+        <v>-12.195046172526611</v>
       </c>
       <c r="D481">
-        <v>-41.739104752113967</v>
+        <v>-42.202625087928219</v>
       </c>
     </row>
     <row r="482" spans="2:4">
@@ -14819,10 +14819,10 @@
         <v>877</v>
       </c>
       <c r="C483">
-        <v>-8.9973820727996046</v>
+        <v>-9.5524700549726198</v>
       </c>
       <c r="D483">
-        <v>-39.13125314739046</v>
+        <v>-39.601059013745463</v>
       </c>
     </row>
     <row r="484" spans="2:4">
@@ -14830,10 +14830,10 @@
         <v>878</v>
       </c>
       <c r="C484">
-        <v>-17.368182173860266</v>
+        <v>-15.814810636517883</v>
       </c>
       <c r="D484">
-        <v>-41.776285527714045</v>
+        <v>-41.506025266362961</v>
       </c>
     </row>
     <row r="485" spans="2:4">
@@ -14841,10 +14841,10 @@
         <v>879</v>
       </c>
       <c r="C485">
-        <v>-14.960456290979568</v>
+        <v>-12.981951490785582</v>
       </c>
       <c r="D485">
-        <v>-41.357382122619882</v>
+        <v>-39.039780443548558</v>
       </c>
     </row>
     <row r="486" spans="2:4">
@@ -14852,10 +14852,10 @@
         <v>880</v>
       </c>
       <c r="C486">
-        <v>-12.981951490785582</v>
+        <v>-11.641402073608694</v>
       </c>
       <c r="D486">
-        <v>-39.039780443548558</v>
+        <v>-39.489667828309457</v>
       </c>
     </row>
     <row r="487" spans="2:4">
@@ -14863,10 +14863,10 @@
         <v>881</v>
       </c>
       <c r="C487">
-        <v>-11.641402073608694</v>
+        <v>0.56780865599745611</v>
       </c>
       <c r="D487">
-        <v>-39.489667828309457</v>
+        <v>-50.346041183802321</v>
       </c>
     </row>
     <row r="488" spans="2:4">
@@ -14874,10 +14874,10 @@
         <v>882</v>
       </c>
       <c r="C488">
-        <v>0.56780865599745611</v>
+        <v>-1.8224438009213897</v>
       </c>
       <c r="D488">
-        <v>-50.346041183802321</v>
+        <v>-46.302133663503504</v>
       </c>
     </row>
     <row r="489" spans="2:4">
@@ -14885,10 +14885,10 @@
         <v>883</v>
       </c>
       <c r="C489">
-        <v>-1.8224438009213897</v>
+        <v>-2.692908965809846</v>
       </c>
       <c r="D489">
-        <v>-46.302133663503504</v>
+        <v>-43.461814021584082</v>
       </c>
     </row>
     <row r="490" spans="2:4">
@@ -14896,10 +14896,10 @@
         <v>884</v>
       </c>
       <c r="C490">
-        <v>-2.692908965809846</v>
+        <v>-9.7708487803103203</v>
       </c>
       <c r="D490">
-        <v>-43.461814021584082</v>
+        <v>-36.614719032644885</v>
       </c>
     </row>
     <row r="491" spans="2:4">
@@ -14907,10 +14907,10 @@
         <v>885</v>
       </c>
       <c r="C491">
-        <v>-9.7708487803103203</v>
+        <v>-4.6375432587986198</v>
       </c>
       <c r="D491">
-        <v>-36.614719032644885</v>
+        <v>-40.426446322118963</v>
       </c>
     </row>
     <row r="492" spans="2:4">
@@ -14918,10 +14918,10 @@
         <v>886</v>
       </c>
       <c r="C492">
-        <v>-4.6375432587986198</v>
+        <v>-5.781767828716001</v>
       </c>
       <c r="D492">
-        <v>-40.426446322118963</v>
+        <v>-36.456336218936713</v>
       </c>
     </row>
     <row r="493" spans="2:4">
@@ -14929,10 +14929,10 @@
         <v>887</v>
       </c>
       <c r="C493">
-        <v>-5.781767828716001</v>
+        <v>-5.9998142531104177</v>
       </c>
       <c r="D493">
-        <v>-36.456336218936713</v>
+        <v>-38.133424249380312</v>
       </c>
     </row>
     <row r="494" spans="2:4">
@@ -14940,10 +14940,10 @@
         <v>888</v>
       </c>
       <c r="C494">
-        <v>-5.9998142531104177</v>
+        <v>3.4859879388010531</v>
       </c>
       <c r="D494">
-        <v>-38.133424249380312</v>
+        <v>-60.164562445002161</v>
       </c>
     </row>
     <row r="495" spans="2:4">
@@ -14951,10 +14951,10 @@
         <v>889</v>
       </c>
       <c r="C495">
-        <v>3.4859879388010531</v>
+        <v>-16.938961091173553</v>
       </c>
       <c r="D495">
-        <v>-60.164562445002161</v>
+        <v>-39.460454361766544</v>
       </c>
     </row>
     <row r="496" spans="2:4">
@@ -14962,10 +14962,10 @@
         <v>890</v>
       </c>
       <c r="C496">
-        <v>-16.938961091173553</v>
+        <v>-17.959343811553321</v>
       </c>
       <c r="D496">
-        <v>-39.460454361766544</v>
+        <v>-40.491165386460189</v>
       </c>
     </row>
     <row r="497" spans="2:4">
@@ -14973,10 +14973,10 @@
         <v>891</v>
       </c>
       <c r="C497">
-        <v>-17.959343811553321</v>
+        <v>-19.925989442115782</v>
       </c>
       <c r="D497">
-        <v>-40.491165386460189</v>
+        <v>-40.083674981348743</v>
       </c>
     </row>
     <row r="498" spans="2:4">
@@ -14984,10 +14984,10 @@
         <v>892</v>
       </c>
       <c r="C498">
-        <v>-19.925989442115782</v>
+        <v>-21.946540389185209</v>
       </c>
       <c r="D498">
-        <v>-40.083674981348743</v>
+        <v>-41.379690587979908</v>
       </c>
     </row>
     <row r="499" spans="2:4">
@@ -14995,10 +14995,10 @@
         <v>893</v>
       </c>
       <c r="C499">
-        <v>-21.946540389185209</v>
+        <v>-28.405295728661457</v>
       </c>
       <c r="D499">
-        <v>-41.379690587979908</v>
+        <v>-48.964568810395107</v>
       </c>
     </row>
     <row r="500" spans="2:4">
@@ -15006,10 +15006,10 @@
         <v>894</v>
       </c>
       <c r="C500">
-        <v>-28.405295728661457</v>
+        <v>-23.346618682710911</v>
       </c>
       <c r="D500">
-        <v>-48.964568810395107</v>
+        <v>-44.465694962786102</v>
       </c>
     </row>
     <row r="501" spans="2:4">
@@ -15017,10 +15017,10 @@
         <v>895</v>
       </c>
       <c r="C501">
-        <v>-23.346618682710911</v>
+        <v>-10.07503066804068</v>
       </c>
       <c r="D501">
-        <v>-44.465694962786102</v>
+        <v>-46.302133663503497</v>
       </c>
     </row>
     <row r="502" spans="2:4">
@@ -15028,10 +15028,10 @@
         <v>896</v>
       </c>
       <c r="C502">
-        <v>-10.07503066804068</v>
+        <v>-12.161321658886941</v>
       </c>
       <c r="D502">
-        <v>-46.302133663503497</v>
+        <v>-48.351086012993882</v>
       </c>
     </row>
     <row r="503" spans="2:4">
@@ -15039,10 +15039,10 @@
         <v>897</v>
       </c>
       <c r="C503">
-        <v>-12.161321658886941</v>
+        <v>-12.570833610225796</v>
       </c>
       <c r="D503">
-        <v>-48.351086012993882</v>
+        <v>-46.393783754618518</v>
       </c>
     </row>
     <row r="504" spans="2:4">
@@ -15050,10 +15050,10 @@
         <v>898</v>
       </c>
       <c r="C504">
-        <v>-12.570833610225796</v>
+        <v>-6.7466636356287859</v>
       </c>
       <c r="D504">
-        <v>-46.393783754618518</v>
+        <v>-44.602024473319695</v>
       </c>
     </row>
     <row r="505" spans="2:4">
@@ -15061,10 +15061,10 @@
         <v>899</v>
       </c>
       <c r="C505">
-        <v>-6.7466636356287859</v>
+        <v>-7.1390141864693932</v>
       </c>
       <c r="D505">
-        <v>-44.602024473319695</v>
+        <v>-43.51138838905085</v>
       </c>
     </row>
     <row r="506" spans="2:4">
@@ -15072,10 +15072,10 @@
         <v>900</v>
       </c>
       <c r="C506">
-        <v>-7.1390141864693932</v>
+        <v>-9.9467452632152664</v>
       </c>
       <c r="D506">
-        <v>-43.51138838905085</v>
+        <v>-44.738353983853301</v>
       </c>
     </row>
     <row r="507" spans="2:4">
@@ -15083,10 +15083,10 @@
         <v>901</v>
       </c>
       <c r="C507">
-        <v>-9.9467452632152664</v>
+        <v>-8.3856424144456074</v>
       </c>
       <c r="D507">
-        <v>-44.738353983853301</v>
+        <v>-42.076964843436379</v>
       </c>
     </row>
     <row r="508" spans="2:4">
@@ -15094,10 +15094,10 @@
         <v>902</v>
       </c>
       <c r="C508">
-        <v>-8.3856424144456074</v>
+        <v>-16.211569620513998</v>
       </c>
       <c r="D508">
-        <v>-42.076964843436379</v>
+        <v>-45.083187451673609</v>
       </c>
     </row>
     <row r="509" spans="2:4">
@@ -15105,10 +15105,10 @@
         <v>903</v>
       </c>
       <c r="C509">
-        <v>-16.211569620513998</v>
+        <v>-13.664261940654852</v>
       </c>
       <c r="D509">
-        <v>-45.083187451673609</v>
+        <v>-45.147342515454127</v>
       </c>
     </row>
     <row r="510" spans="2:4">
@@ -15116,10 +15116,10 @@
         <v>904</v>
       </c>
       <c r="C510">
-        <v>-13.664261940654852</v>
+        <v>-16.435769935280067</v>
       </c>
       <c r="D510">
-        <v>-45.147342515454127</v>
+        <v>-43.485420863234928</v>
       </c>
     </row>
     <row r="511" spans="2:4">
@@ -15127,10 +15127,10 @@
         <v>905</v>
       </c>
       <c r="C511">
-        <v>-16.244920375690491</v>
+        <v>-12.779604408947565</v>
       </c>
       <c r="D511">
-        <v>-43.440259948772457</v>
+        <v>-43.511388389050857</v>
       </c>
     </row>
     <row r="512" spans="2:4">
@@ -15138,10 +15138,10 @@
         <v>906</v>
       </c>
       <c r="C512">
-        <v>-12.779604408947565</v>
+        <v>-16.921666468794236</v>
       </c>
       <c r="D512">
-        <v>-43.511388389050857</v>
+        <v>-50.306890144879851</v>
       </c>
     </row>
     <row r="513" spans="2:4">
@@ -15182,10 +15182,10 @@
         <v>910</v>
       </c>
       <c r="C516">
-        <v>-29.884660564910089</v>
+        <v>-33.819187156204961</v>
       </c>
       <c r="D516">
-        <v>-48.041622626778846</v>
+        <v>-52.172869539803003</v>
       </c>
     </row>
     <row r="517" spans="2:4">
@@ -15193,10 +15193,10 @@
         <v>911</v>
       </c>
       <c r="C517">
-        <v>-29.986856060787883</v>
+        <v>-33.200904406144339</v>
       </c>
       <c r="D517">
-        <v>-49.136498542094962</v>
+        <v>-50.632404589183821</v>
       </c>
     </row>
     <row r="518" spans="2:4">
@@ -15204,10 +15204,10 @@
         <v>912</v>
       </c>
       <c r="C518">
-        <v>-31.554826954684241</v>
+        <v>-31.908131383290311</v>
       </c>
       <c r="D518">
-        <v>-50.322310995228015</v>
+        <v>-50.562383455064769</v>
       </c>
     </row>
     <row r="519" spans="2:4">
@@ -15215,10 +15215,10 @@
         <v>913</v>
       </c>
       <c r="C519">
-        <v>-32.987315819759758</v>
+        <v>-29.300102328489139</v>
       </c>
       <c r="D519">
-        <v>-50.954501806131468</v>
+        <v>-49.105943865388461</v>
       </c>
     </row>
     <row r="520" spans="2:4">
@@ -15226,10 +15226,10 @@
         <v>914</v>
       </c>
       <c r="C520">
-        <v>-33.916613528941788</v>
+        <v>-30.604116855889725</v>
       </c>
       <c r="D520">
-        <v>-52.168201464195072</v>
+        <v>-49.554079123750412</v>
       </c>
     </row>
     <row r="521" spans="2:4">
@@ -15237,10 +15237,10 @@
         <v>915</v>
       </c>
       <c r="C521">
-        <v>-26.152481055453244</v>
+        <v>-29.884660564910089</v>
       </c>
       <c r="D521">
-        <v>-47.537470461121664</v>
+        <v>-48.041622626778846</v>
       </c>
     </row>
     <row r="522" spans="2:4">
@@ -15248,10 +15248,10 @@
         <v>916</v>
       </c>
       <c r="C522">
-        <v>-27.051801419177785</v>
+        <v>-28.400781964764601</v>
       </c>
       <c r="D522">
-        <v>-48.097639534074077</v>
+        <v>-47.593487368416909</v>
       </c>
     </row>
     <row r="523" spans="2:4">
@@ -15259,10 +15259,10 @@
         <v>917</v>
       </c>
       <c r="C523">
-        <v>-27.26164283738018</v>
+        <v>-25.291702993031183</v>
       </c>
       <c r="D523">
-        <v>-46.734561456556527</v>
+        <v>-46.64119994439779</v>
       </c>
     </row>
     <row r="524" spans="2:4">
@@ -15270,10 +15270,10 @@
         <v>918</v>
       </c>
       <c r="C524">
-        <v>-28.351728126743261</v>
+        <v>-26.062549019080791</v>
       </c>
       <c r="D524">
-        <v>-47.557840245592665</v>
+        <v>-45.800946334969154</v>
       </c>
     </row>
     <row r="525" spans="2:4">
@@ -15281,10 +15281,10 @@
         <v>919</v>
       </c>
       <c r="C525">
-        <v>-24.263908291631708</v>
+        <v>-27.347292395830131</v>
       </c>
       <c r="D525">
-        <v>-45.120741032098337</v>
+        <v>-46.801248250955616</v>
       </c>
     </row>
     <row r="526" spans="2:4">
@@ -15292,10 +15292,10 @@
         <v>920</v>
       </c>
       <c r="C526">
-        <v>-23.51447465519459</v>
+        <v>-26.602141237315514</v>
       </c>
       <c r="D526">
-        <v>-43.653631555318178</v>
+        <v>-47.817554997597867</v>
       </c>
     </row>
     <row r="527" spans="2:4">
@@ -15303,10 +15303,10 @@
         <v>921</v>
       </c>
       <c r="C527">
-        <v>-24.78851183713769</v>
+        <v>-23.764285867340291</v>
       </c>
       <c r="D527">
-        <v>-44.400523652588085</v>
+        <v>-42.595534417519154</v>
       </c>
     </row>
     <row r="528" spans="2:4">
@@ -15314,10 +15314,10 @@
         <v>922</v>
       </c>
       <c r="C528">
-        <v>-25.163228655356249</v>
+        <v>-24.376323337097279</v>
       </c>
       <c r="D528">
-        <v>-46.921284480874007</v>
+        <v>-45.170756127897661</v>
       </c>
     </row>
     <row r="529" spans="2:4">
@@ -15325,10 +15325,10 @@
         <v>923</v>
       </c>
       <c r="C529">
-        <v>-25.837718928149656</v>
+        <v>-23.51447465519459</v>
       </c>
       <c r="D529">
-        <v>-45.894307847127891</v>
+        <v>-43.653631555318178</v>
       </c>
     </row>
     <row r="530" spans="2:4">
@@ -15336,10 +15336,10 @@
         <v>924</v>
       </c>
       <c r="C530">
-        <v>4.7391734384846727</v>
+        <v>-24.78851183713769</v>
       </c>
       <c r="D530">
-        <v>-50.469021942906032</v>
+        <v>-44.400523652588085</v>
       </c>
     </row>
     <row r="531" spans="2:4">
@@ -15347,10 +15347,10 @@
         <v>925</v>
       </c>
       <c r="C531">
-        <v>3.0368884642917968</v>
+        <v>4.7391734384846727</v>
       </c>
       <c r="D531">
-        <v>-49.28199700260209</v>
+        <v>-50.469021942906032</v>
       </c>
     </row>
     <row r="532" spans="2:4">
@@ -15358,10 +15358,10 @@
         <v>926</v>
       </c>
       <c r="C532">
-        <v>-15.945194927179701</v>
+        <v>3.1307735572080948</v>
       </c>
       <c r="D532">
-        <v>-37.958579313635177</v>
+        <v>-49.355865451782627</v>
       </c>
     </row>
     <row r="533" spans="2:4">
@@ -15369,10 +15369,10 @@
         <v>927</v>
       </c>
       <c r="C533">
-        <v>-17.331647154588367</v>
+        <v>-15.945194927179701</v>
       </c>
       <c r="D533">
-        <v>-38.051940825793913</v>
+        <v>-37.958579313635177</v>
       </c>
     </row>
     <row r="534" spans="2:4">
@@ -15380,10 +15380,10 @@
         <v>928</v>
       </c>
       <c r="C534">
-        <v>-19.767306473009</v>
+        <v>-17.331647154588367</v>
       </c>
       <c r="D534">
-        <v>-39.639086532492456</v>
+        <v>-38.051940825793913</v>
       </c>
     </row>
     <row r="535" spans="2:4">
@@ -15391,10 +15391,10 @@
         <v>929</v>
       </c>
       <c r="C535">
-        <v>-19.285527706728001</v>
+        <v>-19.767306473009</v>
       </c>
       <c r="D535">
-        <v>-38.238663850111386</v>
+        <v>-39.639086532492456</v>
       </c>
     </row>
     <row r="536" spans="2:4">
@@ -15402,10 +15402,10 @@
         <v>930</v>
       </c>
       <c r="C536">
-        <v>-23.764285867340291</v>
+        <v>-19.285527706728001</v>
       </c>
       <c r="D536">
-        <v>-42.595534417519154</v>
+        <v>-38.238663850111386</v>
       </c>
     </row>
     <row r="537" spans="2:4">
@@ -15435,10 +15435,10 @@
         <v>933</v>
       </c>
       <c r="C539">
-        <v>0.79715251082544769</v>
+        <v>1.0805746860598473</v>
       </c>
       <c r="D539">
-        <v>-46.678544549261268</v>
+        <v>-47.252293478527697</v>
       </c>
     </row>
     <row r="540" spans="2:4">
@@ -15446,10 +15446,10 @@
         <v>934</v>
       </c>
       <c r="C540">
-        <v>-0.78691353334900216</v>
+        <v>-3.8465993801935897E-2</v>
       </c>
       <c r="D540">
-        <v>-44.223628155866265</v>
+        <v>-44.960692725540511</v>
       </c>
     </row>
     <row r="541" spans="2:4">
@@ -15479,10 +15479,10 @@
         <v>937</v>
       </c>
       <c r="C543">
-        <v>-7.2267836232945966</v>
+        <v>-1.9058048045910807</v>
       </c>
       <c r="D543">
-        <v>-34.441962355656052</v>
+        <v>-42.533293409413325</v>
       </c>
     </row>
     <row r="544" spans="2:4">
@@ -15490,10 +15490,10 @@
         <v>938</v>
       </c>
       <c r="C544">
-        <v>-2.2980084076598377</v>
+        <v>-7.2267836232945966</v>
       </c>
       <c r="D544">
-        <v>-40.367306327330617</v>
+        <v>-34.441962355656052</v>
       </c>
     </row>
     <row r="545" spans="2:4">
@@ -15512,10 +15512,10 @@
         <v>940</v>
       </c>
       <c r="C546">
-        <v>-4.0651729223785544</v>
+        <v>-3.5923873597347971</v>
       </c>
       <c r="D546">
-        <v>-36.31168223915504</v>
+        <v>-37.118325704206541</v>
       </c>
     </row>
   </sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3EE21C4-9BC9-463B-91F6-8F3AB24D2584}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97D64882-575E-48A4-939D-590B8A30CD7B}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22033,7 +22033,7 @@
         <v>941</v>
       </c>
       <c r="H334" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
     </row>
     <row r="335" spans="2:8">
@@ -22113,7 +22113,7 @@
         <v>941</v>
       </c>
       <c r="H338" t="s">
-        <v>943</v>
+        <v>951</v>
       </c>
     </row>
     <row r="339" spans="2:8">
@@ -22153,7 +22153,7 @@
         <v>941</v>
       </c>
       <c r="H340" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="341" spans="2:8">
@@ -22173,7 +22173,7 @@
         <v>941</v>
       </c>
       <c r="H341" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
     </row>
     <row r="342" spans="2:8">
@@ -22213,7 +22213,7 @@
         <v>941</v>
       </c>
       <c r="H343" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
     </row>
     <row r="344" spans="2:8">
@@ -22233,7 +22233,7 @@
         <v>941</v>
       </c>
       <c r="H344" t="s">
-        <v>953</v>
+        <v>945</v>
       </c>
     </row>
     <row r="345" spans="2:8">
@@ -22253,7 +22253,7 @@
         <v>941</v>
       </c>
       <c r="H345" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="346" spans="2:8">
@@ -22313,7 +22313,7 @@
         <v>941</v>
       </c>
       <c r="H348" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
     </row>
     <row r="349" spans="2:8">
@@ -22333,7 +22333,7 @@
         <v>941</v>
       </c>
       <c r="H349" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
     </row>
     <row r="350" spans="2:8">
@@ -22353,7 +22353,7 @@
         <v>941</v>
       </c>
       <c r="H350" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
     </row>
     <row r="351" spans="2:8">
@@ -22373,7 +22373,7 @@
         <v>941</v>
       </c>
       <c r="H351" t="s">
-        <v>951</v>
+        <v>969</v>
       </c>
     </row>
     <row r="352" spans="2:8">
@@ -22393,7 +22393,7 @@
         <v>941</v>
       </c>
       <c r="H352" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
     </row>
     <row r="353" spans="2:8">
@@ -22413,7 +22413,7 @@
         <v>941</v>
       </c>
       <c r="H353" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
     </row>
     <row r="354" spans="2:8">
@@ -22433,7 +22433,7 @@
         <v>941</v>
       </c>
       <c r="H354" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
     </row>
     <row r="355" spans="2:8">
@@ -22453,7 +22453,7 @@
         <v>941</v>
       </c>
       <c r="H355" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
     </row>
     <row r="356" spans="2:8">
@@ -22473,7 +22473,7 @@
         <v>941</v>
       </c>
       <c r="H356" t="s">
-        <v>952</v>
+        <v>944</v>
       </c>
     </row>
     <row r="357" spans="2:8">
@@ -22493,7 +22493,7 @@
         <v>941</v>
       </c>
       <c r="H357" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="358" spans="2:8">
@@ -22513,7 +22513,7 @@
         <v>941</v>
       </c>
       <c r="H358" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="359" spans="2:8">
@@ -22533,7 +22533,7 @@
         <v>941</v>
       </c>
       <c r="H359" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="360" spans="2:8">
@@ -22553,7 +22553,7 @@
         <v>941</v>
       </c>
       <c r="H360" t="s">
-        <v>968</v>
+        <v>954</v>
       </c>
     </row>
     <row r="361" spans="2:8">
@@ -22573,7 +22573,7 @@
         <v>941</v>
       </c>
       <c r="H361" t="s">
-        <v>968</v>
+        <v>953</v>
       </c>
     </row>
     <row r="362" spans="2:8">
@@ -22593,7 +22593,7 @@
         <v>941</v>
       </c>
       <c r="H362" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
     </row>
     <row r="363" spans="2:8">
@@ -22613,7 +22613,7 @@
         <v>941</v>
       </c>
       <c r="H363" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
     </row>
     <row r="364" spans="2:8">
@@ -22633,7 +22633,7 @@
         <v>941</v>
       </c>
       <c r="H364" t="s">
-        <v>947</v>
+        <v>956</v>
       </c>
     </row>
     <row r="365" spans="2:8">
@@ -22653,7 +22653,7 @@
         <v>941</v>
       </c>
       <c r="H365" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
     </row>
     <row r="366" spans="2:8">
@@ -22673,7 +22673,7 @@
         <v>941</v>
       </c>
       <c r="H366" t="s">
-        <v>948</v>
+        <v>957</v>
       </c>
     </row>
     <row r="367" spans="2:8">
@@ -22693,7 +22693,7 @@
         <v>941</v>
       </c>
       <c r="H367" t="s">
-        <v>948</v>
+        <v>961</v>
       </c>
     </row>
     <row r="368" spans="2:8">
@@ -22713,7 +22713,7 @@
         <v>941</v>
       </c>
       <c r="H368" t="s">
-        <v>947</v>
+        <v>960</v>
       </c>
     </row>
     <row r="369" spans="2:8">
@@ -22733,7 +22733,7 @@
         <v>941</v>
       </c>
       <c r="H369" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
     </row>
     <row r="370" spans="2:8">
@@ -22753,7 +22753,7 @@
         <v>941</v>
       </c>
       <c r="H370" t="s">
-        <v>947</v>
+        <v>961</v>
       </c>
     </row>
     <row r="371" spans="2:8">
@@ -22773,7 +22773,7 @@
         <v>941</v>
       </c>
       <c r="H371" t="s">
-        <v>947</v>
+        <v>950</v>
       </c>
     </row>
     <row r="372" spans="2:8">
@@ -22793,7 +22793,7 @@
         <v>941</v>
       </c>
       <c r="H372" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
     <row r="373" spans="2:8">
@@ -22813,7 +22813,7 @@
         <v>941</v>
       </c>
       <c r="H373" t="s">
-        <v>949</v>
+        <v>957</v>
       </c>
     </row>
     <row r="374" spans="2:8">
@@ -22833,7 +22833,7 @@
         <v>941</v>
       </c>
       <c r="H374" t="s">
-        <v>949</v>
+        <v>961</v>
       </c>
     </row>
     <row r="375" spans="2:8">
@@ -22853,7 +22853,7 @@
         <v>941</v>
       </c>
       <c r="H375" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
     </row>
     <row r="376" spans="2:8">
@@ -22873,7 +22873,7 @@
         <v>941</v>
       </c>
       <c r="H376" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="377" spans="2:8">
@@ -22893,7 +22893,7 @@
         <v>941</v>
       </c>
       <c r="H377" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="378" spans="2:8">
@@ -22913,7 +22913,7 @@
         <v>941</v>
       </c>
       <c r="H378" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="379" spans="2:8">
@@ -22933,7 +22933,7 @@
         <v>941</v>
       </c>
       <c r="H379" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
     </row>
     <row r="380" spans="2:8">
@@ -22953,7 +22953,7 @@
         <v>941</v>
       </c>
       <c r="H380" t="s">
-        <v>952</v>
+        <v>967</v>
       </c>
     </row>
     <row r="381" spans="2:8">
@@ -22973,7 +22973,7 @@
         <v>941</v>
       </c>
       <c r="H381" t="s">
-        <v>952</v>
+        <v>965</v>
       </c>
     </row>
     <row r="382" spans="2:8">
@@ -22993,7 +22993,7 @@
         <v>941</v>
       </c>
       <c r="H382" t="s">
-        <v>952</v>
+        <v>955</v>
       </c>
     </row>
     <row r="383" spans="2:8">
@@ -23013,7 +23013,7 @@
         <v>941</v>
       </c>
       <c r="H383" t="s">
-        <v>969</v>
+        <v>956</v>
       </c>
     </row>
     <row r="384" spans="2:8">
@@ -23033,7 +23033,7 @@
         <v>941</v>
       </c>
       <c r="H384" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
     </row>
     <row r="385" spans="2:8">
@@ -23053,7 +23053,7 @@
         <v>941</v>
       </c>
       <c r="H385" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
     </row>
     <row r="386" spans="2:8">
@@ -23073,7 +23073,7 @@
         <v>941</v>
       </c>
       <c r="H386" t="s">
-        <v>970</v>
+        <v>956</v>
       </c>
     </row>
     <row r="387" spans="2:8">
@@ -23093,7 +23093,7 @@
         <v>941</v>
       </c>
       <c r="H387" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="388" spans="2:8">
@@ -23113,7 +23113,7 @@
         <v>941</v>
       </c>
       <c r="H388" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="389" spans="2:8">
@@ -23133,7 +23133,7 @@
         <v>941</v>
       </c>
       <c r="H389" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="390" spans="2:8">
@@ -23193,7 +23193,7 @@
         <v>941</v>
       </c>
       <c r="H392" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
     </row>
     <row r="393" spans="2:8">
@@ -23213,7 +23213,7 @@
         <v>941</v>
       </c>
       <c r="H393" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
     </row>
     <row r="394" spans="2:8">
@@ -23233,7 +23233,7 @@
         <v>941</v>
       </c>
       <c r="H394" t="s">
-        <v>971</v>
+        <v>949</v>
       </c>
     </row>
     <row r="395" spans="2:8">
@@ -23253,7 +23253,7 @@
         <v>941</v>
       </c>
       <c r="H395" t="s">
-        <v>971</v>
+        <v>949</v>
       </c>
     </row>
     <row r="396" spans="2:8">
@@ -23293,7 +23293,7 @@
         <v>941</v>
       </c>
       <c r="H397" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
     </row>
     <row r="398" spans="2:8">
@@ -23313,7 +23313,7 @@
         <v>941</v>
       </c>
       <c r="H398" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
     </row>
     <row r="399" spans="2:8">
@@ -23333,7 +23333,7 @@
         <v>941</v>
       </c>
       <c r="H399" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
     </row>
     <row r="400" spans="2:8">
@@ -23353,7 +23353,7 @@
         <v>941</v>
       </c>
       <c r="H400" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
     </row>
     <row r="401" spans="2:8">
@@ -23373,7 +23373,7 @@
         <v>941</v>
       </c>
       <c r="H401" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="402" spans="2:8">
@@ -23393,7 +23393,7 @@
         <v>941</v>
       </c>
       <c r="H402" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
     </row>
     <row r="403" spans="2:8">
@@ -23413,7 +23413,7 @@
         <v>941</v>
       </c>
       <c r="H403" t="s">
-        <v>954</v>
+        <v>970</v>
       </c>
     </row>
     <row r="404" spans="2:8">
@@ -23433,7 +23433,7 @@
         <v>941</v>
       </c>
       <c r="H404" t="s">
-        <v>950</v>
+        <v>970</v>
       </c>
     </row>
     <row r="405" spans="2:8">
@@ -23453,7 +23453,7 @@
         <v>941</v>
       </c>
       <c r="H405" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
     </row>
     <row r="406" spans="2:8">
@@ -23473,7 +23473,7 @@
         <v>941</v>
       </c>
       <c r="H406" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
     </row>
     <row r="407" spans="2:8">
@@ -23493,7 +23493,7 @@
         <v>941</v>
       </c>
       <c r="H407" t="s">
-        <v>960</v>
+        <v>947</v>
       </c>
     </row>
     <row r="408" spans="2:8">
@@ -23513,7 +23513,7 @@
         <v>941</v>
       </c>
       <c r="H408" t="s">
-        <v>957</v>
+        <v>947</v>
       </c>
     </row>
     <row r="409" spans="2:8">
@@ -23533,7 +23533,7 @@
         <v>941</v>
       </c>
       <c r="H409" t="s">
-        <v>960</v>
+        <v>950</v>
       </c>
     </row>
     <row r="410" spans="2:8">
@@ -23553,7 +23553,7 @@
         <v>941</v>
       </c>
       <c r="H410" t="s">
-        <v>961</v>
+        <v>954</v>
       </c>
     </row>
     <row r="411" spans="2:8">
@@ -23573,7 +23573,7 @@
         <v>941</v>
       </c>
       <c r="H411" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
     </row>
     <row r="412" spans="2:8">
@@ -23593,7 +23593,7 @@
         <v>941</v>
       </c>
       <c r="H412" t="s">
-        <v>961</v>
+        <v>947</v>
       </c>
     </row>
     <row r="413" spans="2:8">
@@ -23613,7 +23613,7 @@
         <v>941</v>
       </c>
       <c r="H413" t="s">
-        <v>961</v>
+        <v>949</v>
       </c>
     </row>
     <row r="414" spans="2:8">
@@ -23633,7 +23633,7 @@
         <v>941</v>
       </c>
       <c r="H414" t="s">
-        <v>958</v>
+        <v>949</v>
       </c>
     </row>
     <row r="415" spans="2:8">
@@ -23653,7 +23653,7 @@
         <v>941</v>
       </c>
       <c r="H415" t="s">
-        <v>956</v>
+        <v>949</v>
       </c>
     </row>
     <row r="416" spans="2:8">
@@ -23673,7 +23673,7 @@
         <v>941</v>
       </c>
       <c r="H416" t="s">
-        <v>956</v>
+        <v>949</v>
       </c>
     </row>
     <row r="417" spans="2:8">
@@ -23693,7 +23693,7 @@
         <v>941</v>
       </c>
       <c r="H417" t="s">
-        <v>963</v>
+        <v>949</v>
       </c>
     </row>
     <row r="418" spans="2:8">
@@ -23713,7 +23713,7 @@
         <v>941</v>
       </c>
       <c r="H418" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
     </row>
     <row r="419" spans="2:8">
@@ -23733,7 +23733,7 @@
         <v>941</v>
       </c>
       <c r="H419" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
     </row>
     <row r="420" spans="2:8">
@@ -23753,7 +23753,7 @@
         <v>941</v>
       </c>
       <c r="H420" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
     </row>
     <row r="421" spans="2:8">
@@ -23773,7 +23773,7 @@
         <v>941</v>
       </c>
       <c r="H421" t="s">
-        <v>956</v>
+        <v>971</v>
       </c>
     </row>
     <row r="422" spans="2:8">
@@ -23793,7 +23793,7 @@
         <v>941</v>
       </c>
       <c r="H422" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
     </row>
     <row r="423" spans="2:8">
@@ -23813,7 +23813,7 @@
         <v>941</v>
       </c>
       <c r="H423" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
     </row>
     <row r="424" spans="2:8">
@@ -23833,7 +23833,7 @@
         <v>941</v>
       </c>
       <c r="H424" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="425" spans="2:8">
@@ -23853,7 +23853,7 @@
         <v>941</v>
       </c>
       <c r="H425" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="426" spans="2:8">
@@ -23873,7 +23873,7 @@
         <v>941</v>
       </c>
       <c r="H426" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
     </row>
     <row r="427" spans="2:8">
@@ -23893,7 +23893,7 @@
         <v>941</v>
       </c>
       <c r="H427" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
     </row>
     <row r="428" spans="2:8">
@@ -23913,7 +23913,7 @@
         <v>941</v>
       </c>
       <c r="H428" t="s">
-        <v>954</v>
+        <v>968</v>
       </c>
     </row>
     <row r="429" spans="2:8">
@@ -23933,7 +23933,7 @@
         <v>941</v>
       </c>
       <c r="H429" t="s">
-        <v>954</v>
+        <v>948</v>
       </c>
     </row>
     <row r="430" spans="2:8">
@@ -23953,7 +23953,7 @@
         <v>941</v>
       </c>
       <c r="H430" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
     </row>
     <row r="431" spans="2:8">
@@ -23973,7 +23973,7 @@
         <v>941</v>
       </c>
       <c r="H431" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
     </row>
     <row r="432" spans="2:8">
@@ -24013,7 +24013,7 @@
         <v>941</v>
       </c>
       <c r="H433" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
     </row>
     <row r="434" spans="2:8">
@@ -24033,7 +24033,7 @@
         <v>941</v>
       </c>
       <c r="H434" t="s">
-        <v>969</v>
+        <v>947</v>
       </c>
     </row>
     <row r="435" spans="2:8">
@@ -24053,7 +24053,7 @@
         <v>941</v>
       </c>
       <c r="H435" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
     </row>
     <row r="436" spans="2:8">
@@ -24073,7 +24073,7 @@
         <v>941</v>
       </c>
       <c r="H436" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="437" spans="2:8">
@@ -24093,7 +24093,7 @@
         <v>941</v>
       </c>
       <c r="H437" t="s">
-        <v>946</v>
+        <v>953</v>
       </c>
     </row>
     <row r="438" spans="2:8">
@@ -24113,7 +24113,7 @@
         <v>941</v>
       </c>
       <c r="H438" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="439" spans="2:8">
@@ -24133,7 +24133,7 @@
         <v>941</v>
       </c>
       <c r="H439" t="s">
-        <v>944</v>
+        <v>947</v>
       </c>
     </row>
     <row r="440" spans="2:8">
@@ -24153,7 +24153,7 @@
         <v>941</v>
       </c>
       <c r="H440" t="s">
-        <v>944</v>
+        <v>947</v>
       </c>
     </row>
     <row r="441" spans="2:8">
@@ -24173,7 +24173,7 @@
         <v>941</v>
       </c>
       <c r="H441" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
     </row>
     <row r="442" spans="2:8">
@@ -24193,7 +24193,7 @@
         <v>941</v>
       </c>
       <c r="H442" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="443" spans="2:8">
@@ -24213,7 +24213,7 @@
         <v>941</v>
       </c>
       <c r="H443" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
     </row>
     <row r="444" spans="2:8">
@@ -24233,7 +24233,7 @@
         <v>941</v>
       </c>
       <c r="H444" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
     </row>
     <row r="445" spans="2:8">
@@ -24253,7 +24253,7 @@
         <v>941</v>
       </c>
       <c r="H445" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="446" spans="2:8">
@@ -24273,7 +24273,7 @@
         <v>941</v>
       </c>
       <c r="H446" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
     </row>
     <row r="447" spans="2:8">
@@ -24293,7 +24293,7 @@
         <v>941</v>
       </c>
       <c r="H447" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
     </row>
     <row r="448" spans="2:8">
@@ -24313,7 +24313,7 @@
         <v>941</v>
       </c>
       <c r="H448" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="449" spans="2:8">
@@ -24333,7 +24333,7 @@
         <v>941</v>
       </c>
       <c r="H449" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
     </row>
     <row r="450" spans="2:8">
@@ -24353,7 +24353,7 @@
         <v>941</v>
       </c>
       <c r="H450" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="451" spans="2:8">
@@ -24373,7 +24373,7 @@
         <v>941</v>
       </c>
       <c r="H451" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
     </row>
     <row r="452" spans="2:8">
@@ -24393,7 +24393,7 @@
         <v>941</v>
       </c>
       <c r="H452" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
     </row>
     <row r="453" spans="2:8">
@@ -24413,7 +24413,7 @@
         <v>941</v>
       </c>
       <c r="H453" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
     </row>
     <row r="454" spans="2:8">
@@ -24453,7 +24453,7 @@
         <v>941</v>
       </c>
       <c r="H455" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
     </row>
     <row r="456" spans="2:8">
@@ -24473,7 +24473,7 @@
         <v>941</v>
       </c>
       <c r="H456" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
     </row>
     <row r="457" spans="2:8">
@@ -24493,7 +24493,7 @@
         <v>941</v>
       </c>
       <c r="H457" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
     </row>
     <row r="458" spans="2:8">
@@ -24513,7 +24513,7 @@
         <v>941</v>
       </c>
       <c r="H458" t="s">
-        <v>942</v>
+        <v>969</v>
       </c>
     </row>
     <row r="459" spans="2:8">
@@ -24573,7 +24573,7 @@
         <v>941</v>
       </c>
       <c r="H461" t="s">
-        <v>969</v>
+        <v>946</v>
       </c>
     </row>
     <row r="462" spans="2:8">
@@ -24593,7 +24593,7 @@
         <v>941</v>
       </c>
       <c r="H462" t="s">
-        <v>943</v>
+        <v>946</v>
       </c>
     </row>
     <row r="463" spans="2:8">
@@ -24613,7 +24613,7 @@
         <v>941</v>
       </c>
       <c r="H463" t="s">
-        <v>943</v>
+        <v>946</v>
       </c>
     </row>
     <row r="464" spans="2:8">
@@ -24633,7 +24633,7 @@
         <v>941</v>
       </c>
       <c r="H464" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
     </row>
     <row r="465" spans="2:8">
@@ -24653,7 +24653,7 @@
         <v>941</v>
       </c>
       <c r="H465" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
     </row>
     <row r="466" spans="2:8">
@@ -24673,7 +24673,7 @@
         <v>941</v>
       </c>
       <c r="H466" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="467" spans="2:8">
@@ -24713,7 +24713,7 @@
         <v>941</v>
       </c>
       <c r="H468" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
     </row>
     <row r="469" spans="2:8">
@@ -24733,7 +24733,7 @@
         <v>941</v>
       </c>
       <c r="H469" t="s">
-        <v>946</v>
+        <v>953</v>
       </c>
     </row>
     <row r="470" spans="2:8">
@@ -24753,7 +24753,7 @@
         <v>941</v>
       </c>
       <c r="H470" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
     </row>
     <row r="471" spans="2:8">
@@ -24773,7 +24773,7 @@
         <v>941</v>
       </c>
       <c r="H471" t="s">
-        <v>942</v>
+        <v>951</v>
       </c>
     </row>
     <row r="472" spans="2:8">
@@ -24853,7 +24853,7 @@
         <v>941</v>
       </c>
       <c r="H475" t="s">
-        <v>954</v>
+        <v>942</v>
       </c>
     </row>
     <row r="476" spans="2:8">
@@ -24873,7 +24873,7 @@
         <v>941</v>
       </c>
       <c r="H476" t="s">
-        <v>951</v>
+        <v>942</v>
       </c>
     </row>
     <row r="477" spans="2:8">
@@ -24893,7 +24893,7 @@
         <v>941</v>
       </c>
       <c r="H477" t="s">
-        <v>953</v>
+        <v>942</v>
       </c>
     </row>
     <row r="478" spans="2:8">
@@ -24913,7 +24913,7 @@
         <v>941</v>
       </c>
       <c r="H478" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="479" spans="2:8">
@@ -24933,7 +24933,7 @@
         <v>941</v>
       </c>
       <c r="H479" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="480" spans="2:8">
@@ -24953,7 +24953,7 @@
         <v>941</v>
       </c>
       <c r="H480" t="s">
-        <v>951</v>
+        <v>942</v>
       </c>
     </row>
     <row r="481" spans="2:8">
@@ -25093,7 +25093,7 @@
         <v>941</v>
       </c>
       <c r="H487" t="s">
-        <v>956</v>
+        <v>969</v>
       </c>
     </row>
     <row r="488" spans="2:8">
@@ -25113,7 +25113,7 @@
         <v>941</v>
       </c>
       <c r="H488" t="s">
-        <v>969</v>
+        <v>949</v>
       </c>
     </row>
     <row r="489" spans="2:8">
@@ -25133,7 +25133,7 @@
         <v>941</v>
       </c>
       <c r="H489" t="s">
-        <v>949</v>
+        <v>961</v>
       </c>
     </row>
     <row r="490" spans="2:8">
@@ -25153,7 +25153,7 @@
         <v>941</v>
       </c>
       <c r="H490" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
     </row>
     <row r="491" spans="2:8">
@@ -25173,7 +25173,7 @@
         <v>941</v>
       </c>
       <c r="H491" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="492" spans="2:8">
@@ -25193,7 +25193,7 @@
         <v>941</v>
       </c>
       <c r="H492" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
     </row>
     <row r="493" spans="2:8">
@@ -25233,7 +25233,7 @@
         <v>941</v>
       </c>
       <c r="H494" t="s">
-        <v>965</v>
+        <v>970</v>
       </c>
     </row>
     <row r="495" spans="2:8">
@@ -25253,7 +25253,7 @@
         <v>941</v>
       </c>
       <c r="H495" t="s">
-        <v>971</v>
+        <v>956</v>
       </c>
     </row>
     <row r="496" spans="2:8">
@@ -25273,7 +25273,7 @@
         <v>941</v>
       </c>
       <c r="H496" t="s">
-        <v>956</v>
+        <v>967</v>
       </c>
     </row>
     <row r="497" spans="2:8">
@@ -25293,7 +25293,7 @@
         <v>941</v>
       </c>
       <c r="H497" t="s">
-        <v>967</v>
+        <v>969</v>
       </c>
     </row>
     <row r="498" spans="2:8">
@@ -25313,7 +25313,7 @@
         <v>941</v>
       </c>
       <c r="H498" t="s">
-        <v>969</v>
+        <v>944</v>
       </c>
     </row>
     <row r="499" spans="2:8">
@@ -25333,7 +25333,7 @@
         <v>941</v>
       </c>
       <c r="H499" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
     </row>
     <row r="500" spans="2:8">
@@ -25353,7 +25353,7 @@
         <v>941</v>
       </c>
       <c r="H500" t="s">
-        <v>945</v>
+        <v>969</v>
       </c>
     </row>
     <row r="501" spans="2:8">
@@ -25373,7 +25373,7 @@
         <v>941</v>
       </c>
       <c r="H501" t="s">
-        <v>969</v>
+        <v>961</v>
       </c>
     </row>
     <row r="502" spans="2:8">
@@ -25393,7 +25393,7 @@
         <v>941</v>
       </c>
       <c r="H502" t="s">
-        <v>961</v>
+        <v>950</v>
       </c>
     </row>
     <row r="503" spans="2:8">
@@ -25433,7 +25433,7 @@
         <v>941</v>
       </c>
       <c r="H504" t="s">
-        <v>950</v>
+        <v>961</v>
       </c>
     </row>
     <row r="505" spans="2:8">
@@ -25453,7 +25453,7 @@
         <v>941</v>
       </c>
       <c r="H505" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
     </row>
     <row r="506" spans="2:8">
@@ -25513,7 +25513,7 @@
         <v>941</v>
       </c>
       <c r="H508" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
     </row>
     <row r="509" spans="2:8">
@@ -25533,7 +25533,7 @@
         <v>941</v>
       </c>
       <c r="H509" t="s">
-        <v>953</v>
+        <v>956</v>
       </c>
     </row>
     <row r="510" spans="2:8">
@@ -25553,7 +25553,7 @@
         <v>941</v>
       </c>
       <c r="H510" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
     </row>
     <row r="511" spans="2:8">
@@ -25573,7 +25573,7 @@
         <v>941</v>
       </c>
       <c r="H511" t="s">
-        <v>953</v>
+        <v>956</v>
       </c>
     </row>
     <row r="512" spans="2:8">
@@ -25593,7 +25593,7 @@
         <v>941</v>
       </c>
       <c r="H512" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="513" spans="2:8">

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 10:04
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D07C8983-1018-4764-AD9D-80B72AD1517C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABD19684-B0C8-4FDF-93D1-3A99A687F7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9B6772F-99C1-4281-95F0-F7139F5DC23A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB7D81F-AA65-4FD2-B504-BC49CFBCA911}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97D64882-575E-48A4-939D-590B8A30CD7B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9789791-1C2F-4F0B-A9F2-16B6C3EBD80C}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 10:50
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABD19684-B0C8-4FDF-93D1-3A99A687F7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B4A2075-BA28-4C6F-B4A4-1212D163C3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB7D81F-AA65-4FD2-B504-BC49CFBCA911}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC8583D-2450-41A6-8CEA-15ED00FB39F1}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9789791-1C2F-4F0B-A9F2-16B6C3EBD80C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58BA46A1-4858-4C6E-9877-5989E1EDAEAE}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 11:21
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B4A2075-BA28-4C6F-B4A4-1212D163C3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{87332B56-84F1-4BC1-B4F4-199C6B9DECFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC8583D-2450-41A6-8CEA-15ED00FB39F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6678CE58-8113-4DD8-84CD-271A6EE4CEE9}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58BA46A1-4858-4C6E-9877-5989E1EDAEAE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80F1C76-00E7-4DE8-B148-47FB6201E0D1}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 11:53
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87332B56-84F1-4BC1-B4F4-199C6B9DECFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{702C80E7-5DF5-40E6-881C-67D7811DDCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6678CE58-8113-4DD8-84CD-271A6EE4CEE9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{347A00AB-D052-432C-ACF9-DBE3E0ACF28D}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D80F1C76-00E7-4DE8-B148-47FB6201E0D1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DA38D7-DB42-40A7-8B82-E70809FCC677}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 13:08
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{702C80E7-5DF5-40E6-881C-67D7811DDCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D011792-D48D-44EC-8D85-8073B685D231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{347A00AB-D052-432C-ACF9-DBE3E0ACF28D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECDE5239-836A-4EA3-B8EE-80ADBFE0F631}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DA38D7-DB42-40A7-8B82-E70809FCC677}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70A47465-53F6-46D1-829C-37A722620D9D}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 13:59
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D011792-D48D-44EC-8D85-8073B685D231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D911DF41-F638-4FA7-8149-FC3AE9A3F3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECDE5239-836A-4EA3-B8EE-80ADBFE0F631}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7081971C-8A40-43CC-B1B6-C0A75DC16A39}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70A47465-53F6-46D1-829C-37A722620D9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7A50D54-5752-456E-A039-B3B68B72D9EB}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 19:16
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D911DF41-F638-4FA7-8149-FC3AE9A3F3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{697417AD-D363-40E6-AD8E-9AE35C796D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9602,7 +9602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7081971C-8A40-43CC-B1B6-C0A75DC16A39}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3D8A965-56FD-430D-AF4E-7688F2052581}">
   <dimension ref="B9:D546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15524,7 +15524,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7A50D54-5752-456E-A039-B3B68B72D9EB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFE258ED-623F-47EE-9246-1CC8211E1F4C}">
   <dimension ref="B9:H546"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA model - 2025-09-22 21:57
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EDAC0B3-16E7-4131-AFF6-F9219A102B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{503D5609-D00B-4D74-A0F8-FFC21FB15A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12950,6 +12950,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BD3AABB-DB33-4DC6-9596-A875D26342E1}">
   <dimension ref="B9:H567"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="6" max="6" width="21.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="9" spans="2:8">
       <c r="B9" t="s">
@@ -23939,6 +23942,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9FF79CD-3181-4163-89A7-7B1673009CC6}">
   <dimension ref="B9:L567"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="11.9296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.06640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="17.73046875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="9" spans="2:12">
       <c r="B9" t="s">

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-27 20:49
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D488C883-A4B4-4223-8A21-56AE7D6F116E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{60F80283-589E-4C81-A471-8D920261AB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13081,7 +13081,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09995298-36CC-4588-BA1C-AF42F2F6A3A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{821D884B-2B6A-4C79-AF39-1D43EB83D1F1}">
   <dimension ref="B9:H567"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -24070,7 +24070,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C6F86D0-DCAA-4702-87B2-E068630C8444}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CEDC1B1-6DAC-4495-90A6-D0F902516FCD}">
   <dimension ref="B9:L567"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>